<commit_message>
Complete Work of Home Page and some KPI's & Filter
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC446B6-2E32-4894-AFC7-8488DB66EAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5236EBF7-D99E-4571-9907-9195C03E6024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Data Cleaning" sheetId="2" r:id="rId2"/>
     <sheet name="Data-Transformation-Wrangling" sheetId="3" r:id="rId3"/>
     <sheet name="StoryTelling KPI-Charts" sheetId="4" r:id="rId4"/>
-    <sheet name="Plan" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
+    <sheet name="Plan" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="189">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -753,12 +754,102 @@
       <t>.</t>
     </r>
   </si>
+  <si>
+    <t>Globale KPIS</t>
+  </si>
+  <si>
+    <t>KPI No.</t>
+  </si>
+  <si>
+    <t>KPI Name</t>
+  </si>
+  <si>
+    <t>Formula / Basis</t>
+  </si>
+  <si>
+    <t>Total Sales (₹)</t>
+  </si>
+  <si>
+    <t>SUM(Total Amount)</t>
+  </si>
+  <si>
+    <t>Shows total revenue from all orders. This is the main business performance metric.</t>
+  </si>
+  <si>
+    <t>Total Orders</t>
+  </si>
+  <si>
+    <t>COUNTROWS(DISTINCT('Table'[Order ID]))</t>
+  </si>
+  <si>
+    <t>Total number of unique orders placed — helps track order volume.</t>
+  </si>
+  <si>
+    <t>Total Quantity Sold</t>
+  </si>
+  <si>
+    <t>SUM(Qty)</t>
+  </si>
+  <si>
+    <t>Total number of products sold — helps see demand and sales movement.</t>
+  </si>
+  <si>
+    <t>Average Order Value (AOV)</t>
+  </si>
+  <si>
+    <t>DIVIDE(SUM(Total Amount), COUNTROWS(DISTINCT('Table'[Order ID])))</t>
+  </si>
+  <si>
+    <t>Shows average revenue per order — a quality indicator for business performance.</t>
+  </si>
+  <si>
+    <t>KPI</t>
+  </si>
+  <si>
+    <t>When to Use</t>
+  </si>
+  <si>
+    <r>
+      <t>Delivered %</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = Delivered Orders ÷ Total Orders</t>
+    </r>
+  </si>
+  <si>
+    <t>On Fulfilment/Delivery Page</t>
+  </si>
+  <si>
+    <t>Return/Cancelled %</t>
+  </si>
+  <si>
+    <t>On Fulfilment or Overview Page</t>
+  </si>
+  <si>
+    <t>Promotion Sales %</t>
+  </si>
+  <si>
+    <t>On Promotion Page</t>
+  </si>
+  <si>
+    <t>B2B Sales %</t>
+  </si>
+  <si>
+    <t>On Promotion/Revenue Page</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -856,6 +947,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -946,7 +1042,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1029,6 +1125,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1346,7 +1459,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B3E6E2D-EEAD-4E4A-8798-C3B53E352FF0}">
   <dimension ref="B3:H30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" bestFit="1" customWidth="1"/>
@@ -1357,12 +1470,12 @@
     <col min="8" max="8" width="36.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:8" ht="25.8">
       <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:8" ht="21">
       <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1370,7 +1483,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="15.6">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1390,7 +1503,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="15.6">
       <c r="B7" s="22">
         <v>1</v>
       </c>
@@ -1410,7 +1523,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="31.2">
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -1430,7 +1543,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="15.6">
       <c r="B9" s="22">
         <v>3</v>
       </c>
@@ -1450,7 +1563,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="31.2">
       <c r="B10" s="22">
         <v>4</v>
       </c>
@@ -1470,7 +1583,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="31.2">
       <c r="B11" s="22">
         <v>5</v>
       </c>
@@ -1490,7 +1603,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="31.2">
       <c r="B12" s="22">
         <v>6</v>
       </c>
@@ -1510,7 +1623,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="31.2">
       <c r="B13" s="22">
         <v>7</v>
       </c>
@@ -1530,7 +1643,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="31.2">
       <c r="B14" s="22">
         <v>8</v>
       </c>
@@ -1550,7 +1663,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" ht="31.2">
       <c r="B15" s="22">
         <v>9</v>
       </c>
@@ -1570,7 +1683,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="31.2">
       <c r="B16" s="22">
         <v>10</v>
       </c>
@@ -1590,7 +1703,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="31.2">
       <c r="B17" s="22">
         <v>11</v>
       </c>
@@ -1610,7 +1723,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="31.2">
       <c r="B18" s="22">
         <v>12</v>
       </c>
@@ -1630,7 +1743,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" ht="15.6">
       <c r="B19" s="22">
         <v>13</v>
       </c>
@@ -1650,7 +1763,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="15.6">
       <c r="B20" s="22">
         <v>14</v>
       </c>
@@ -1670,7 +1783,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="15.6">
       <c r="B21" s="22">
         <v>15</v>
       </c>
@@ -1690,7 +1803,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="31.2">
       <c r="B22" s="22">
         <v>16</v>
       </c>
@@ -1710,7 +1823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="31.2">
       <c r="B23" s="22">
         <v>17</v>
       </c>
@@ -1730,7 +1843,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="15.6">
       <c r="B24" s="22">
         <v>18</v>
       </c>
@@ -1750,7 +1863,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="15.6">
       <c r="B25" s="22">
         <v>19</v>
       </c>
@@ -1770,7 +1883,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="31.2">
       <c r="B26" s="22">
         <v>20</v>
       </c>
@@ -1790,7 +1903,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="31.2">
       <c r="B27" s="22">
         <v>21</v>
       </c>
@@ -1810,7 +1923,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="28" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="31.2">
       <c r="B28" s="22">
         <v>22</v>
       </c>
@@ -1830,7 +1943,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="31.2">
       <c r="B29" s="22">
         <v>23</v>
       </c>
@@ -1841,7 +1954,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="31.2">
       <c r="B30" s="22">
         <v>24</v>
       </c>
@@ -1860,7 +1973,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6ADD15-B19C-416D-8A8B-7194E6C0A6D6}">
   <dimension ref="B3:K25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.77734375" bestFit="1" customWidth="1"/>
@@ -1874,12 +1987,12 @@
     <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:11" ht="25.8">
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:11" ht="15.6">
       <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
@@ -1909,7 +2022,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:11" ht="15.6">
       <c r="B6" s="20">
         <v>0</v>
       </c>
@@ -1938,7 +2051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:11" ht="15.6">
       <c r="B7" s="20">
         <v>1</v>
       </c>
@@ -1970,7 +2083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:11" ht="15.6">
       <c r="B8" s="20">
         <v>2</v>
       </c>
@@ -2002,7 +2115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:11" ht="15.6">
       <c r="B9" s="20">
         <v>3</v>
       </c>
@@ -2034,7 +2147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:11" ht="15.6">
       <c r="B10" s="20">
         <v>4</v>
       </c>
@@ -2066,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:11" ht="15.6">
       <c r="B11" s="20">
         <v>5</v>
       </c>
@@ -2098,7 +2211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:11" ht="15.6">
       <c r="B12" s="20">
         <v>6</v>
       </c>
@@ -2129,7 +2242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:11" ht="15.6">
       <c r="B13" s="20">
         <v>7</v>
       </c>
@@ -2160,7 +2273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:11" ht="15.6">
       <c r="B14" s="20">
         <v>8</v>
       </c>
@@ -2191,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:11" ht="15.6">
       <c r="B15" s="20">
         <v>9</v>
       </c>
@@ -2225,7 +2338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:11" ht="15.6">
       <c r="B16" s="20">
         <v>10</v>
       </c>
@@ -2258,7 +2371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" ht="15.6">
       <c r="B17" s="20">
         <v>11</v>
       </c>
@@ -2292,7 +2405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:11" ht="15.6">
       <c r="B18" s="20">
         <v>12</v>
       </c>
@@ -2325,7 +2438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:11" ht="15.6">
       <c r="B19" s="20">
         <v>13</v>
       </c>
@@ -2358,7 +2471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:11" ht="15.6">
       <c r="B20" s="20">
         <v>14</v>
       </c>
@@ -2391,7 +2504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:11" ht="15.6">
       <c r="B21" s="20">
         <v>15</v>
       </c>
@@ -2424,7 +2537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:11" ht="15.6">
       <c r="B22" s="20">
         <v>16</v>
       </c>
@@ -2457,7 +2570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:11" ht="15.6">
       <c r="B23" s="20">
         <v>17</v>
       </c>
@@ -2490,7 +2603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:11" ht="15.6">
       <c r="B24" s="20">
         <v>18</v>
       </c>
@@ -2523,7 +2636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:11" ht="15.6">
       <c r="B25" s="20">
         <v>19</v>
       </c>
@@ -2564,7 +2677,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7AAEBDA-2918-4347-B5CD-94210A58680A}">
   <dimension ref="B3:J13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -2572,12 +2685,12 @@
     <col min="10" max="10" width="190.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="25.8">
       <c r="D3" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" ht="15.6">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -2588,7 +2701,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10">
       <c r="I7">
         <v>1</v>
       </c>
@@ -2596,7 +2709,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10">
       <c r="I8">
         <v>2</v>
       </c>
@@ -2604,7 +2717,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10">
       <c r="I9">
         <v>3</v>
       </c>
@@ -2612,7 +2725,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10">
       <c r="I10">
         <v>4</v>
       </c>
@@ -2620,7 +2733,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10">
       <c r="I11">
         <v>5</v>
       </c>
@@ -2628,7 +2741,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10">
       <c r="I12">
         <v>6</v>
       </c>
@@ -2636,7 +2749,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10">
       <c r="I13">
         <v>7</v>
       </c>
@@ -2652,7 +2765,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FDCB3-6CAE-4927-8D50-CB20F0599746}">
   <dimension ref="B3:S7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.109375" bestFit="1" customWidth="1"/>
@@ -2671,7 +2784,7 @@
     <col min="19" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:19" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:19" ht="23.4">
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -2693,7 +2806,7 @@
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
     </row>
-    <row r="5" spans="2:19" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:19" ht="20.399999999999999">
       <c r="B5" s="13" t="s">
         <v>18</v>
       </c>
@@ -2721,7 +2834,7 @@
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
     </row>
-    <row r="7" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:19" ht="31.2">
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="18" t="s">
@@ -2771,9 +2884,141 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4BAE5E-D7E8-4F3F-BBD9-8CAD9399CE65}">
+  <dimension ref="C2:G16"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="52.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:7" ht="25.8">
+      <c r="C2" s="36" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="3:7" ht="18">
+      <c r="D4" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>166</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="3:7" ht="31.2">
+      <c r="D5" s="28">
+        <v>1</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="3:7" ht="31.2">
+      <c r="D6" s="28">
+        <v>2</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="7" spans="3:7" ht="31.2">
+      <c r="D7" s="28">
+        <v>3</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>174</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="3:7" ht="45">
+      <c r="D8" s="28">
+        <v>4</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>177</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="3:7">
+      <c r="D12" s="34" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="3:7" ht="28.8">
+      <c r="D13" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="E13" s="33" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="3:7">
+      <c r="D14" s="34" t="s">
+        <v>183</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="15" spans="3:7">
+      <c r="D15" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="3:7">
+      <c r="D16" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>188</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D08B4F4-38F3-4EC4-8131-B24327749222}">
-  <dimension ref="B3:G12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B3:H12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.21875" bestFit="1" customWidth="1"/>
@@ -2783,12 +3028,12 @@
     <col min="7" max="7" width="54.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:8" ht="25.8">
       <c r="B3" s="29" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="31.2">
       <c r="C5" s="30" t="s">
         <v>129</v>
       </c>
@@ -2804,8 +3049,11 @@
       <c r="G5" s="31" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H5" s="31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="46.8">
       <c r="C6" s="28">
         <v>1</v>
       </c>
@@ -2821,8 +3069,9 @@
       <c r="G6" s="27" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H6" s="32"/>
+    </row>
+    <row r="7" spans="2:8" ht="46.8">
       <c r="C7" s="28">
         <v>2</v>
       </c>
@@ -2838,8 +3087,9 @@
       <c r="G7" s="27" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" spans="2:8" ht="31.2">
       <c r="C8" s="28">
         <v>3</v>
       </c>
@@ -2855,8 +3105,9 @@
       <c r="G8" s="27" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H8" s="32"/>
+    </row>
+    <row r="9" spans="2:8" ht="46.8">
       <c r="C9" s="28">
         <v>4</v>
       </c>
@@ -2872,8 +3123,9 @@
       <c r="G9" s="27" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H9" s="32"/>
+    </row>
+    <row r="10" spans="2:8" ht="31.2">
       <c r="C10" s="28">
         <v>5</v>
       </c>
@@ -2889,8 +3141,9 @@
       <c r="G10" s="27" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H10" s="32"/>
+    </row>
+    <row r="11" spans="2:8" ht="31.2">
       <c r="C11" s="28">
         <v>6</v>
       </c>
@@ -2906,8 +3159,9 @@
       <c r="G11" s="27" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H11" s="32"/>
+    </row>
+    <row r="12" spans="2:8" ht="46.8">
       <c r="C12" s="28" t="s">
         <v>152</v>
       </c>
@@ -2923,6 +3177,7 @@
       <c r="G12" s="27" t="s">
         <v>156</v>
       </c>
+      <c r="H12" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Complete Overview Dashboard & add some things in Report
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5236EBF7-D99E-4571-9907-9195C03E6024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F54D98-8632-48A9-B314-8D20AA6BBBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
   <sheets>
     <sheet name="KYV - Column" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="209">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -95,9 +95,6 @@
     <t>Story Telling KPI's &amp; Charts</t>
   </si>
   <si>
-    <t xml:space="preserve">Main Dashboard </t>
-  </si>
-  <si>
     <t>KPI's</t>
   </si>
   <si>
@@ -116,16 +113,10 @@
     <t>Formula</t>
   </si>
   <si>
-    <t>Chart Name</t>
-  </si>
-  <si>
     <t>Columns Used</t>
   </si>
   <si>
     <t>Visual Type</t>
-  </si>
-  <si>
-    <t>Insight / Purpose</t>
   </si>
   <si>
     <t>Filter / Slicer Name</t>
@@ -844,12 +835,81 @@
   <si>
     <t>On Promotion/Revenue Page</t>
   </si>
+  <si>
+    <t>Visual Focus</t>
+  </si>
+  <si>
+    <t>Bar Chart (Top 5 Categories by Sales)</t>
+  </si>
+  <si>
+    <t>“Which product categories bring the most revenue?”</t>
+  </si>
+  <si>
+    <t>Category, Total Amount</t>
+  </si>
+  <si>
+    <t>Highlights top-performing product categories; instantly shows best sellers.</t>
+  </si>
+  <si>
+    <t>Donut Chart (Order Type or Fulfilment Share)</t>
+  </si>
+  <si>
+    <t>“Amazon vs Merchant contribution”</t>
+  </si>
+  <si>
+    <t>Order Type / Fulfilment, Total Amount</t>
+  </si>
+  <si>
+    <t>Quick view of FBA vs FBM performance — easy to understand fulfilment split.</t>
+  </si>
+  <si>
+    <t>Map or Filled Map (Sales by State)</t>
+  </si>
+  <si>
+    <t>“Which regions are driving sales?”</t>
+  </si>
+  <si>
+    <t>State, Total Amount</t>
+  </si>
+  <si>
+    <t>Displays sales distribution across India — great visual impact with color intensity.</t>
+  </si>
+  <si>
+    <t>Clustered Column Chart (Promotion vs Non-Promotion Sales)</t>
+  </si>
+  <si>
+    <t>“Are promotions increasing revenue?”</t>
+  </si>
+  <si>
+    <t>Promotion IDs, Total Amount</t>
+  </si>
+  <si>
+    <t>Compare sales from promoted vs regular orders. Quick insight into offer performance.</t>
+  </si>
+  <si>
+    <t>Line Chart (Sales Trend Over Time)</t>
+  </si>
+  <si>
+    <t>“How sales are moving month by month?”</t>
+  </si>
+  <si>
+    <t>Date, Month, Total Amount</t>
+  </si>
+  <si>
+    <t>Monthly trend or forecast line — helps users see growth or dip over time.</t>
+  </si>
+  <si>
+    <t>Overview</t>
+  </si>
+  <si>
+    <t>Promotion Type</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -952,6 +1012,11 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -1042,7 +1107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1143,6 +1208,26 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1508,19 +1593,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F7" s="22">
         <v>1</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H7" s="27" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="31.2">
@@ -1528,19 +1613,19 @@
         <v>2</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F8" s="22">
         <v>2</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H8" s="27" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15.6">
@@ -1548,19 +1633,19 @@
         <v>3</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F9" s="22">
         <v>3</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="31.2">
@@ -1568,19 +1653,19 @@
         <v>4</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F10" s="22">
         <v>4</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="31.2">
@@ -1588,19 +1673,19 @@
         <v>5</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F11" s="22">
         <v>5</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H11" s="27" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="31.2">
@@ -1608,19 +1693,19 @@
         <v>6</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F12" s="22">
         <v>6</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H12" s="27" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="31.2">
@@ -1628,19 +1713,19 @@
         <v>7</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F13" s="22">
         <v>7</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="31.2">
@@ -1648,19 +1733,19 @@
         <v>8</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F14" s="22">
         <v>8</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="31.2">
@@ -1668,19 +1753,19 @@
         <v>9</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F15" s="22">
         <v>9</v>
       </c>
       <c r="G15" s="26" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H15" s="27" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="31.2">
@@ -1688,19 +1773,19 @@
         <v>10</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F16" s="22">
         <v>10</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="31.2">
@@ -1708,19 +1793,19 @@
         <v>11</v>
       </c>
       <c r="C17" s="24" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F17" s="22">
         <v>11</v>
       </c>
       <c r="G17" s="26" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="31.2">
@@ -1728,19 +1813,19 @@
         <v>12</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F18" s="22">
         <v>12</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H18" s="27" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="15.6">
@@ -1748,19 +1833,19 @@
         <v>13</v>
       </c>
       <c r="C19" s="24" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F19" s="22">
         <v>13</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="15.6">
@@ -1768,19 +1853,19 @@
         <v>14</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F20" s="22">
         <v>14</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="15.6">
@@ -1788,19 +1873,19 @@
         <v>15</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F21" s="22">
         <v>15</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H21" s="27" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="31.2">
@@ -1808,19 +1893,19 @@
         <v>16</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F22" s="22">
         <v>16</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="31.2">
@@ -1828,19 +1913,19 @@
         <v>17</v>
       </c>
       <c r="C23" s="24" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F23" s="22">
         <v>17</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="15.6">
@@ -1848,19 +1933,19 @@
         <v>18</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F24" s="22">
         <v>18</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="H24" s="27" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="15.6">
@@ -1868,19 +1953,19 @@
         <v>19</v>
       </c>
       <c r="C25" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F25" s="22">
         <v>19</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H25" s="27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="31.2">
@@ -1888,19 +1973,19 @@
         <v>20</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F26" s="22">
         <v>20</v>
       </c>
       <c r="G26" s="26" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H26" s="27" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="31.2">
@@ -1908,19 +1993,19 @@
         <v>21</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F27" s="22">
         <v>21</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="H27" s="27" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="31.2">
@@ -1928,19 +2013,19 @@
         <v>22</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F28" s="22">
         <v>22</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H28" s="27" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="31.2">
@@ -1948,21 +2033,28 @@
         <v>23</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>105</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="F29" s="43">
+        <v>23</v>
+      </c>
+      <c r="G29" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="H29" s="21"/>
     </row>
     <row r="30" spans="2:8" ht="31.2">
       <c r="B30" s="22">
         <v>24</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1972,7 +2064,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6ADD15-B19C-416D-8A8B-7194E6C0A6D6}">
-  <dimension ref="B3:K25"/>
+  <dimension ref="B3:K26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
@@ -2027,7 +2119,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E6" s="21">
         <v>0</v>
@@ -2056,10 +2148,10 @@
         <v>1</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E7" s="21">
         <v>1</v>
@@ -2088,10 +2180,10 @@
         <v>2</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E8" s="21">
         <v>2</v>
@@ -2120,10 +2212,10 @@
         <v>3</v>
       </c>
       <c r="C9" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
         <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>53</v>
       </c>
       <c r="E9" s="21">
         <v>3</v>
@@ -2152,10 +2244,10 @@
         <v>4</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E10" s="21">
         <v>4</v>
@@ -2184,10 +2276,10 @@
         <v>5</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E11" s="21">
         <v>5</v>
@@ -2216,7 +2308,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="21">
@@ -2247,7 +2339,7 @@
         <v>7</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="21">
@@ -2278,7 +2370,7 @@
         <v>8</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E14" s="21">
         <v>8</v>
@@ -2309,10 +2401,10 @@
         <v>9</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E15" s="21">
         <v>9</v>
@@ -2343,10 +2435,10 @@
         <v>10</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E16" s="21">
         <v>10</v>
@@ -2376,10 +2468,10 @@
         <v>11</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E17" s="21">
         <v>11</v>
@@ -2410,10 +2502,10 @@
         <v>12</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E18" s="21">
         <v>12</v>
@@ -2443,10 +2535,10 @@
         <v>13</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E19" s="21">
         <v>13</v>
@@ -2476,10 +2568,10 @@
         <v>14</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E20" s="21">
         <v>14</v>
@@ -2509,10 +2601,10 @@
         <v>15</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E21" s="21">
         <v>15</v>
@@ -2542,10 +2634,10 @@
         <v>16</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E22" s="21">
         <v>16</v>
@@ -2575,10 +2667,10 @@
         <v>17</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E23" s="21">
         <v>17</v>
@@ -2608,10 +2700,10 @@
         <v>18</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E24" s="21">
         <v>18</v>
@@ -2641,10 +2733,10 @@
         <v>19</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D25" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E25" s="21">
         <v>19</v>
@@ -2666,6 +2758,39 @@
         <v>22</v>
       </c>
       <c r="K25" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="15.6">
+      <c r="B26" s="45">
+        <v>20</v>
+      </c>
+      <c r="C26" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="42" t="s">
+        <v>208</v>
+      </c>
+      <c r="E26" s="46">
+        <v>20</v>
+      </c>
+      <c r="F26" s="46">
+        <f>G25</f>
+        <v>113698</v>
+      </c>
+      <c r="G26" s="46">
+        <v>113698</v>
+      </c>
+      <c r="H26" s="46">
+        <v>0</v>
+      </c>
+      <c r="I26" s="46">
+        <v>22</v>
+      </c>
+      <c r="J26" s="46">
+        <v>23</v>
+      </c>
+      <c r="K26" s="46">
         <v>1</v>
       </c>
     </row>
@@ -2706,7 +2831,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="2:10">
@@ -2714,7 +2839,7 @@
         <v>2</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="2:10">
@@ -2722,7 +2847,7 @@
         <v>3</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="2:10">
@@ -2730,7 +2855,7 @@
         <v>4</v>
       </c>
       <c r="J10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="2:10">
@@ -2738,7 +2863,7 @@
         <v>5</v>
       </c>
       <c r="J11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="2:10">
@@ -2746,7 +2871,7 @@
         <v>6</v>
       </c>
       <c r="J12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="2:10">
@@ -2754,7 +2879,7 @@
         <v>7</v>
       </c>
       <c r="J13" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2764,20 +2889,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FDCB3-6CAE-4927-8D50-CB20F0599746}">
-  <dimension ref="B3:S7"/>
+  <dimension ref="B3:S14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" customWidth="1"/>
-    <col min="13" max="13" width="17.21875" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
+    <col min="11" max="11" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="44.5546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="25.88671875" customWidth="1"/>
@@ -2808,18 +2933,18 @@
     </row>
     <row r="5" spans="2:19" ht="20.399999999999999">
       <c r="B5" s="13" t="s">
-        <v>18</v>
+        <v>207</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J5" s="11"/>
       <c r="K5" s="11"/>
@@ -2828,58 +2953,259 @@
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
       <c r="P5" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
     </row>
-    <row r="7" spans="2:19" ht="31.2">
+    <row r="7" spans="2:19" ht="15.6">
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="18" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="G7" s="18" t="s">
         <v>23</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>24</v>
       </c>
       <c r="H7" s="11"/>
       <c r="I7" s="11"/>
       <c r="J7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>28</v>
+      <c r="L7" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="M7" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="39" t="s">
+        <v>5</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="11"/>
-      <c r="Q7" s="4" t="s">
+      <c r="Q7" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="R7" s="4" t="s">
+      <c r="R7" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19" ht="46.8">
+      <c r="D8" s="20">
+        <v>1</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="J8" s="20">
+        <v>1</v>
+      </c>
+      <c r="K8" s="26" t="s">
+        <v>187</v>
+      </c>
+      <c r="L8" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="M8" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="N8" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>1</v>
+      </c>
+      <c r="R8" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="2:19" ht="46.8">
+      <c r="D9" s="20">
+        <v>2</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="G9" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="J9" s="20">
+        <v>2</v>
+      </c>
+      <c r="K9" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="L9" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="M9" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="N9" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q9" s="27">
+        <v>2</v>
+      </c>
+      <c r="R9" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="S7" s="4" t="s">
+      <c r="S9" s="27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19" ht="31.2">
+      <c r="D10" s="20">
+        <v>3</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" s="20">
+        <v>3</v>
+      </c>
+      <c r="K10" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="L10" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="M10" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="N10" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q10" s="27">
+        <v>3</v>
+      </c>
+      <c r="R10" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="S10" s="27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" ht="46.8">
+      <c r="D11" s="20">
+        <v>4</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="G11" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="J11" s="20">
+        <v>4</v>
+      </c>
+      <c r="K11" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="L11" s="27" t="s">
+        <v>200</v>
+      </c>
+      <c r="M11" s="27" t="s">
+        <v>201</v>
+      </c>
+      <c r="N11" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q11" s="27">
+        <v>4</v>
+      </c>
+      <c r="R11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="S11" s="27" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" ht="31.2">
+      <c r="J12" s="20">
+        <v>5</v>
+      </c>
+      <c r="K12" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="L12" s="27" t="s">
+        <v>204</v>
+      </c>
+      <c r="M12" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="N12" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q12" s="27">
+        <v>5</v>
+      </c>
+      <c r="R12" s="26" t="s">
         <v>30</v>
+      </c>
+      <c r="S12" s="27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" ht="15.6">
+      <c r="Q13" s="27">
+        <v>6</v>
+      </c>
+      <c r="R13" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="S13" s="27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" ht="31.2">
+      <c r="Q14" s="27">
+        <v>7</v>
+      </c>
+      <c r="R14" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="S14" s="27" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2897,18 +3223,18 @@
   <sheetData>
     <row r="2" spans="3:7" ht="25.8">
       <c r="C2" s="36" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="3:7" ht="18">
       <c r="D4" s="37" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E4" s="38" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F4" s="38" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G4" s="38" t="s">
         <v>5</v>
@@ -2919,13 +3245,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="3:7" ht="31.2">
@@ -2933,13 +3259,13 @@
         <v>2</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="3:7" ht="31.2">
@@ -2947,13 +3273,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="3:7" ht="45">
@@ -2961,53 +3287,53 @@
         <v>4</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="3:7">
       <c r="D12" s="34" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="3:7" ht="28.8">
       <c r="D13" s="34" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="3:7">
       <c r="D14" s="34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="3:7">
       <c r="D15" s="34" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="3:7">
       <c r="D16" s="34" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3030,27 +3356,27 @@
   <sheetData>
     <row r="3" spans="2:8" ht="25.8">
       <c r="B3" s="29" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="31.2">
       <c r="C5" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="G5" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="E5" s="31" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="G5" s="31" t="s">
-        <v>133</v>
-      </c>
       <c r="H5" s="31" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="46.8">
@@ -3058,16 +3384,16 @@
         <v>1</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H6" s="32"/>
     </row>
@@ -3076,16 +3402,16 @@
         <v>2</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H7" s="32"/>
     </row>
@@ -3094,16 +3420,16 @@
         <v>3</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H8" s="32"/>
     </row>
@@ -3112,16 +3438,16 @@
         <v>4</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H9" s="32"/>
     </row>
@@ -3130,16 +3456,16 @@
         <v>5</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H10" s="32"/>
     </row>
@@ -3148,34 +3474,34 @@
         <v>6</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H11" s="32"/>
     </row>
     <row r="12" spans="2:8" ht="46.8">
       <c r="C12" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="F12" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="G12" s="27" t="s">
         <v>153</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="F12" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="G12" s="27" t="s">
-        <v>156</v>
       </c>
       <c r="H12" s="32"/>
     </row>

</xml_diff>

<commit_message>
complete overview dashboard and set up next dashboard kpi's
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F54D98-8632-48A9-B314-8D20AA6BBBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2FF7BE-498E-4FDA-8B73-2A9C88CA4448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -17,8 +17,8 @@
     <sheet name="Data Cleaning" sheetId="2" r:id="rId2"/>
     <sheet name="Data-Transformation-Wrangling" sheetId="3" r:id="rId3"/>
     <sheet name="StoryTelling KPI-Charts" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
-    <sheet name="Plan" sheetId="5" r:id="rId6"/>
+    <sheet name="Plan" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="377">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -903,13 +903,1328 @@
   </si>
   <si>
     <t>Promotion Type</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Acts as the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>main navigation hub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; only contains buttons (no visuals/slicers).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>High-level summary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — contains 1 key visual from each section + buttons to open detailed pages.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Focus on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>what products drive performance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Focus on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>who fulfilled orders and shipping performance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Focus on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>where sales are coming from</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Focus on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>offers, B2B orders, and revenue patterns</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Page</t>
+  </si>
+  <si>
+    <t>1️⃣ Product Insights</t>
+  </si>
+  <si>
+    <t>2️⃣ Fulfilment &amp; Delivery</t>
+  </si>
+  <si>
+    <t>3️⃣ Regional Analysis</t>
+  </si>
+  <si>
+    <t>4️⃣ Promotion &amp; Revenue Analysis</t>
+  </si>
+  <si>
+    <t>5️⃣ Trend &amp; Forecasting (Advanced)</t>
+  </si>
+  <si>
+    <t>DAX / Field Logic</t>
+  </si>
+  <si>
+    <t>Purpose / Insight</t>
+  </si>
+  <si>
+    <t>Best-Selling Category</t>
+  </si>
+  <si>
+    <t>Top Performing Size</t>
+  </si>
+  <si>
+    <t>Top SKU by Sales</t>
+  </si>
+  <si>
+    <t>Field Mapping (Power BI)</t>
+  </si>
+  <si>
+    <t>Column Chart – Size-wise Performance</t>
+  </si>
+  <si>
+    <t>Size, Total Amount</t>
+  </si>
+  <si>
+    <t>Understand which product sizes generate the most revenue.</t>
+  </si>
+  <si>
+    <t>Combo Chart – Category vs Quantity &amp; Sales</t>
+  </si>
+  <si>
+    <t>Category, Quantity, Total Amount</t>
+  </si>
+  <si>
+    <t>Compare category performance based on both sales volume and revenue.</t>
+  </si>
+  <si>
+    <t>Bar Chart – Top 10 SKUs by Profit</t>
+  </si>
+  <si>
+    <t>SKU, Total Amount, Cost</t>
+  </si>
+  <si>
+    <t>Shows most profitable products (SKUs).</t>
+  </si>
+  <si>
+    <t>Line Chart – Product Demand Trend (Monthly)</t>
+  </si>
+  <si>
+    <t>Month, Quantity, Category</t>
+  </si>
+  <si>
+    <t>Analyzes monthly demand pattern for each category.</t>
+  </si>
+  <si>
+    <t>Treemap – Sales by Subcategory</t>
+  </si>
+  <si>
+    <t>Category, Sub-Category, Total Amount</t>
+  </si>
+  <si>
+    <t>Visualize contribution of each subcategory to overall sales.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">X-Axis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Size</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Values: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SUM(Total Amount)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">X-Axis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Column: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SUM(Quantity)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Line: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SUM(Total Amount)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Axis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SKU</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Values: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Profit = [Total Amount] - [Cost]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Filter: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Top 10 by Profit</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">X-Axis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Y-Axis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SUM(Quantity)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Legend: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Group: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Details: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Sub-Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Values: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SUM(Total Amount)</t>
+    </r>
+  </si>
+  <si>
+    <t>Global KPI's</t>
+  </si>
+  <si>
+    <t>Best Selling Category = CALCULATE(SELECTEDVALUE('Sales'[Category]), TOPN(1, SUMMARIZE('Sales', 'Sales'[Category], "Sales", SUM('Sales'[Total Amount])), [Sales], DESC))</t>
+  </si>
+  <si>
+    <t>Identifies the product category with the highest total sales.</t>
+  </si>
+  <si>
+    <t>Top Performing Size = CALCULATE(SELECTEDVALUE('Sales'[Size]), TOPN(1, SUMMARIZE('Sales', 'Sales'[Size], "Sales", SUM('Sales'[Total Amount])), [Sales], DESC))</t>
+  </si>
+  <si>
+    <t>Highlights which product size sells the most.</t>
+  </si>
+  <si>
+    <t>Top SKU by Sales = CALCULATE(SELECTEDVALUE('Sales'[SKU]), TOPN(1, SUMMARIZE('Sales', 'Sales'[SKU], "Sales", SUM('Sales'[Total Amount])), [Sales], DESC))</t>
+  </si>
+  <si>
+    <t>Shows the SKU that generates maximum revenue.</t>
+  </si>
+  <si>
+    <t>Average Category Revenue (₹)</t>
+  </si>
+  <si>
+    <t>Avg Category Sales = AVERAGEX(VALUES('Sales'[Category]), SUM('Sales'[Total Amount]))</t>
+  </si>
+  <si>
+    <t>Finds the average sales per category to compare overall product strength.</t>
+  </si>
+  <si>
+    <t>Category Contribution % (Top vs Rest)</t>
+  </si>
+  <si>
+    <t>Category Contribution % = DIVIDE([Top Category Sales], [Total Sales])</t>
+  </si>
+  <si>
+    <t>Shows how much percentage of total revenue comes from the top-selling category.</t>
+  </si>
+  <si>
+    <t>Globle</t>
+  </si>
+  <si>
+    <t>Total Orders (Fulfilment)</t>
+  </si>
+  <si>
+    <t>Total Orders = COUNTROWS('Sales')</t>
+  </si>
+  <si>
+    <t>Shows how many total orders were processed.</t>
+  </si>
+  <si>
+    <t>FBA vs FBM % Share</t>
+  </si>
+  <si>
+    <t>Fulfilment % = DIVIDE(SUMX(FILTER('Sales', 'Sales'[Fulfilment] = "Amazon"), 'Sales'[Total Amount]), [Total Sales])</t>
+  </si>
+  <si>
+    <t>Measures percentage contribution of Amazon (FBA) in total sales.</t>
+  </si>
+  <si>
+    <t>Avg Delivery Value (₹)</t>
+  </si>
+  <si>
+    <t>Avg Delivery Value = AVERAGEX(VALUES('Sales'[Fulfilment]), SUM('Sales'[Total Amount]))</t>
+  </si>
+  <si>
+    <t>Compares average order value handled by each fulfilment method.</t>
+  </si>
+  <si>
+    <t>Delivered Orders %</t>
+  </si>
+  <si>
+    <t>Delivered % = DIVIDE(CALCULATE(COUNTROWS('Sales'), 'Sales'[Order Status Group] = "Delivered"), [Total Orders])</t>
+  </si>
+  <si>
+    <t>Tracks delivery efficiency — % of total delivered orders.</t>
+  </si>
+  <si>
+    <t>Visual Focus / Question</t>
+  </si>
+  <si>
+    <r>
+      <t>Donut Chart – Fulfilment Share</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Already used in Overview)</t>
+    </r>
+  </si>
+  <si>
+    <t>Fulfilment / Order Type, Total Amount</t>
+  </si>
+  <si>
+    <t>Compare overall revenue share between FBA (Amazon) and FBM (Merchant).</t>
+  </si>
+  <si>
+    <t>Clustered Column Chart – Avg Delivery Amount by Fulfilment</t>
+  </si>
+  <si>
+    <t>“Which fulfilment type gives higher average order value?”</t>
+  </si>
+  <si>
+    <t>Fulfilment, Total Amount</t>
+  </si>
+  <si>
+    <t>Shows which fulfilment type (Amazon or Merchant) handles higher-value orders on average.</t>
+  </si>
+  <si>
+    <t>Bar Chart – Orders by Courier Status</t>
+  </si>
+  <si>
+    <t>“What’s the delivery progress for each fulfilment type?”</t>
+  </si>
+  <si>
+    <t>Courier Status, Fulfilment, Qty</t>
+  </si>
+  <si>
+    <t>Visualizes shipment stages (Delivered, Shipped, Cancelled etc.) under each fulfilment type to measure performance.</t>
+  </si>
+  <si>
+    <t>Stacked Column Chart – Orders by Fulfilment &amp; Status</t>
+  </si>
+  <si>
+    <t>“How each fulfilment type performs across different statuses?”</t>
+  </si>
+  <si>
+    <t>Fulfilment, Order Status Group, Qty</t>
+  </si>
+  <si>
+    <t>Compare delivery performance (Delivered / Shipped / Cancelled) for Amazon vs Merchant in one visual.</t>
+  </si>
+  <si>
+    <t>Card / Gauge – Fulfilment Efficiency %</t>
+  </si>
+  <si>
+    <t>“What is the delivery success rate for each fulfilment type?”</t>
+  </si>
+  <si>
+    <t>Fulfilment, Order Status Group</t>
+  </si>
+  <si>
+    <t>Simple KPI visual showing % of Delivered orders vs Total — great to measure operational efficiency.</t>
+  </si>
+  <si>
+    <t>Regional</t>
+  </si>
+  <si>
+    <r>
+      <t>Smart Narrative (AI Visual)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Add automatically generated insights like:</t>
+    </r>
+  </si>
+  <si>
+    <t>“Amazon fulfilled 60% of total orders with 95% delivery success, while Merchant handled 40% with 80% success.”</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ye </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Power BI Smart Narrative Visual</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> se auto insights deta hai.</t>
+    </r>
+  </si>
+  <si>
+    <t>Top State by Sales</t>
+  </si>
+  <si>
+    <t>TOPN(1, SUMMARIZE('Orders','Orders'[State],"StateSales",SUM('Orders'[Total Amount])),[StateSales],DESC)</t>
+  </si>
+  <si>
+    <t>Highlights the state contributing the most to sales</t>
+  </si>
+  <si>
+    <t>Filled / Shape / Bubble Map</t>
+  </si>
+  <si>
+    <r>
+      <t>State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <t>Shows total sales per state with color intensity / bubble size</t>
+  </si>
+  <si>
+    <t>Bar Chart – State vs Total Amount</t>
+  </si>
+  <si>
+    <t>“Top-performing states?”</t>
+  </si>
+  <si>
+    <t>Easy comparison of sales across states</t>
+  </si>
+  <si>
+    <t>Stacked Column Chart – Fulfilment by State</t>
+  </si>
+  <si>
+    <t>“Amazon vs Merchant contribution per region?”</t>
+  </si>
+  <si>
+    <r>
+      <t>State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Fulfilment</t>
+    </r>
+  </si>
+  <si>
+    <t>Highlights fulfillment trends region-wise</t>
+  </si>
+  <si>
+    <t>Card Visual – Total Regional Sales</t>
+  </si>
+  <si>
+    <t>“What is total sales across all regions?”</t>
+  </si>
+  <si>
+    <t>Quick KPI summary</t>
+  </si>
+  <si>
+    <t>Card Visual – Top State by Sales</t>
+  </si>
+  <si>
+    <t>“Which state contributes most to sales?”</t>
+  </si>
+  <si>
+    <t>Highlights the best-performing state</t>
+  </si>
+  <si>
+    <t>Table / Matrix – State / City / Total Amount / Qty</t>
+  </si>
+  <si>
+    <t>“Detailed breakdown of sales by city and state”</t>
+  </si>
+  <si>
+    <r>
+      <t>State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>City</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Qty</t>
+    </r>
+  </si>
+  <si>
+    <t>Drill-down view for detailed analysis</t>
+  </si>
+  <si>
+    <t>Promotion</t>
+  </si>
+  <si>
+    <t>Forcasting</t>
+  </si>
+  <si>
+    <t>YoY Growth %</t>
+  </si>
+  <si>
+    <t>(SUM(CurrentYearSales)-SUM(PreviousYearSales))/SUM(PreviousYearSales)</t>
+  </si>
+  <si>
+    <t>Shows sales growth compared to same period last year</t>
+  </si>
+  <si>
+    <t>Cumulative Sales</t>
+  </si>
+  <si>
+    <t>CALCULATE(SUM('Orders'[Total Amount]), FILTER(ALLSELECTED('Orders'[Date]), 'Orders'[Date]&lt;=MAX('Orders'[Date])))</t>
+  </si>
+  <si>
+    <t>Shows running total of sales over time</t>
+  </si>
+  <si>
+    <t>Line Chart – Sales Trend Over Time</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <t>Shows revenue trend; detects peaks, dips, and seasonality</t>
+  </si>
+  <si>
+    <t>Area Chart – Qty Trend</t>
+  </si>
+  <si>
+    <t>“How units sold are changing over time?”</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Qty</t>
+    </r>
+  </si>
+  <si>
+    <t>Visualizes demand trend and sales volume changes</t>
+  </si>
+  <si>
+    <t>Forecast Line (Power BI Analytics)</t>
+  </si>
+  <si>
+    <t>“Predict next 3–6 months sales”</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <t>Predicts future revenue using historical trend + confidence interval</t>
+  </si>
+  <si>
+    <t>Line Chart – Cumulative Sales</t>
+  </si>
+  <si>
+    <t>“How sales accumulate over time”</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Cumulative Sales</t>
+    </r>
+  </si>
+  <si>
+    <t>Shows running total trend for period-wise progress</t>
+  </si>
+  <si>
+    <t>Combo Chart – Sales vs Quantity</t>
+  </si>
+  <si>
+    <t>“Is revenue growth due to volume or price?”</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Qty</t>
+    </r>
+  </si>
+  <si>
+    <t>Line for sales + Column for Qty to compare revenue vs units</t>
+  </si>
+  <si>
+    <t>Decomposition Tree</t>
+  </si>
+  <si>
+    <t>“What caused the increase/decrease?”</t>
+  </si>
+  <si>
+    <r>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Fulfilment</t>
+    </r>
+  </si>
+  <si>
+    <t>Drill into sales trend by different dimensions to find causes</t>
+  </si>
+  <si>
+    <t>Total Promotion Sales</t>
+  </si>
+  <si>
+    <t>CALCULATE(SUM('Orders'[Total Amount]), NOT(ISBLANK('Orders'[Promotion IDs])))</t>
+  </si>
+  <si>
+    <t>Shows total revenue generated from all promoted orders</t>
+  </si>
+  <si>
+    <t>Promotion Contribution (%)</t>
+  </si>
+  <si>
+    <t>DIVIDE(CALCULATE(SUM('Orders'[Total Amount]), NOT(ISBLANK('Orders'[Promotion IDs]))), SUM('Orders'[Total Amount]))</t>
+  </si>
+  <si>
+    <t>Shows percentage of total sales coming from promotions</t>
+  </si>
+  <si>
+    <t>Top Promotion Type by Sales</t>
+  </si>
+  <si>
+    <t>TOPN(1, SUMMARIZE('Orders','Orders'[Promotion Type],"PromoSales",SUM('Orders'[Total Amount])),[PromoSales],DESC)</t>
+  </si>
+  <si>
+    <t>Highlights the most effective promotion type</t>
+  </si>
+  <si>
+    <t>Clustered Column Chart</t>
+  </si>
+  <si>
+    <t>“Promotion vs Non-Promotion Sales”</t>
+  </si>
+  <si>
+    <r>
+      <t>Promotion IDs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <t>Compare revenue from promoted vs regular orders</t>
+  </si>
+  <si>
+    <t>Stacked Column Chart</t>
+  </si>
+  <si>
+    <t>“Sales by Promotion Type”</t>
+  </si>
+  <si>
+    <r>
+      <t>Promotion Type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <t>Shows which type of promotion brings the most revenue</t>
+  </si>
+  <si>
+    <t>Card Visual – Total Promotion Sales</t>
+  </si>
+  <si>
+    <t>“Total revenue from promotions”</t>
+  </si>
+  <si>
+    <r>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (filtered by Promotion IDs)</t>
+    </r>
+  </si>
+  <si>
+    <t>Quick view of total promotion revenue</t>
+  </si>
+  <si>
+    <t>Table / Matrix</t>
+  </si>
+  <si>
+    <t>“Detailed promotion-wise sales”</t>
+  </si>
+  <si>
+    <r>
+      <t>Promotion IDs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Promotion Type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Qty</t>
+    </r>
+  </si>
+  <si>
+    <t>Drill-down view for detailed analysis per promotion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1017,6 +2332,14 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -1107,7 +2430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1219,15 +2542,30 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1544,7 +2882,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B3E6E2D-EEAD-4E4A-8798-C3B53E352FF0}">
   <dimension ref="B3:H30"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" bestFit="1" customWidth="1"/>
@@ -1555,12 +2893,12 @@
     <col min="8" max="8" width="36.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="25.8">
+    <row r="3" spans="2:8" ht="25.8" x14ac:dyDescent="0.5">
       <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="21">
+    <row r="4" spans="2:8" ht="21" x14ac:dyDescent="0.4">
       <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1568,7 +2906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15.6">
+    <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1588,7 +2926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15.6">
+    <row r="7" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="22">
         <v>1</v>
       </c>
@@ -1608,7 +2946,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="31.2">
+    <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -1628,7 +2966,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="15.6">
+    <row r="9" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="22">
         <v>3</v>
       </c>
@@ -1648,7 +2986,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="31.2">
+    <row r="10" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B10" s="22">
         <v>4</v>
       </c>
@@ -1668,7 +3006,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="31.2">
+    <row r="11" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B11" s="22">
         <v>5</v>
       </c>
@@ -1688,7 +3026,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="31.2">
+    <row r="12" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B12" s="22">
         <v>6</v>
       </c>
@@ -1708,7 +3046,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="31.2">
+    <row r="13" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B13" s="22">
         <v>7</v>
       </c>
@@ -1728,7 +3066,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="31.2">
+    <row r="14" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B14" s="22">
         <v>8</v>
       </c>
@@ -1748,7 +3086,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="31.2">
+    <row r="15" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B15" s="22">
         <v>9</v>
       </c>
@@ -1768,7 +3106,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="31.2">
+    <row r="16" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B16" s="22">
         <v>10</v>
       </c>
@@ -1788,7 +3126,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="31.2">
+    <row r="17" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B17" s="22">
         <v>11</v>
       </c>
@@ -1808,7 +3146,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="31.2">
+    <row r="18" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B18" s="22">
         <v>12</v>
       </c>
@@ -1828,7 +3166,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15.6">
+    <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B19" s="22">
         <v>13</v>
       </c>
@@ -1848,7 +3186,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="15.6">
+    <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B20" s="22">
         <v>14</v>
       </c>
@@ -1868,7 +3206,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="15.6">
+    <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B21" s="22">
         <v>15</v>
       </c>
@@ -1888,7 +3226,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="31.2">
+    <row r="22" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B22" s="22">
         <v>16</v>
       </c>
@@ -1908,7 +3246,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="31.2">
+    <row r="23" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B23" s="22">
         <v>17</v>
       </c>
@@ -1928,7 +3266,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="15.6">
+    <row r="24" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B24" s="22">
         <v>18</v>
       </c>
@@ -1948,7 +3286,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="15.6">
+    <row r="25" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B25" s="22">
         <v>19</v>
       </c>
@@ -1968,7 +3306,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="31.2">
+    <row r="26" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B26" s="22">
         <v>20</v>
       </c>
@@ -1988,7 +3326,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="31.2">
+    <row r="27" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B27" s="22">
         <v>21</v>
       </c>
@@ -2008,7 +3346,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="2:8" ht="31.2">
+    <row r="28" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B28" s="22">
         <v>22</v>
       </c>
@@ -2028,7 +3366,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="31.2">
+    <row r="29" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B29" s="22">
         <v>23</v>
       </c>
@@ -2038,15 +3376,15 @@
       <c r="D29" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="F29" s="43">
+      <c r="F29" s="22">
         <v>23</v>
       </c>
-      <c r="G29" s="44" t="s">
+      <c r="G29" s="43" t="s">
         <v>208</v>
       </c>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="2:8" ht="31.2">
+    <row r="30" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B30" s="22">
         <v>24</v>
       </c>
@@ -2065,7 +3403,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6ADD15-B19C-416D-8A8B-7194E6C0A6D6}">
   <dimension ref="B3:K26"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.77734375" bestFit="1" customWidth="1"/>
@@ -2079,12 +3417,12 @@
     <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11" ht="25.8">
+    <row r="3" spans="2:11" ht="25.8" x14ac:dyDescent="0.5">
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="15.6">
+    <row r="5" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
@@ -2114,7 +3452,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="15.6">
+    <row r="6" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="20">
         <v>0</v>
       </c>
@@ -2143,7 +3481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="15.6">
+    <row r="7" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="20">
         <v>1</v>
       </c>
@@ -2175,7 +3513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="15.6">
+    <row r="8" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="20">
         <v>2</v>
       </c>
@@ -2207,7 +3545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="15.6">
+    <row r="9" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="20">
         <v>3</v>
       </c>
@@ -2239,7 +3577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="15.6">
+    <row r="10" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="20">
         <v>4</v>
       </c>
@@ -2271,7 +3609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="15.6">
+    <row r="11" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="20">
         <v>5</v>
       </c>
@@ -2303,7 +3641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="15.6">
+    <row r="12" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="20">
         <v>6</v>
       </c>
@@ -2334,7 +3672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:11" ht="15.6">
+    <row r="13" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="20">
         <v>7</v>
       </c>
@@ -2365,7 +3703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="15.6">
+    <row r="14" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="20">
         <v>8</v>
       </c>
@@ -2396,7 +3734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:11" ht="15.6">
+    <row r="15" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="20">
         <v>9</v>
       </c>
@@ -2430,7 +3768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:11" ht="15.6">
+    <row r="16" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="20">
         <v>10</v>
       </c>
@@ -2463,7 +3801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:11" ht="15.6">
+    <row r="17" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B17" s="20">
         <v>11</v>
       </c>
@@ -2497,7 +3835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:11" ht="15.6">
+    <row r="18" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="20">
         <v>12</v>
       </c>
@@ -2530,7 +3868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:11" ht="15.6">
+    <row r="19" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B19" s="20">
         <v>13</v>
       </c>
@@ -2563,7 +3901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:11" ht="15.6">
+    <row r="20" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B20" s="20">
         <v>14</v>
       </c>
@@ -2596,7 +3934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:11" ht="15.6">
+    <row r="21" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B21" s="20">
         <v>15</v>
       </c>
@@ -2629,7 +3967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:11" ht="15.6">
+    <row r="22" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B22" s="20">
         <v>16</v>
       </c>
@@ -2662,7 +4000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:11" ht="15.6">
+    <row r="23" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B23" s="20">
         <v>17</v>
       </c>
@@ -2695,7 +4033,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:11" ht="15.6">
+    <row r="24" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B24" s="20">
         <v>18</v>
       </c>
@@ -2728,7 +4066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15.6">
+    <row r="25" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B25" s="20">
         <v>19</v>
       </c>
@@ -2761,36 +4099,36 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:11" ht="15.6">
-      <c r="B26" s="45">
+    <row r="26" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="20">
         <v>20</v>
       </c>
-      <c r="C26" s="45" t="s">
+      <c r="C26" s="20" t="s">
         <v>60</v>
       </c>
       <c r="D26" s="42" t="s">
         <v>208</v>
       </c>
-      <c r="E26" s="46">
+      <c r="E26" s="21">
         <v>20</v>
       </c>
-      <c r="F26" s="46">
+      <c r="F26" s="21">
         <f>G25</f>
         <v>113698</v>
       </c>
-      <c r="G26" s="46">
+      <c r="G26" s="21">
         <v>113698</v>
       </c>
-      <c r="H26" s="46">
+      <c r="H26" s="21">
         <v>0</v>
       </c>
-      <c r="I26" s="46">
+      <c r="I26" s="21">
         <v>22</v>
       </c>
-      <c r="J26" s="46">
+      <c r="J26" s="21">
         <v>23</v>
       </c>
-      <c r="K26" s="46">
+      <c r="K26" s="21">
         <v>1</v>
       </c>
     </row>
@@ -2802,7 +4140,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7AAEBDA-2918-4347-B5CD-94210A58680A}">
   <dimension ref="B3:J13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -2810,12 +4148,12 @@
     <col min="10" max="10" width="190.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="25.8">
+    <row r="3" spans="2:10" ht="25.8" x14ac:dyDescent="0.3">
       <c r="D3" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="15.6">
+    <row r="5" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -2826,7 +4164,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:10">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I7">
         <v>1</v>
       </c>
@@ -2834,7 +4172,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:10">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I8">
         <v>2</v>
       </c>
@@ -2842,7 +4180,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="2:10">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I9">
         <v>3</v>
       </c>
@@ -2850,7 +4188,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:10">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I10">
         <v>4</v>
       </c>
@@ -2858,7 +4196,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="2:10">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I11">
         <v>5</v>
       </c>
@@ -2866,7 +4204,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:10">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I12">
         <v>6</v>
       </c>
@@ -2874,7 +4212,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="2:10">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="I13">
         <v>7</v>
       </c>
@@ -2889,27 +4227,27 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FDCB3-6CAE-4927-8D50-CB20F0599746}">
-  <dimension ref="B3:S14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="B3:S71"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.88671875" customWidth="1"/>
     <col min="7" max="7" width="40.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="39.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="42.44140625" customWidth="1"/>
     <col min="14" max="14" width="44.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="31.21875" customWidth="1"/>
     <col min="17" max="17" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="25.88671875" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:19" ht="23.4">
+    <row r="3" spans="2:19" ht="23.4" x14ac:dyDescent="0.3">
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -2931,15 +4269,17 @@
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
     </row>
-    <row r="5" spans="2:19" ht="20.399999999999999">
+    <row r="5" spans="2:19" ht="21" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
         <v>207</v>
       </c>
       <c r="C5" s="14"/>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="11"/>
+      <c r="E5" s="50" t="s">
+        <v>248</v>
+      </c>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -2956,10 +4296,12 @@
         <v>20</v>
       </c>
       <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
+      <c r="R5" s="11" t="s">
+        <v>261</v>
+      </c>
       <c r="S5" s="11"/>
     </row>
-    <row r="7" spans="2:19" ht="15.6">
+    <row r="7" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="18" t="s">
@@ -3003,8 +4345,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:19" ht="46.8">
-      <c r="D8" s="20">
+    <row r="8" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="D8" s="44">
         <v>1</v>
       </c>
       <c r="E8" s="26" t="s">
@@ -3016,7 +4358,7 @@
       <c r="G8" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="J8" s="20">
+      <c r="J8" s="44">
         <v>1</v>
       </c>
       <c r="K8" s="26" t="s">
@@ -3031,7 +4373,7 @@
       <c r="N8" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="22">
         <v>1</v>
       </c>
       <c r="R8" s="26" t="s">
@@ -3041,8 +4383,8 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="2:19" ht="46.8">
-      <c r="D9" s="20">
+    <row r="9" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="D9" s="44">
         <v>2</v>
       </c>
       <c r="E9" s="26" t="s">
@@ -3054,7 +4396,7 @@
       <c r="G9" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="J9" s="20">
+      <c r="J9" s="44">
         <v>2</v>
       </c>
       <c r="K9" s="26" t="s">
@@ -3069,7 +4411,7 @@
       <c r="N9" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="22">
         <v>2</v>
       </c>
       <c r="R9" s="26" t="s">
@@ -3079,8 +4421,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:19" ht="31.2">
-      <c r="D10" s="20">
+    <row r="10" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="D10" s="44">
         <v>3</v>
       </c>
       <c r="E10" s="26" t="s">
@@ -3092,7 +4434,7 @@
       <c r="G10" s="40" t="s">
         <v>171</v>
       </c>
-      <c r="J10" s="20">
+      <c r="J10" s="44">
         <v>3</v>
       </c>
       <c r="K10" s="26" t="s">
@@ -3107,7 +4449,7 @@
       <c r="N10" s="27" t="s">
         <v>198</v>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="22">
         <v>3</v>
       </c>
       <c r="R10" s="26" t="s">
@@ -3117,8 +4459,8 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:19" ht="46.8">
-      <c r="D11" s="20">
+    <row r="11" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="D11" s="44">
         <v>4</v>
       </c>
       <c r="E11" s="26" t="s">
@@ -3130,7 +4472,7 @@
       <c r="G11" s="40" t="s">
         <v>174</v>
       </c>
-      <c r="J11" s="20">
+      <c r="J11" s="44">
         <v>4</v>
       </c>
       <c r="K11" s="26" t="s">
@@ -3145,7 +4487,7 @@
       <c r="N11" s="27" t="s">
         <v>202</v>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="22">
         <v>4</v>
       </c>
       <c r="R11" s="26" t="s">
@@ -3155,8 +4497,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:19" ht="31.2">
-      <c r="J12" s="20">
+    <row r="12" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="J12" s="44">
         <v>5</v>
       </c>
       <c r="K12" s="26" t="s">
@@ -3171,7 +4513,7 @@
       <c r="N12" s="27" t="s">
         <v>206</v>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="22">
         <v>5</v>
       </c>
       <c r="R12" s="26" t="s">
@@ -3181,8 +4523,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="2:19" ht="15.6">
-      <c r="Q13" s="27">
+    <row r="13" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="Q13" s="22">
         <v>6</v>
       </c>
       <c r="R13" s="26" t="s">
@@ -3192,8 +4534,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="2:19" ht="31.2">
-      <c r="Q14" s="27">
+    <row r="14" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="Q14" s="22">
         <v>7</v>
       </c>
       <c r="R14" s="26" t="s">
@@ -3201,6 +4543,826 @@
       </c>
       <c r="S14" s="27" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B16" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D18" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="F18" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G18" s="49" t="s">
+        <v>223</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="D19" s="22">
+        <v>1</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="F19" s="40" t="s">
+        <v>249</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="J19" s="23">
+        <v>1</v>
+      </c>
+      <c r="K19" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="L19" s="23" t="s">
+        <v>229</v>
+      </c>
+      <c r="M19" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="N19" s="23" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="D20" s="22">
+        <v>2</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>251</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>252</v>
+      </c>
+      <c r="J20" s="23">
+        <v>2</v>
+      </c>
+      <c r="K20" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="L20" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="M20" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="N20" s="23" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="D21" s="22">
+        <v>3</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>253</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="J21" s="23">
+        <v>3</v>
+      </c>
+      <c r="K21" s="24" t="s">
+        <v>234</v>
+      </c>
+      <c r="L21" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="M21" s="23" t="s">
+        <v>245</v>
+      </c>
+      <c r="N21" s="23" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="D22" s="22">
+        <v>4</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>255</v>
+      </c>
+      <c r="F22" s="40" t="s">
+        <v>256</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="J22" s="23">
+        <v>4</v>
+      </c>
+      <c r="K22" s="24" t="s">
+        <v>237</v>
+      </c>
+      <c r="L22" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="M22" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="N22" s="23" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="D23" s="22">
+        <v>5</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>258</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>259</v>
+      </c>
+      <c r="G23" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="J23" s="23">
+        <v>5</v>
+      </c>
+      <c r="K23" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="L23" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="M23" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="N23" s="23" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B26" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D28" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="F28" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="G28" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="J28" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K28" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L28" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="M28" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="N28" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="P28" s="46" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D29" s="19">
+        <v>1</v>
+      </c>
+      <c r="E29" s="47" t="s">
+        <v>262</v>
+      </c>
+      <c r="F29" s="48" t="s">
+        <v>263</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>264</v>
+      </c>
+      <c r="J29" s="19">
+        <v>1</v>
+      </c>
+      <c r="K29" s="47" t="s">
+        <v>275</v>
+      </c>
+      <c r="L29" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="M29" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="N29" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="P29" s="51"/>
+    </row>
+    <row r="30" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D30" s="19">
+        <v>2</v>
+      </c>
+      <c r="E30" s="47" t="s">
+        <v>265</v>
+      </c>
+      <c r="F30" s="48" t="s">
+        <v>266</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="J30" s="19">
+        <v>2</v>
+      </c>
+      <c r="K30" s="47" t="s">
+        <v>278</v>
+      </c>
+      <c r="L30" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="M30" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="N30" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="P30" s="51" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D31" s="19">
+        <v>3</v>
+      </c>
+      <c r="E31" s="47" t="s">
+        <v>268</v>
+      </c>
+      <c r="F31" s="48" t="s">
+        <v>269</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="J31" s="19">
+        <v>3</v>
+      </c>
+      <c r="K31" s="47" t="s">
+        <v>282</v>
+      </c>
+      <c r="L31" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="N31" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="P31" s="51" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D32" s="19">
+        <v>4</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>271</v>
+      </c>
+      <c r="F32" s="48" t="s">
+        <v>272</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="J32" s="19">
+        <v>4</v>
+      </c>
+      <c r="K32" s="47" t="s">
+        <v>286</v>
+      </c>
+      <c r="L32" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="M32" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="N32" s="19" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J33" s="19">
+        <v>5</v>
+      </c>
+      <c r="K33" s="47" t="s">
+        <v>290</v>
+      </c>
+      <c r="L33" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="M33" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="N33" s="19" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B36" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D38" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="F38" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="G38" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="J38" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K38" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L38" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="M38" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="N38" s="45" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D39" s="19">
+        <v>1</v>
+      </c>
+      <c r="E39" s="47" t="s">
+        <v>298</v>
+      </c>
+      <c r="F39" s="48" t="s">
+        <v>299</v>
+      </c>
+      <c r="G39" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="J39" s="19">
+        <v>1</v>
+      </c>
+      <c r="K39" s="47" t="s">
+        <v>301</v>
+      </c>
+      <c r="L39" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="M39" s="48" t="s">
+        <v>302</v>
+      </c>
+      <c r="N39" s="19" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="J40" s="19">
+        <v>2</v>
+      </c>
+      <c r="K40" s="47" t="s">
+        <v>304</v>
+      </c>
+      <c r="L40" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="M40" s="48" t="s">
+        <v>302</v>
+      </c>
+      <c r="N40" s="19" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="41" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J41" s="19">
+        <v>3</v>
+      </c>
+      <c r="K41" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="L41" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="M41" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="N41" s="19" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J42" s="19">
+        <v>4</v>
+      </c>
+      <c r="K42" s="47" t="s">
+        <v>311</v>
+      </c>
+      <c r="L42" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="M42" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="N42" s="19" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="43" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J43" s="19">
+        <v>5</v>
+      </c>
+      <c r="K43" s="47" t="s">
+        <v>314</v>
+      </c>
+      <c r="L43" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="M43" s="48" t="s">
+        <v>302</v>
+      </c>
+      <c r="N43" s="19" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J44" s="19">
+        <v>6</v>
+      </c>
+      <c r="K44" s="47" t="s">
+        <v>317</v>
+      </c>
+      <c r="L44" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="M44" s="48" t="s">
+        <v>319</v>
+      </c>
+      <c r="N44" s="19" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="47" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B47" s="13" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D49" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E49" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="F49" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="G49" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="J49" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K49" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L49" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="M49" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="N49" s="45" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="50" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D50" s="19">
+        <v>1</v>
+      </c>
+      <c r="E50" s="47" t="s">
+        <v>352</v>
+      </c>
+      <c r="F50" s="48" t="s">
+        <v>353</v>
+      </c>
+      <c r="G50" s="19" t="s">
+        <v>354</v>
+      </c>
+      <c r="J50" s="19">
+        <v>1</v>
+      </c>
+      <c r="K50" s="47" t="s">
+        <v>361</v>
+      </c>
+      <c r="L50" s="19" t="s">
+        <v>362</v>
+      </c>
+      <c r="M50" s="48" t="s">
+        <v>363</v>
+      </c>
+      <c r="N50" s="19" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D51" s="19">
+        <v>2</v>
+      </c>
+      <c r="E51" s="47" t="s">
+        <v>355</v>
+      </c>
+      <c r="F51" s="48" t="s">
+        <v>356</v>
+      </c>
+      <c r="G51" s="19" t="s">
+        <v>357</v>
+      </c>
+      <c r="J51" s="19">
+        <v>2</v>
+      </c>
+      <c r="K51" s="47" t="s">
+        <v>365</v>
+      </c>
+      <c r="L51" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="M51" s="48" t="s">
+        <v>367</v>
+      </c>
+      <c r="N51" s="19" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D52" s="19">
+        <v>3</v>
+      </c>
+      <c r="E52" s="47" t="s">
+        <v>358</v>
+      </c>
+      <c r="F52" s="48" t="s">
+        <v>359</v>
+      </c>
+      <c r="G52" s="19" t="s">
+        <v>360</v>
+      </c>
+      <c r="J52" s="19">
+        <v>3</v>
+      </c>
+      <c r="K52" s="47" t="s">
+        <v>369</v>
+      </c>
+      <c r="L52" s="19" t="s">
+        <v>370</v>
+      </c>
+      <c r="M52" s="48" t="s">
+        <v>371</v>
+      </c>
+      <c r="N52" s="19" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="J53" s="19">
+        <v>4</v>
+      </c>
+      <c r="K53" s="47" t="s">
+        <v>373</v>
+      </c>
+      <c r="L53" s="19" t="s">
+        <v>374</v>
+      </c>
+      <c r="M53" s="48" t="s">
+        <v>375</v>
+      </c>
+      <c r="N53" s="19" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="63" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B63" s="13" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="65" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D65" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E65" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="F65" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="G65" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="J65" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K65" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L65" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="M65" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="N65" s="45" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="66" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D66" s="19">
+        <v>1</v>
+      </c>
+      <c r="E66" s="47" t="s">
+        <v>323</v>
+      </c>
+      <c r="F66" s="48" t="s">
+        <v>324</v>
+      </c>
+      <c r="G66" s="19" t="s">
+        <v>325</v>
+      </c>
+      <c r="J66" s="19">
+        <v>1</v>
+      </c>
+      <c r="K66" s="47" t="s">
+        <v>329</v>
+      </c>
+      <c r="L66" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="M66" s="48" t="s">
+        <v>330</v>
+      </c>
+      <c r="N66" s="19" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="67" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D67" s="19">
+        <v>2</v>
+      </c>
+      <c r="E67" s="47" t="s">
+        <v>326</v>
+      </c>
+      <c r="F67" s="48" t="s">
+        <v>327</v>
+      </c>
+      <c r="G67" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="J67" s="19">
+        <v>2</v>
+      </c>
+      <c r="K67" s="47" t="s">
+        <v>332</v>
+      </c>
+      <c r="L67" s="19" t="s">
+        <v>333</v>
+      </c>
+      <c r="M67" s="48" t="s">
+        <v>334</v>
+      </c>
+      <c r="N67" s="19" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="68" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J68" s="19">
+        <v>3</v>
+      </c>
+      <c r="K68" s="47" t="s">
+        <v>336</v>
+      </c>
+      <c r="L68" s="19" t="s">
+        <v>337</v>
+      </c>
+      <c r="M68" s="48" t="s">
+        <v>338</v>
+      </c>
+      <c r="N68" s="19" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="69" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="J69" s="19">
+        <v>4</v>
+      </c>
+      <c r="K69" s="47" t="s">
+        <v>340</v>
+      </c>
+      <c r="L69" s="19" t="s">
+        <v>341</v>
+      </c>
+      <c r="M69" s="48" t="s">
+        <v>342</v>
+      </c>
+      <c r="N69" s="19" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="70" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J70" s="19">
+        <v>5</v>
+      </c>
+      <c r="K70" s="47" t="s">
+        <v>344</v>
+      </c>
+      <c r="L70" s="19" t="s">
+        <v>345</v>
+      </c>
+      <c r="M70" s="48" t="s">
+        <v>346</v>
+      </c>
+      <c r="N70" s="19" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="71" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J71" s="19">
+        <v>6</v>
+      </c>
+      <c r="K71" s="47" t="s">
+        <v>348</v>
+      </c>
+      <c r="L71" s="19" t="s">
+        <v>349</v>
+      </c>
+      <c r="M71" s="48" t="s">
+        <v>350</v>
+      </c>
+      <c r="N71" s="19" t="s">
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -3210,141 +5372,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4BAE5E-D7E8-4F3F-BBD9-8CAD9399CE65}">
-  <dimension ref="C2:G16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.6640625" customWidth="1"/>
-    <col min="5" max="5" width="30.33203125" customWidth="1"/>
-    <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="52.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="3:7" ht="25.8">
-      <c r="C2" s="36" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" spans="3:7" ht="18">
-      <c r="D4" s="37" t="s">
-        <v>161</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="3:7" ht="31.2">
-      <c r="D5" s="28">
-        <v>1</v>
-      </c>
-      <c r="E5" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="F5" s="35" t="s">
-        <v>165</v>
-      </c>
-      <c r="G5" s="27" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="6" spans="3:7" ht="31.2">
-      <c r="D6" s="28">
-        <v>2</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>168</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="7" spans="3:7" ht="31.2">
-      <c r="D7" s="28">
-        <v>3</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="F7" s="35" t="s">
-        <v>171</v>
-      </c>
-      <c r="G7" s="27" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="8" spans="3:7" ht="45">
-      <c r="D8" s="28">
-        <v>4</v>
-      </c>
-      <c r="E8" s="26" t="s">
-        <v>173</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>174</v>
-      </c>
-      <c r="G8" s="27" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="3:7">
-      <c r="D12" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="13" spans="3:7" ht="28.8">
-      <c r="D13" s="34" t="s">
-        <v>178</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="14" spans="3:7">
-      <c r="D14" s="34" t="s">
-        <v>180</v>
-      </c>
-      <c r="E14" s="33" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="15" spans="3:7">
-      <c r="D15" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="E15" s="33" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="16" spans="3:7">
-      <c r="D16" s="34" t="s">
-        <v>184</v>
-      </c>
-      <c r="E16" s="33" t="s">
-        <v>185</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D08B4F4-38F3-4EC4-8131-B24327749222}">
-  <dimension ref="B3:H12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="B3:H36"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.21875" bestFit="1" customWidth="1"/>
@@ -3354,12 +5384,12 @@
     <col min="7" max="7" width="54.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="25.8">
+    <row r="3" spans="2:8" ht="25.8" x14ac:dyDescent="0.5">
       <c r="B3" s="29" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="31.2">
+    <row r="5" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="C5" s="30" t="s">
         <v>126</v>
       </c>
@@ -3379,7 +5409,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="46.8">
+    <row r="6" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="C6" s="28">
         <v>1</v>
       </c>
@@ -3397,7 +5427,7 @@
       </c>
       <c r="H6" s="32"/>
     </row>
-    <row r="7" spans="2:8" ht="46.8">
+    <row r="7" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="C7" s="28">
         <v>2</v>
       </c>
@@ -3415,7 +5445,7 @@
       </c>
       <c r="H7" s="32"/>
     </row>
-    <row r="8" spans="2:8" ht="31.2">
+    <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="C8" s="28">
         <v>3</v>
       </c>
@@ -3433,7 +5463,7 @@
       </c>
       <c r="H8" s="32"/>
     </row>
-    <row r="9" spans="2:8" ht="46.8">
+    <row r="9" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="C9" s="28">
         <v>4</v>
       </c>
@@ -3451,7 +5481,7 @@
       </c>
       <c r="H9" s="32"/>
     </row>
-    <row r="10" spans="2:8" ht="31.2">
+    <row r="10" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="C10" s="28">
         <v>5</v>
       </c>
@@ -3469,7 +5499,7 @@
       </c>
       <c r="H10" s="32"/>
     </row>
-    <row r="11" spans="2:8" ht="31.2">
+    <row r="11" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="C11" s="28">
         <v>6</v>
       </c>
@@ -3487,7 +5517,7 @@
       </c>
       <c r="H11" s="32"/>
     </row>
-    <row r="12" spans="2:8" ht="46.8">
+    <row r="12" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="C12" s="28" t="s">
         <v>149</v>
       </c>
@@ -3504,6 +5534,376 @@
         <v>153</v>
       </c>
       <c r="H12" s="32"/>
+    </row>
+    <row r="17" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C17" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="G17" s="34" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C18" s="45">
+        <v>1</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="G18" s="33" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C19" s="45">
+        <v>2</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>211</v>
+      </c>
+      <c r="F19" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C20" s="45">
+        <v>3</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>212</v>
+      </c>
+      <c r="F20" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="33" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C21" s="45">
+        <v>4</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="E21" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="F21" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="G21" s="33" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="22" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C22" s="45">
+        <v>5</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C23" s="45">
+        <v>6</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="F23" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="24" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C24" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="F24" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="G24" s="33" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="31" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="C31" s="34" t="s">
+        <v>216</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="34" t="s">
+        <v>186</v>
+      </c>
+      <c r="F31" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="G31" s="34" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C32" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="F32" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="G32" s="33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C33" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="E33" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="F33" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="G33" s="33" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C34" s="34" t="s">
+        <v>219</v>
+      </c>
+      <c r="D34" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="F34" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="G34" s="33" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C35" s="34" t="s">
+        <v>220</v>
+      </c>
+      <c r="D35" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="E35" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="F35" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="G35" s="33" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C36" s="34" t="s">
+        <v>221</v>
+      </c>
+      <c r="D36" s="34" t="s">
+        <v>203</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>204</v>
+      </c>
+      <c r="F36" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>206</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4BAE5E-D7E8-4F3F-BBD9-8CAD9399CE65}">
+  <dimension ref="C2:G16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="52.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:7" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="C2" s="36" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="3:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="D4" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="D5" s="28">
+        <v>1</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="D6" s="28">
+        <v>2</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="D7" s="28">
+        <v>3</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="3:7" ht="45" x14ac:dyDescent="0.3">
+      <c r="D8" s="28">
+        <v>4</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="D12" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D13" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="33" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="14" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="D14" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="D15" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="D16" s="34" t="s">
+        <v>184</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>185</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
work on product page
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2FF7BE-498E-4FDA-8B73-2A9C88CA4448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C17F29-9402-4E14-9AC0-3954A9FC0DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -2224,7 +2224,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2430,7 +2430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2566,6 +2566,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2882,7 +2885,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B3E6E2D-EEAD-4E4A-8798-C3B53E352FF0}">
   <dimension ref="B3:H30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" bestFit="1" customWidth="1"/>
@@ -2893,12 +2896,12 @@
     <col min="8" max="8" width="36.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:8" ht="25.8">
       <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:8" ht="21">
       <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
@@ -2906,7 +2909,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="15.6">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="15.6">
       <c r="B7" s="22">
         <v>1</v>
       </c>
@@ -2946,7 +2949,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="31.2">
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -2966,7 +2969,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="15.6">
       <c r="B9" s="22">
         <v>3</v>
       </c>
@@ -2986,7 +2989,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="31.2">
       <c r="B10" s="22">
         <v>4</v>
       </c>
@@ -3006,7 +3009,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="31.2">
       <c r="B11" s="22">
         <v>5</v>
       </c>
@@ -3026,7 +3029,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="31.2">
       <c r="B12" s="22">
         <v>6</v>
       </c>
@@ -3046,7 +3049,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="31.2">
       <c r="B13" s="22">
         <v>7</v>
       </c>
@@ -3066,7 +3069,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="31.2">
       <c r="B14" s="22">
         <v>8</v>
       </c>
@@ -3086,7 +3089,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" ht="31.2">
       <c r="B15" s="22">
         <v>9</v>
       </c>
@@ -3106,7 +3109,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="31.2">
       <c r="B16" s="22">
         <v>10</v>
       </c>
@@ -3126,7 +3129,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="31.2">
       <c r="B17" s="22">
         <v>11</v>
       </c>
@@ -3146,7 +3149,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="31.2">
       <c r="B18" s="22">
         <v>12</v>
       </c>
@@ -3166,7 +3169,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" ht="15.6">
       <c r="B19" s="22">
         <v>13</v>
       </c>
@@ -3186,7 +3189,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="15.6">
       <c r="B20" s="22">
         <v>14</v>
       </c>
@@ -3206,7 +3209,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="15.6">
       <c r="B21" s="22">
         <v>15</v>
       </c>
@@ -3226,7 +3229,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="31.2">
       <c r="B22" s="22">
         <v>16</v>
       </c>
@@ -3246,7 +3249,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="31.2">
       <c r="B23" s="22">
         <v>17</v>
       </c>
@@ -3266,7 +3269,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="15.6">
       <c r="B24" s="22">
         <v>18</v>
       </c>
@@ -3286,7 +3289,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="15.6">
       <c r="B25" s="22">
         <v>19</v>
       </c>
@@ -3306,7 +3309,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="31.2">
       <c r="B26" s="22">
         <v>20</v>
       </c>
@@ -3326,7 +3329,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="31.2">
       <c r="B27" s="22">
         <v>21</v>
       </c>
@@ -3346,7 +3349,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="31.2">
       <c r="B28" s="22">
         <v>22</v>
       </c>
@@ -3366,7 +3369,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="31.2">
       <c r="B29" s="22">
         <v>23</v>
       </c>
@@ -3384,7 +3387,7 @@
       </c>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="31.2">
       <c r="B30" s="22">
         <v>24</v>
       </c>
@@ -3403,7 +3406,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6ADD15-B19C-416D-8A8B-7194E6C0A6D6}">
   <dimension ref="B3:K26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.77734375" bestFit="1" customWidth="1"/>
@@ -3417,12 +3420,12 @@
     <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:11" ht="25.8">
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:11" ht="15.6">
       <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:11" ht="15.6">
       <c r="B6" s="20">
         <v>0</v>
       </c>
@@ -3481,7 +3484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:11" ht="15.6">
       <c r="B7" s="20">
         <v>1</v>
       </c>
@@ -3513,7 +3516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:11" ht="15.6">
       <c r="B8" s="20">
         <v>2</v>
       </c>
@@ -3545,7 +3548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:11" ht="15.6">
       <c r="B9" s="20">
         <v>3</v>
       </c>
@@ -3577,7 +3580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:11" ht="15.6">
       <c r="B10" s="20">
         <v>4</v>
       </c>
@@ -3609,7 +3612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:11" ht="15.6">
       <c r="B11" s="20">
         <v>5</v>
       </c>
@@ -3641,7 +3644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:11" ht="15.6">
       <c r="B12" s="20">
         <v>6</v>
       </c>
@@ -3672,7 +3675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:11" ht="15.6">
       <c r="B13" s="20">
         <v>7</v>
       </c>
@@ -3703,7 +3706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:11" ht="15.6">
       <c r="B14" s="20">
         <v>8</v>
       </c>
@@ -3734,7 +3737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:11" ht="15.6">
       <c r="B15" s="20">
         <v>9</v>
       </c>
@@ -3768,7 +3771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:11" ht="15.6">
       <c r="B16" s="20">
         <v>10</v>
       </c>
@@ -3801,7 +3804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" ht="15.6">
       <c r="B17" s="20">
         <v>11</v>
       </c>
@@ -3835,7 +3838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:11" ht="15.6">
       <c r="B18" s="20">
         <v>12</v>
       </c>
@@ -3868,7 +3871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:11" ht="15.6">
       <c r="B19" s="20">
         <v>13</v>
       </c>
@@ -3901,7 +3904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:11" ht="15.6">
       <c r="B20" s="20">
         <v>14</v>
       </c>
@@ -3934,7 +3937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:11" ht="15.6">
       <c r="B21" s="20">
         <v>15</v>
       </c>
@@ -3967,7 +3970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:11" ht="15.6">
       <c r="B22" s="20">
         <v>16</v>
       </c>
@@ -4000,7 +4003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:11" ht="15.6">
       <c r="B23" s="20">
         <v>17</v>
       </c>
@@ -4033,7 +4036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:11" ht="15.6">
       <c r="B24" s="20">
         <v>18</v>
       </c>
@@ -4066,7 +4069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:11" ht="15.6">
       <c r="B25" s="20">
         <v>19</v>
       </c>
@@ -4099,7 +4102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:11" ht="15.6">
       <c r="B26" s="20">
         <v>20</v>
       </c>
@@ -4140,7 +4143,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7AAEBDA-2918-4347-B5CD-94210A58680A}">
   <dimension ref="B3:J13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -4148,12 +4151,12 @@
     <col min="10" max="10" width="190.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="25.8">
       <c r="D3" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" ht="15.6">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -4164,7 +4167,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10">
       <c r="I7">
         <v>1</v>
       </c>
@@ -4172,7 +4175,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10">
       <c r="I8">
         <v>2</v>
       </c>
@@ -4180,7 +4183,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10">
       <c r="I9">
         <v>3</v>
       </c>
@@ -4188,7 +4191,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10">
       <c r="I10">
         <v>4</v>
       </c>
@@ -4196,7 +4199,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10">
       <c r="I11">
         <v>5</v>
       </c>
@@ -4204,7 +4207,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10">
       <c r="I12">
         <v>6</v>
       </c>
@@ -4212,7 +4215,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10">
       <c r="I13">
         <v>7</v>
       </c>
@@ -4228,7 +4231,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FDCB3-6CAE-4927-8D50-CB20F0599746}">
   <dimension ref="B3:S71"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.109375" bestFit="1" customWidth="1"/>
@@ -4247,7 +4250,7 @@
     <col min="19" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:19" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:19" ht="23.4">
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -4269,7 +4272,7 @@
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
     </row>
-    <row r="5" spans="2:19" ht="21" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:19" ht="21">
       <c r="B5" s="13" t="s">
         <v>207</v>
       </c>
@@ -4301,7 +4304,7 @@
       </c>
       <c r="S5" s="11"/>
     </row>
-    <row r="7" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:19" ht="15.6">
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="18" t="s">
@@ -4345,7 +4348,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:19" ht="31.2">
       <c r="D8" s="44">
         <v>1</v>
       </c>
@@ -4383,7 +4386,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:19" ht="31.2">
       <c r="D9" s="44">
         <v>2</v>
       </c>
@@ -4421,7 +4424,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:19" ht="31.2">
       <c r="D10" s="44">
         <v>3</v>
       </c>
@@ -4459,7 +4462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:19" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:19" ht="46.8">
       <c r="D11" s="44">
         <v>4</v>
       </c>
@@ -4497,7 +4500,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:19" ht="31.2">
       <c r="J12" s="44">
         <v>5</v>
       </c>
@@ -4523,7 +4526,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:19" ht="15.6">
       <c r="Q13" s="22">
         <v>6</v>
       </c>
@@ -4534,7 +4537,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:19" ht="31.2">
       <c r="Q14" s="22">
         <v>7</v>
       </c>
@@ -4545,7 +4548,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="2:19" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:19" ht="20.399999999999999">
       <c r="B16" s="13" t="s">
         <v>209</v>
       </c>
@@ -4556,7 +4559,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" ht="15.6">
       <c r="D18" s="49" t="s">
         <v>7</v>
       </c>
@@ -4585,11 +4588,11 @@
         <v>223</v>
       </c>
     </row>
-    <row r="19" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" ht="39.6">
       <c r="D19" s="22">
         <v>1</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="52" t="s">
         <v>224</v>
       </c>
       <c r="F19" s="40" t="s">
@@ -4614,11 +4617,11 @@
         <v>230</v>
       </c>
     </row>
-    <row r="20" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" ht="39.6">
       <c r="D20" s="22">
         <v>2</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="52" t="s">
         <v>225</v>
       </c>
       <c r="F20" s="40" t="s">
@@ -4643,11 +4646,11 @@
         <v>233</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" ht="39.6">
       <c r="D21" s="22">
         <v>3</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="E21" s="52" t="s">
         <v>226</v>
       </c>
       <c r="F21" s="40" t="s">
@@ -4672,7 +4675,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" ht="31.2">
       <c r="D22" s="22">
         <v>4</v>
       </c>
@@ -4701,7 +4704,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" ht="46.8">
       <c r="D23" s="22">
         <v>5</v>
       </c>
@@ -4730,7 +4733,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="26" spans="2:16" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" ht="20.399999999999999">
       <c r="B26" s="13" t="s">
         <v>31</v>
       </c>
@@ -4741,7 +4744,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16">
       <c r="D28" s="45" t="s">
         <v>7</v>
       </c>
@@ -4773,7 +4776,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="29" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" ht="28.8">
       <c r="D29" s="19">
         <v>1</v>
       </c>
@@ -4803,7 +4806,7 @@
       </c>
       <c r="P29" s="51"/>
     </row>
-    <row r="30" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" ht="28.8">
       <c r="D30" s="19">
         <v>2</v>
       </c>
@@ -4835,7 +4838,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" ht="43.2">
       <c r="D31" s="19">
         <v>3</v>
       </c>
@@ -4867,7 +4870,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="32" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" ht="28.8">
       <c r="D32" s="19">
         <v>4</v>
       </c>
@@ -4896,7 +4899,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="33" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:14" ht="28.8">
       <c r="J33" s="19">
         <v>5</v>
       </c>
@@ -4913,7 +4916,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="36" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:14" ht="20.399999999999999">
       <c r="B36" s="13" t="s">
         <v>294</v>
       </c>
@@ -4924,7 +4927,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:14">
       <c r="D38" s="45" t="s">
         <v>7</v>
       </c>
@@ -4953,7 +4956,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="39" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:14" ht="28.8">
       <c r="D39" s="19">
         <v>1</v>
       </c>
@@ -4982,7 +4985,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:14">
       <c r="J40" s="19">
         <v>2</v>
       </c>
@@ -4999,7 +5002,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="41" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:14" ht="28.8">
       <c r="J41" s="19">
         <v>3</v>
       </c>
@@ -5016,7 +5019,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="42" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:14" ht="28.8">
       <c r="J42" s="19">
         <v>4</v>
       </c>
@@ -5033,7 +5036,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="43" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:14" ht="28.8">
       <c r="J43" s="19">
         <v>5</v>
       </c>
@@ -5050,7 +5053,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="44" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:14" ht="28.8">
       <c r="J44" s="19">
         <v>6</v>
       </c>
@@ -5067,12 +5070,12 @@
         <v>320</v>
       </c>
     </row>
-    <row r="47" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:14" ht="20.399999999999999">
       <c r="B47" s="13" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:14">
       <c r="D49" s="45" t="s">
         <v>7</v>
       </c>
@@ -5101,7 +5104,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="50" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:14" ht="28.8">
       <c r="D50" s="19">
         <v>1</v>
       </c>
@@ -5130,7 +5133,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="51" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:14" ht="28.8">
       <c r="D51" s="19">
         <v>2</v>
       </c>
@@ -5159,7 +5162,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="52" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:14" ht="28.8">
       <c r="D52" s="19">
         <v>3</v>
       </c>
@@ -5188,7 +5191,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:14">
       <c r="J53" s="19">
         <v>4</v>
       </c>
@@ -5205,12 +5208,12 @@
         <v>376</v>
       </c>
     </row>
-    <row r="63" spans="2:14" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:14" ht="20.399999999999999">
       <c r="B63" s="13" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="65" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:14">
       <c r="D65" s="45" t="s">
         <v>7</v>
       </c>
@@ -5239,7 +5242,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="66" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="4:14" ht="28.8">
       <c r="D66" s="19">
         <v>1</v>
       </c>
@@ -5268,7 +5271,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="67" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:14" ht="28.8">
       <c r="D67" s="19">
         <v>2</v>
       </c>
@@ -5297,7 +5300,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="68" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:14" ht="28.8">
       <c r="J68" s="19">
         <v>3</v>
       </c>
@@ -5314,7 +5317,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="69" spans="4:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="4:14">
       <c r="J69" s="19">
         <v>4</v>
       </c>
@@ -5331,7 +5334,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="70" spans="4:14" ht="28.8">
       <c r="J70" s="19">
         <v>5</v>
       </c>
@@ -5348,7 +5351,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="71" spans="4:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:14" ht="28.8">
       <c r="J71" s="19">
         <v>6</v>
       </c>
@@ -5374,7 +5377,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D08B4F4-38F3-4EC4-8131-B24327749222}">
   <dimension ref="B3:H36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.21875" bestFit="1" customWidth="1"/>
@@ -5384,12 +5387,12 @@
     <col min="7" max="7" width="54.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:8" ht="25.8">
       <c r="B3" s="29" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="31.2">
       <c r="C5" s="30" t="s">
         <v>126</v>
       </c>
@@ -5409,7 +5412,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="46.8">
       <c r="C6" s="28">
         <v>1</v>
       </c>
@@ -5427,7 +5430,7 @@
       </c>
       <c r="H6" s="32"/>
     </row>
-    <row r="7" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="46.8">
       <c r="C7" s="28">
         <v>2</v>
       </c>
@@ -5445,7 +5448,7 @@
       </c>
       <c r="H7" s="32"/>
     </row>
-    <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="31.2">
       <c r="C8" s="28">
         <v>3</v>
       </c>
@@ -5463,7 +5466,7 @@
       </c>
       <c r="H8" s="32"/>
     </row>
-    <row r="9" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="46.8">
       <c r="C9" s="28">
         <v>4</v>
       </c>
@@ -5481,7 +5484,7 @@
       </c>
       <c r="H9" s="32"/>
     </row>
-    <row r="10" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="31.2">
       <c r="C10" s="28">
         <v>5</v>
       </c>
@@ -5499,7 +5502,7 @@
       </c>
       <c r="H10" s="32"/>
     </row>
-    <row r="11" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="31.2">
       <c r="C11" s="28">
         <v>6</v>
       </c>
@@ -5517,7 +5520,7 @@
       </c>
       <c r="H11" s="32"/>
     </row>
-    <row r="12" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="46.8">
       <c r="C12" s="28" t="s">
         <v>149</v>
       </c>
@@ -5535,7 +5538,7 @@
       </c>
       <c r="H12" s="32"/>
     </row>
-    <row r="17" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:7" ht="28.8">
       <c r="C17" s="45" t="s">
         <v>126</v>
       </c>
@@ -5552,7 +5555,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:7" ht="28.8">
       <c r="C18" s="45">
         <v>1</v>
       </c>
@@ -5569,7 +5572,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="19" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:7" ht="43.2">
       <c r="C19" s="45">
         <v>2</v>
       </c>
@@ -5586,7 +5589,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:7" ht="28.8">
       <c r="C20" s="45">
         <v>3</v>
       </c>
@@ -5603,7 +5606,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:7" ht="28.8">
       <c r="C21" s="45">
         <v>4</v>
       </c>
@@ -5620,7 +5623,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:7" ht="28.8">
       <c r="C22" s="45">
         <v>5</v>
       </c>
@@ -5637,7 +5640,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="23" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:7" ht="28.8">
       <c r="C23" s="45">
         <v>6</v>
       </c>
@@ -5654,7 +5657,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:7" ht="43.2">
       <c r="C24" s="45" t="s">
         <v>149</v>
       </c>
@@ -5671,7 +5674,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:7">
       <c r="C31" s="34" t="s">
         <v>216</v>
       </c>
@@ -5688,7 +5691,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:7" ht="43.2">
       <c r="C32" s="34" t="s">
         <v>217</v>
       </c>
@@ -5705,7 +5708,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="33" spans="3:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:7" ht="57.6">
       <c r="C33" s="34" t="s">
         <v>218</v>
       </c>
@@ -5722,7 +5725,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="34" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:7" ht="43.2">
       <c r="C34" s="34" t="s">
         <v>219</v>
       </c>
@@ -5739,7 +5742,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="35" spans="3:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:7" ht="86.4">
       <c r="C35" s="34" t="s">
         <v>220</v>
       </c>
@@ -5756,7 +5759,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="36" spans="3:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:7" ht="86.4">
       <c r="C36" s="34" t="s">
         <v>221</v>
       </c>
@@ -5781,7 +5784,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4BAE5E-D7E8-4F3F-BBD9-8CAD9399CE65}">
   <dimension ref="C2:G16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
@@ -5790,12 +5793,12 @@
     <col min="7" max="7" width="52.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:7" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="2" spans="3:7" ht="25.8">
       <c r="C2" s="36" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="3:7" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:7" ht="18">
       <c r="D4" s="37" t="s">
         <v>161</v>
       </c>
@@ -5809,7 +5812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:7" ht="31.2">
       <c r="D5" s="28">
         <v>1</v>
       </c>
@@ -5823,7 +5826,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="6" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:7" ht="31.2">
       <c r="D6" s="28">
         <v>2</v>
       </c>
@@ -5837,7 +5840,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="7" spans="3:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:7" ht="31.2">
       <c r="D7" s="28">
         <v>3</v>
       </c>
@@ -5851,7 +5854,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="8" spans="3:7" ht="45" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:7" ht="60">
       <c r="D8" s="28">
         <v>4</v>
       </c>
@@ -5865,7 +5868,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:7">
       <c r="D12" s="34" t="s">
         <v>176</v>
       </c>
@@ -5873,7 +5876,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="13" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:7" ht="28.8">
       <c r="D13" s="34" t="s">
         <v>178</v>
       </c>
@@ -5881,7 +5884,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:7">
       <c r="D14" s="34" t="s">
         <v>180</v>
       </c>
@@ -5889,7 +5892,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="15" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:7">
       <c r="D15" s="34" t="s">
         <v>182</v>
       </c>
@@ -5897,7 +5900,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="16" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:7">
       <c r="D16" s="34" t="s">
         <v>184</v>
       </c>

</xml_diff>

<commit_message>
Work on Fulfilment Page & Report
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C17F29-9402-4E14-9AC0-3954A9FC0DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD1FE65-57DF-4554-8148-50800044C42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="374">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -1389,15 +1389,6 @@
   </si>
   <si>
     <t>Finds the average sales per category to compare overall product strength.</t>
-  </si>
-  <si>
-    <t>Category Contribution % (Top vs Rest)</t>
-  </si>
-  <si>
-    <t>Category Contribution % = DIVIDE([Top Category Sales], [Total Sales])</t>
-  </si>
-  <si>
-    <t>Shows how much percentage of total revenue comes from the top-selling category.</t>
   </si>
   <si>
     <t>Globle</t>
@@ -2567,8 +2558,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4300,7 +4291,7 @@
       </c>
       <c r="Q5" s="11"/>
       <c r="R5" s="11" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="S5" s="11"/>
     </row>
@@ -4462,7 +4453,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:19" ht="46.8">
+    <row r="11" spans="2:19" ht="31.2">
       <c r="D11" s="44">
         <v>4</v>
       </c>
@@ -4679,7 +4670,7 @@
       <c r="D22" s="22">
         <v>4</v>
       </c>
-      <c r="E22" s="26" t="s">
+      <c r="E22" s="52" t="s">
         <v>255</v>
       </c>
       <c r="F22" s="40" t="s">
@@ -4704,19 +4695,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="46.8">
-      <c r="D23" s="22">
-        <v>5</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>258</v>
-      </c>
-      <c r="F23" s="40" t="s">
-        <v>259</v>
-      </c>
-      <c r="G23" s="27" t="s">
-        <v>260</v>
-      </c>
+    <row r="23" spans="2:16" ht="31.2">
       <c r="J23" s="23">
         <v>5</v>
       </c>
@@ -4764,7 +4743,7 @@
         <v>25</v>
       </c>
       <c r="L28" s="45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="M28" s="45" t="s">
         <v>24</v>
@@ -4773,7 +4752,7 @@
         <v>223</v>
       </c>
       <c r="P28" s="46" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="2:16" ht="28.8">
@@ -4781,28 +4760,28 @@
         <v>1</v>
       </c>
       <c r="E29" s="47" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F29" s="48" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="J29" s="19">
         <v>1</v>
       </c>
       <c r="K29" s="47" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="L29" s="19" t="s">
         <v>192</v>
       </c>
       <c r="M29" s="19" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="N29" s="19" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="P29" s="51"/>
     </row>
@@ -4811,31 +4790,31 @@
         <v>2</v>
       </c>
       <c r="E30" s="47" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F30" s="48" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="J30" s="19">
         <v>2</v>
       </c>
       <c r="K30" s="47" t="s">
+        <v>275</v>
+      </c>
+      <c r="L30" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="M30" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="N30" s="19" t="s">
         <v>278</v>
       </c>
-      <c r="L30" s="19" t="s">
-        <v>279</v>
-      </c>
-      <c r="M30" s="19" t="s">
-        <v>280</v>
-      </c>
-      <c r="N30" s="19" t="s">
-        <v>281</v>
-      </c>
       <c r="P30" s="51" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="43.2">
@@ -4843,31 +4822,31 @@
         <v>3</v>
       </c>
       <c r="E31" s="47" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F31" s="48" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="J31" s="19">
         <v>3</v>
       </c>
       <c r="K31" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="L31" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="N31" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="L31" s="19" t="s">
-        <v>283</v>
-      </c>
-      <c r="M31" s="19" t="s">
-        <v>284</v>
-      </c>
-      <c r="N31" s="19" t="s">
-        <v>285</v>
-      </c>
       <c r="P31" s="51" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" spans="2:16" ht="28.8">
@@ -4875,28 +4854,28 @@
         <v>4</v>
       </c>
       <c r="E32" s="47" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="F32" s="48" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="J32" s="19">
         <v>4</v>
       </c>
       <c r="K32" s="47" t="s">
+        <v>283</v>
+      </c>
+      <c r="L32" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="M32" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="N32" s="19" t="s">
         <v>286</v>
-      </c>
-      <c r="L32" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="M32" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="N32" s="19" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="33" spans="2:14" ht="28.8">
@@ -4904,21 +4883,21 @@
         <v>5</v>
       </c>
       <c r="K33" s="47" t="s">
+        <v>287</v>
+      </c>
+      <c r="L33" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="M33" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="N33" s="19" t="s">
         <v>290</v>
-      </c>
-      <c r="L33" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="M33" s="19" t="s">
-        <v>292</v>
-      </c>
-      <c r="N33" s="19" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="36" spans="2:14" ht="20.399999999999999">
       <c r="B36" s="13" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D36" s="15" t="s">
         <v>18</v>
@@ -4947,7 +4926,7 @@
         <v>25</v>
       </c>
       <c r="L38" s="45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="M38" s="45" t="s">
         <v>24</v>
@@ -4961,28 +4940,28 @@
         <v>1</v>
       </c>
       <c r="E39" s="47" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F39" s="48" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J39" s="19">
         <v>1</v>
       </c>
       <c r="K39" s="47" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="L39" s="19" t="s">
         <v>196</v>
       </c>
       <c r="M39" s="48" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="N39" s="19" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40" spans="2:14">
@@ -4990,16 +4969,16 @@
         <v>2</v>
       </c>
       <c r="K40" s="47" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="L40" s="19" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="M40" s="48" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="N40" s="19" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="41" spans="2:14" ht="28.8">
@@ -5007,16 +4986,16 @@
         <v>3</v>
       </c>
       <c r="K41" s="47" t="s">
+        <v>304</v>
+      </c>
+      <c r="L41" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="M41" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="N41" s="19" t="s">
         <v>307</v>
-      </c>
-      <c r="L41" s="19" t="s">
-        <v>308</v>
-      </c>
-      <c r="M41" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="N41" s="19" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="42" spans="2:14" ht="28.8">
@@ -5024,16 +5003,16 @@
         <v>4</v>
       </c>
       <c r="K42" s="47" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="L42" s="19" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="M42" s="48" t="s">
         <v>61</v>
       </c>
       <c r="N42" s="19" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43" spans="2:14" ht="28.8">
@@ -5041,16 +5020,16 @@
         <v>5</v>
       </c>
       <c r="K43" s="47" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="L43" s="19" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="M43" s="48" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="N43" s="19" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="44" spans="2:14" ht="28.8">
@@ -5058,21 +5037,21 @@
         <v>6</v>
       </c>
       <c r="K44" s="47" t="s">
+        <v>314</v>
+      </c>
+      <c r="L44" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="M44" s="48" t="s">
+        <v>316</v>
+      </c>
+      <c r="N44" s="19" t="s">
         <v>317</v>
-      </c>
-      <c r="L44" s="19" t="s">
-        <v>318</v>
-      </c>
-      <c r="M44" s="48" t="s">
-        <v>319</v>
-      </c>
-      <c r="N44" s="19" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="47" spans="2:14" ht="20.399999999999999">
       <c r="B47" s="13" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="49" spans="2:14">
@@ -5095,7 +5074,7 @@
         <v>25</v>
       </c>
       <c r="L49" s="45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="M49" s="45" t="s">
         <v>24</v>
@@ -5109,28 +5088,28 @@
         <v>1</v>
       </c>
       <c r="E50" s="47" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F50" s="48" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="J50" s="19">
         <v>1</v>
       </c>
       <c r="K50" s="47" t="s">
+        <v>358</v>
+      </c>
+      <c r="L50" s="19" t="s">
+        <v>359</v>
+      </c>
+      <c r="M50" s="48" t="s">
+        <v>360</v>
+      </c>
+      <c r="N50" s="19" t="s">
         <v>361</v>
-      </c>
-      <c r="L50" s="19" t="s">
-        <v>362</v>
-      </c>
-      <c r="M50" s="48" t="s">
-        <v>363</v>
-      </c>
-      <c r="N50" s="19" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="51" spans="2:14" ht="28.8">
@@ -5138,28 +5117,28 @@
         <v>2</v>
       </c>
       <c r="E51" s="47" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F51" s="48" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="J51" s="19">
         <v>2</v>
       </c>
       <c r="K51" s="47" t="s">
+        <v>362</v>
+      </c>
+      <c r="L51" s="19" t="s">
+        <v>363</v>
+      </c>
+      <c r="M51" s="48" t="s">
+        <v>364</v>
+      </c>
+      <c r="N51" s="19" t="s">
         <v>365</v>
-      </c>
-      <c r="L51" s="19" t="s">
-        <v>366</v>
-      </c>
-      <c r="M51" s="48" t="s">
-        <v>367</v>
-      </c>
-      <c r="N51" s="19" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="52" spans="2:14" ht="28.8">
@@ -5167,28 +5146,28 @@
         <v>3</v>
       </c>
       <c r="E52" s="47" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="F52" s="48" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="J52" s="19">
         <v>3</v>
       </c>
       <c r="K52" s="47" t="s">
+        <v>366</v>
+      </c>
+      <c r="L52" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="M52" s="48" t="s">
+        <v>368</v>
+      </c>
+      <c r="N52" s="19" t="s">
         <v>369</v>
-      </c>
-      <c r="L52" s="19" t="s">
-        <v>370</v>
-      </c>
-      <c r="M52" s="48" t="s">
-        <v>371</v>
-      </c>
-      <c r="N52" s="19" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="53" spans="2:14">
@@ -5196,21 +5175,21 @@
         <v>4</v>
       </c>
       <c r="K53" s="47" t="s">
+        <v>370</v>
+      </c>
+      <c r="L53" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="M53" s="48" t="s">
+        <v>372</v>
+      </c>
+      <c r="N53" s="19" t="s">
         <v>373</v>
-      </c>
-      <c r="L53" s="19" t="s">
-        <v>374</v>
-      </c>
-      <c r="M53" s="48" t="s">
-        <v>375</v>
-      </c>
-      <c r="N53" s="19" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="63" spans="2:14" ht="20.399999999999999">
       <c r="B63" s="13" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="65" spans="4:14">
@@ -5233,7 +5212,7 @@
         <v>25</v>
       </c>
       <c r="L65" s="45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="M65" s="45" t="s">
         <v>24</v>
@@ -5247,28 +5226,28 @@
         <v>1</v>
       </c>
       <c r="E66" s="47" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F66" s="48" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="J66" s="19">
         <v>1</v>
       </c>
       <c r="K66" s="47" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="L66" s="19" t="s">
         <v>204</v>
       </c>
       <c r="M66" s="48" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="N66" s="19" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="67" spans="4:14" ht="28.8">
@@ -5276,28 +5255,28 @@
         <v>2</v>
       </c>
       <c r="E67" s="47" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F67" s="48" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="G67" s="19" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="J67" s="19">
         <v>2</v>
       </c>
       <c r="K67" s="47" t="s">
+        <v>329</v>
+      </c>
+      <c r="L67" s="19" t="s">
+        <v>330</v>
+      </c>
+      <c r="M67" s="48" t="s">
+        <v>331</v>
+      </c>
+      <c r="N67" s="19" t="s">
         <v>332</v>
-      </c>
-      <c r="L67" s="19" t="s">
-        <v>333</v>
-      </c>
-      <c r="M67" s="48" t="s">
-        <v>334</v>
-      </c>
-      <c r="N67" s="19" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="68" spans="4:14" ht="28.8">
@@ -5305,16 +5284,16 @@
         <v>3</v>
       </c>
       <c r="K68" s="47" t="s">
+        <v>333</v>
+      </c>
+      <c r="L68" s="19" t="s">
+        <v>334</v>
+      </c>
+      <c r="M68" s="48" t="s">
+        <v>335</v>
+      </c>
+      <c r="N68" s="19" t="s">
         <v>336</v>
-      </c>
-      <c r="L68" s="19" t="s">
-        <v>337</v>
-      </c>
-      <c r="M68" s="48" t="s">
-        <v>338</v>
-      </c>
-      <c r="N68" s="19" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="69" spans="4:14">
@@ -5322,16 +5301,16 @@
         <v>4</v>
       </c>
       <c r="K69" s="47" t="s">
+        <v>337</v>
+      </c>
+      <c r="L69" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="M69" s="48" t="s">
+        <v>339</v>
+      </c>
+      <c r="N69" s="19" t="s">
         <v>340</v>
-      </c>
-      <c r="L69" s="19" t="s">
-        <v>341</v>
-      </c>
-      <c r="M69" s="48" t="s">
-        <v>342</v>
-      </c>
-      <c r="N69" s="19" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="70" spans="4:14" ht="28.8">
@@ -5339,16 +5318,16 @@
         <v>5</v>
       </c>
       <c r="K70" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="L70" s="19" t="s">
+        <v>342</v>
+      </c>
+      <c r="M70" s="48" t="s">
+        <v>343</v>
+      </c>
+      <c r="N70" s="19" t="s">
         <v>344</v>
-      </c>
-      <c r="L70" s="19" t="s">
-        <v>345</v>
-      </c>
-      <c r="M70" s="48" t="s">
-        <v>346</v>
-      </c>
-      <c r="N70" s="19" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="71" spans="4:14" ht="28.8">
@@ -5356,16 +5335,16 @@
         <v>6</v>
       </c>
       <c r="K71" s="47" t="s">
+        <v>345</v>
+      </c>
+      <c r="L71" s="19" t="s">
+        <v>346</v>
+      </c>
+      <c r="M71" s="48" t="s">
+        <v>347</v>
+      </c>
+      <c r="N71" s="19" t="s">
         <v>348</v>
-      </c>
-      <c r="L71" s="19" t="s">
-        <v>349</v>
-      </c>
-      <c r="M71" s="48" t="s">
-        <v>350</v>
-      </c>
-      <c r="N71" s="19" t="s">
-        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -5854,7 +5833,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="8" spans="3:7" ht="60">
+    <row r="8" spans="3:7" ht="45">
       <c r="D8" s="28">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
deasing page of regional Analysis & Find some related KPIs & add report
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD1FE65-57DF-4554-8148-50800044C42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEE9589-55A8-4292-8F99-BEFE19FBE9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="377">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -1563,12 +1563,6 @@
     <t>Top State by Sales</t>
   </si>
   <si>
-    <t>TOPN(1, SUMMARIZE('Orders','Orders'[State],"StateSales",SUM('Orders'[Total Amount])),[StateSales],DESC)</t>
-  </si>
-  <si>
-    <t>Highlights the state contributing the most to sales</t>
-  </si>
-  <si>
     <t>Filled / Shape / Bubble Map</t>
   </si>
   <si>
@@ -2209,6 +2203,109 @@
   </si>
   <si>
     <t>Drill-down view for detailed analysis per promotion</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Identifies the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that generates the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>highest total sales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Top City by Sales</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Finds the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>City</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>maximum revenue contribution</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Top State by Sales = CALCULATE( SELECTEDVALUE('Amazon Sale Data'[State]), TOPN( 1, SUMMARIZE('Amazon Sale Data', 'Amazon Sale Data'[State], "Sales", SUM('Amazon Sale Data'[Total Amount]) ), [Sales], DESC ) )</t>
+  </si>
+  <si>
+    <t>Top City by Sales = CALCULATE( SELECTEDVALUE('Amazon Sale Data'[City]), TOPN( 1, SUMMARIZE('Amazon Sale Data', 'Amazon Sale Data'[City], "Sales", SUM('Amazon Sale Data'[Total Amount]) ), [Sales], DESC ) )</t>
   </si>
 </sst>
 </file>
@@ -4935,7 +5032,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="39" spans="2:14" ht="28.8">
+    <row r="39" spans="2:14" ht="52.8">
       <c r="D39" s="19">
         <v>1</v>
       </c>
@@ -4943,42 +5040,54 @@
         <v>295</v>
       </c>
       <c r="F39" s="48" t="s">
-        <v>296</v>
+        <v>375</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>297</v>
+        <v>372</v>
       </c>
       <c r="J39" s="19">
         <v>1</v>
       </c>
       <c r="K39" s="47" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="L39" s="19" t="s">
         <v>196</v>
       </c>
       <c r="M39" s="48" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="N39" s="19" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="40" spans="2:14">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" ht="52.8">
+      <c r="D40" s="19">
+        <v>2</v>
+      </c>
+      <c r="E40" s="47" t="s">
+        <v>373</v>
+      </c>
+      <c r="F40" s="48" t="s">
+        <v>376</v>
+      </c>
+      <c r="G40" s="19" t="s">
+        <v>374</v>
+      </c>
       <c r="J40" s="19">
         <v>2</v>
       </c>
       <c r="K40" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="L40" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="M40" s="48" t="s">
+        <v>297</v>
+      </c>
+      <c r="N40" s="19" t="s">
         <v>301</v>
-      </c>
-      <c r="L40" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="M40" s="48" t="s">
-        <v>299</v>
-      </c>
-      <c r="N40" s="19" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="41" spans="2:14" ht="28.8">
@@ -4986,16 +5095,16 @@
         <v>3</v>
       </c>
       <c r="K41" s="47" t="s">
+        <v>302</v>
+      </c>
+      <c r="L41" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="M41" s="48" t="s">
         <v>304</v>
       </c>
-      <c r="L41" s="19" t="s">
+      <c r="N41" s="19" t="s">
         <v>305</v>
-      </c>
-      <c r="M41" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="N41" s="19" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="42" spans="2:14" ht="28.8">
@@ -5003,16 +5112,16 @@
         <v>4</v>
       </c>
       <c r="K42" s="47" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="L42" s="19" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="M42" s="48" t="s">
         <v>61</v>
       </c>
       <c r="N42" s="19" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="43" spans="2:14" ht="28.8">
@@ -5020,16 +5129,16 @@
         <v>5</v>
       </c>
       <c r="K43" s="47" t="s">
+        <v>309</v>
+      </c>
+      <c r="L43" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="M43" s="48" t="s">
+        <v>297</v>
+      </c>
+      <c r="N43" s="19" t="s">
         <v>311</v>
-      </c>
-      <c r="L43" s="19" t="s">
-        <v>312</v>
-      </c>
-      <c r="M43" s="48" t="s">
-        <v>299</v>
-      </c>
-      <c r="N43" s="19" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="44" spans="2:14" ht="28.8">
@@ -5037,21 +5146,21 @@
         <v>6</v>
       </c>
       <c r="K44" s="47" t="s">
+        <v>312</v>
+      </c>
+      <c r="L44" s="19" t="s">
+        <v>313</v>
+      </c>
+      <c r="M44" s="48" t="s">
         <v>314</v>
       </c>
-      <c r="L44" s="19" t="s">
+      <c r="N44" s="19" t="s">
         <v>315</v>
-      </c>
-      <c r="M44" s="48" t="s">
-        <v>316</v>
-      </c>
-      <c r="N44" s="19" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="47" spans="2:14" ht="20.399999999999999">
       <c r="B47" s="13" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="49" spans="2:14">
@@ -5088,28 +5197,28 @@
         <v>1</v>
       </c>
       <c r="E50" s="47" t="s">
+        <v>347</v>
+      </c>
+      <c r="F50" s="48" t="s">
+        <v>348</v>
+      </c>
+      <c r="G50" s="19" t="s">
         <v>349</v>
-      </c>
-      <c r="F50" s="48" t="s">
-        <v>350</v>
-      </c>
-      <c r="G50" s="19" t="s">
-        <v>351</v>
       </c>
       <c r="J50" s="19">
         <v>1</v>
       </c>
       <c r="K50" s="47" t="s">
+        <v>356</v>
+      </c>
+      <c r="L50" s="19" t="s">
+        <v>357</v>
+      </c>
+      <c r="M50" s="48" t="s">
         <v>358</v>
       </c>
-      <c r="L50" s="19" t="s">
+      <c r="N50" s="19" t="s">
         <v>359</v>
-      </c>
-      <c r="M50" s="48" t="s">
-        <v>360</v>
-      </c>
-      <c r="N50" s="19" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="51" spans="2:14" ht="28.8">
@@ -5117,28 +5226,28 @@
         <v>2</v>
       </c>
       <c r="E51" s="47" t="s">
+        <v>350</v>
+      </c>
+      <c r="F51" s="48" t="s">
+        <v>351</v>
+      </c>
+      <c r="G51" s="19" t="s">
         <v>352</v>
-      </c>
-      <c r="F51" s="48" t="s">
-        <v>353</v>
-      </c>
-      <c r="G51" s="19" t="s">
-        <v>354</v>
       </c>
       <c r="J51" s="19">
         <v>2</v>
       </c>
       <c r="K51" s="47" t="s">
+        <v>360</v>
+      </c>
+      <c r="L51" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="M51" s="48" t="s">
         <v>362</v>
       </c>
-      <c r="L51" s="19" t="s">
+      <c r="N51" s="19" t="s">
         <v>363</v>
-      </c>
-      <c r="M51" s="48" t="s">
-        <v>364</v>
-      </c>
-      <c r="N51" s="19" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="52" spans="2:14" ht="28.8">
@@ -5146,28 +5255,28 @@
         <v>3</v>
       </c>
       <c r="E52" s="47" t="s">
+        <v>353</v>
+      </c>
+      <c r="F52" s="48" t="s">
+        <v>354</v>
+      </c>
+      <c r="G52" s="19" t="s">
         <v>355</v>
-      </c>
-      <c r="F52" s="48" t="s">
-        <v>356</v>
-      </c>
-      <c r="G52" s="19" t="s">
-        <v>357</v>
       </c>
       <c r="J52" s="19">
         <v>3</v>
       </c>
       <c r="K52" s="47" t="s">
+        <v>364</v>
+      </c>
+      <c r="L52" s="19" t="s">
+        <v>365</v>
+      </c>
+      <c r="M52" s="48" t="s">
         <v>366</v>
       </c>
-      <c r="L52" s="19" t="s">
+      <c r="N52" s="19" t="s">
         <v>367</v>
-      </c>
-      <c r="M52" s="48" t="s">
-        <v>368</v>
-      </c>
-      <c r="N52" s="19" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="53" spans="2:14">
@@ -5175,21 +5284,21 @@
         <v>4</v>
       </c>
       <c r="K53" s="47" t="s">
+        <v>368</v>
+      </c>
+      <c r="L53" s="19" t="s">
+        <v>369</v>
+      </c>
+      <c r="M53" s="48" t="s">
         <v>370</v>
       </c>
-      <c r="L53" s="19" t="s">
+      <c r="N53" s="19" t="s">
         <v>371</v>
-      </c>
-      <c r="M53" s="48" t="s">
-        <v>372</v>
-      </c>
-      <c r="N53" s="19" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="63" spans="2:14" ht="20.399999999999999">
       <c r="B63" s="13" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="65" spans="4:14">
@@ -5226,28 +5335,28 @@
         <v>1</v>
       </c>
       <c r="E66" s="47" t="s">
+        <v>318</v>
+      </c>
+      <c r="F66" s="48" t="s">
+        <v>319</v>
+      </c>
+      <c r="G66" s="19" t="s">
         <v>320</v>
-      </c>
-      <c r="F66" s="48" t="s">
-        <v>321</v>
-      </c>
-      <c r="G66" s="19" t="s">
-        <v>322</v>
       </c>
       <c r="J66" s="19">
         <v>1</v>
       </c>
       <c r="K66" s="47" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="L66" s="19" t="s">
         <v>204</v>
       </c>
       <c r="M66" s="48" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="N66" s="19" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="67" spans="4:14" ht="28.8">
@@ -5255,28 +5364,28 @@
         <v>2</v>
       </c>
       <c r="E67" s="47" t="s">
+        <v>321</v>
+      </c>
+      <c r="F67" s="48" t="s">
+        <v>322</v>
+      </c>
+      <c r="G67" s="19" t="s">
         <v>323</v>
-      </c>
-      <c r="F67" s="48" t="s">
-        <v>324</v>
-      </c>
-      <c r="G67" s="19" t="s">
-        <v>325</v>
       </c>
       <c r="J67" s="19">
         <v>2</v>
       </c>
       <c r="K67" s="47" t="s">
+        <v>327</v>
+      </c>
+      <c r="L67" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="M67" s="48" t="s">
         <v>329</v>
       </c>
-      <c r="L67" s="19" t="s">
+      <c r="N67" s="19" t="s">
         <v>330</v>
-      </c>
-      <c r="M67" s="48" t="s">
-        <v>331</v>
-      </c>
-      <c r="N67" s="19" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="68" spans="4:14" ht="28.8">
@@ -5284,16 +5393,16 @@
         <v>3</v>
       </c>
       <c r="K68" s="47" t="s">
+        <v>331</v>
+      </c>
+      <c r="L68" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="M68" s="48" t="s">
         <v>333</v>
       </c>
-      <c r="L68" s="19" t="s">
+      <c r="N68" s="19" t="s">
         <v>334</v>
-      </c>
-      <c r="M68" s="48" t="s">
-        <v>335</v>
-      </c>
-      <c r="N68" s="19" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="69" spans="4:14">
@@ -5301,16 +5410,16 @@
         <v>4</v>
       </c>
       <c r="K69" s="47" t="s">
+        <v>335</v>
+      </c>
+      <c r="L69" s="19" t="s">
+        <v>336</v>
+      </c>
+      <c r="M69" s="48" t="s">
         <v>337</v>
       </c>
-      <c r="L69" s="19" t="s">
+      <c r="N69" s="19" t="s">
         <v>338</v>
-      </c>
-      <c r="M69" s="48" t="s">
-        <v>339</v>
-      </c>
-      <c r="N69" s="19" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="70" spans="4:14" ht="28.8">
@@ -5318,16 +5427,16 @@
         <v>5</v>
       </c>
       <c r="K70" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="L70" s="19" t="s">
+        <v>340</v>
+      </c>
+      <c r="M70" s="48" t="s">
         <v>341</v>
       </c>
-      <c r="L70" s="19" t="s">
+      <c r="N70" s="19" t="s">
         <v>342</v>
-      </c>
-      <c r="M70" s="48" t="s">
-        <v>343</v>
-      </c>
-      <c r="N70" s="19" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="71" spans="4:14" ht="28.8">
@@ -5335,16 +5444,16 @@
         <v>6</v>
       </c>
       <c r="K71" s="47" t="s">
+        <v>343</v>
+      </c>
+      <c r="L71" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="M71" s="48" t="s">
         <v>345</v>
       </c>
-      <c r="L71" s="19" t="s">
+      <c r="N71" s="19" t="s">
         <v>346</v>
-      </c>
-      <c r="M71" s="48" t="s">
-        <v>347</v>
-      </c>
-      <c r="N71" s="19" t="s">
-        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
setup Forecasting Page, Add some Visuals & add in report, Aslo Complete Promotion Page
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEE9589-55A8-4292-8F99-BEFE19FBE9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB42C5C0-900A-47E5-84DB-43435B823F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="379">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -1743,312 +1743,6 @@
     <t>Forcasting</t>
   </si>
   <si>
-    <t>YoY Growth %</t>
-  </si>
-  <si>
-    <t>(SUM(CurrentYearSales)-SUM(PreviousYearSales))/SUM(PreviousYearSales)</t>
-  </si>
-  <si>
-    <t>Shows sales growth compared to same period last year</t>
-  </si>
-  <si>
-    <t>Cumulative Sales</t>
-  </si>
-  <si>
-    <t>CALCULATE(SUM('Orders'[Total Amount]), FILTER(ALLSELECTED('Orders'[Date]), 'Orders'[Date]&lt;=MAX('Orders'[Date])))</t>
-  </si>
-  <si>
-    <t>Shows running total of sales over time</t>
-  </si>
-  <si>
-    <t>Line Chart – Sales Trend Over Time</t>
-  </si>
-  <si>
-    <r>
-      <t>Date</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Month</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Total Amount</t>
-    </r>
-  </si>
-  <si>
-    <t>Shows revenue trend; detects peaks, dips, and seasonality</t>
-  </si>
-  <si>
-    <t>Area Chart – Qty Trend</t>
-  </si>
-  <si>
-    <t>“How units sold are changing over time?”</t>
-  </si>
-  <si>
-    <r>
-      <t>Date</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Qty</t>
-    </r>
-  </si>
-  <si>
-    <t>Visualizes demand trend and sales volume changes</t>
-  </si>
-  <si>
-    <t>Forecast Line (Power BI Analytics)</t>
-  </si>
-  <si>
-    <t>“Predict next 3–6 months sales”</t>
-  </si>
-  <si>
-    <r>
-      <t>Date</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Total Amount</t>
-    </r>
-  </si>
-  <si>
-    <t>Predicts future revenue using historical trend + confidence interval</t>
-  </si>
-  <si>
-    <t>Line Chart – Cumulative Sales</t>
-  </si>
-  <si>
-    <t>“How sales accumulate over time”</t>
-  </si>
-  <si>
-    <r>
-      <t>Date</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Cumulative Sales</t>
-    </r>
-  </si>
-  <si>
-    <t>Shows running total trend for period-wise progress</t>
-  </si>
-  <si>
-    <t>Combo Chart – Sales vs Quantity</t>
-  </si>
-  <si>
-    <t>“Is revenue growth due to volume or price?”</t>
-  </si>
-  <si>
-    <r>
-      <t>Date</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Total Amount</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Qty</t>
-    </r>
-  </si>
-  <si>
-    <t>Line for sales + Column for Qty to compare revenue vs units</t>
-  </si>
-  <si>
-    <t>Decomposition Tree</t>
-  </si>
-  <si>
-    <t>“What caused the increase/decrease?”</t>
-  </si>
-  <si>
-    <r>
-      <t>Total Amount</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Category</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>State</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Fulfilment</t>
-    </r>
-  </si>
-  <si>
-    <t>Drill into sales trend by different dimensions to find causes</t>
-  </si>
-  <si>
-    <t>Total Promotion Sales</t>
-  </si>
-  <si>
-    <t>CALCULATE(SUM('Orders'[Total Amount]), NOT(ISBLANK('Orders'[Promotion IDs])))</t>
-  </si>
-  <si>
-    <t>Shows total revenue generated from all promoted orders</t>
-  </si>
-  <si>
-    <t>Promotion Contribution (%)</t>
-  </si>
-  <si>
-    <t>DIVIDE(CALCULATE(SUM('Orders'[Total Amount]), NOT(ISBLANK('Orders'[Promotion IDs]))), SUM('Orders'[Total Amount]))</t>
-  </si>
-  <si>
-    <t>Shows percentage of total sales coming from promotions</t>
-  </si>
-  <si>
-    <t>Top Promotion Type by Sales</t>
-  </si>
-  <si>
-    <t>TOPN(1, SUMMARIZE('Orders','Orders'[Promotion Type],"PromoSales",SUM('Orders'[Total Amount])),[PromoSales],DESC)</t>
-  </si>
-  <si>
-    <t>Highlights the most effective promotion type</t>
-  </si>
-  <si>
     <t>Clustered Column Chart</t>
   </si>
   <si>
@@ -2306,13 +2000,363 @@
   </si>
   <si>
     <t>Top City by Sales = CALCULATE( SELECTEDVALUE('Amazon Sale Data'[City]), TOPN( 1, SUMMARIZE('Amazon Sale Data', 'Amazon Sale Data'[City], "Sales", SUM('Amazon Sale Data'[Total Amount]) ), [Sales], DESC ) )</t>
+  </si>
+  <si>
+    <t>DAX Formula (using ‘Amazon Sale Data’)</t>
+  </si>
+  <si>
+    <t>Avg Monthly Sales (₹)</t>
+  </si>
+  <si>
+    <t>Shows the average sales per month to understand seasonality trends.</t>
+  </si>
+  <si>
+    <t>DAX&lt;br&gt;Avg Monthly Sales (₹) =&lt;br&gt;AVERAGEX(&lt;br&gt; VALUES('Amazon Sale Data'[Month]),&lt;br&gt; CALCULATE(SUM('Amazon Sale Data'[Total Amount]))&lt;br&gt;)</t>
+  </si>
+  <si>
+    <t>Highest Sales Month</t>
+  </si>
+  <si>
+    <t>Identifies which month achieved the highest total sales. Useful for detecting peak sales periods.</t>
+  </si>
+  <si>
+    <t>DAX&lt;br&gt;Highest Sales Month =&lt;br&gt;VAR MonthSales =&lt;br&gt; SUMMARIZE(&lt;br&gt;  'Amazon Sale Data',&lt;br&gt;  'Amazon Sale Data'[Month],&lt;br&gt;  "TotalSales", SUM('Amazon Sale Data'[Total Amount])&lt;br&gt; )&lt;br&gt;RETURN&lt;br&gt;MAXX(&lt;br&gt; TOPN(1, MonthSales, [TotalSales], DESC),&lt;br&gt; 'Amazon Sale Data'[Month]&lt;br&gt;)</t>
+  </si>
+  <si>
+    <t>Visual Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Insight / Focus</t>
+  </si>
+  <si>
+    <t>Sales Trend Over Time</t>
+  </si>
+  <si>
+    <t>Line Chart</t>
+  </si>
+  <si>
+    <t>Track monthly or daily revenue growth and detect upward/downward trends.</t>
+  </si>
+  <si>
+    <t>Quantity Trend Over Time</t>
+  </si>
+  <si>
+    <t>Analyze how product quantity sold fluctuates over time.</t>
+  </si>
+  <si>
+    <t>Forecast Sales (Next 3 Months)</t>
+  </si>
+  <si>
+    <t>Line Chart (with Forecast)</t>
+  </si>
+  <si>
+    <t>Predict future sales values based on past performance.</t>
+  </si>
+  <si>
+    <t>Category-wise Monthly Trend</t>
+  </si>
+  <si>
+    <t>Area Chart</t>
+  </si>
+  <si>
+    <t>Identify seasonal demand patterns for different product categories.</t>
+  </si>
+  <si>
+    <t>Fulfilment Type Trend</t>
+  </si>
+  <si>
+    <t>Combo Chart (Line + Column)</t>
+  </si>
+  <si>
+    <t>Compare monthly performance between Amazon (FBA) and Merchant (FBM).</t>
+  </si>
+  <si>
+    <t>Promotion Impact Trend</t>
+  </si>
+  <si>
+    <t>Dual Line Chart</t>
+  </si>
+  <si>
+    <t>Compare revenue trends for “Promotion Applied” vs “No Promotion”.</t>
+  </si>
+  <si>
+    <t>Top Performing Months</t>
+  </si>
+  <si>
+    <t>Column Chart</t>
+  </si>
+  <si>
+    <t>Highlight months with highest total revenue.</t>
+  </si>
+  <si>
+    <t>Year-over-Year Growth %</t>
+  </si>
+  <si>
+    <t>Card / KPI Visual</t>
+  </si>
+  <si>
+    <t>Show overall sales growth percentage between years.</t>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Qty</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Fulfilment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Promotion Type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Year</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Total Amount</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2428,6 +2472,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -2518,7 +2567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2656,6 +2705,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4318,7 +4373,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FDCB3-6CAE-4927-8D50-CB20F0599746}">
-  <dimension ref="B3:S71"/>
+  <dimension ref="B3:S73"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
@@ -5040,10 +5095,10 @@
         <v>295</v>
       </c>
       <c r="F39" s="48" t="s">
-        <v>375</v>
+        <v>337</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>372</v>
+        <v>334</v>
       </c>
       <c r="J39" s="19">
         <v>1</v>
@@ -5066,13 +5121,13 @@
         <v>2</v>
       </c>
       <c r="E40" s="47" t="s">
-        <v>373</v>
+        <v>335</v>
       </c>
       <c r="F40" s="48" t="s">
-        <v>376</v>
+        <v>338</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>374</v>
+        <v>336</v>
       </c>
       <c r="J40" s="19">
         <v>2</v>
@@ -5162,20 +5217,15 @@
       <c r="B47" s="13" t="s">
         <v>316</v>
       </c>
+      <c r="I47" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="49" spans="2:14">
-      <c r="D49" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="45" t="s">
-        <v>162</v>
-      </c>
-      <c r="F49" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="G49" s="45" t="s">
-        <v>223</v>
-      </c>
+      <c r="D49" s="45"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="45"/>
+      <c r="G49" s="45"/>
       <c r="J49" s="45" t="s">
         <v>7</v>
       </c>
@@ -5192,91 +5242,67 @@
         <v>223</v>
       </c>
     </row>
-    <row r="50" spans="2:14" ht="28.8">
-      <c r="D50" s="19">
-        <v>1</v>
-      </c>
-      <c r="E50" s="47" t="s">
-        <v>347</v>
-      </c>
-      <c r="F50" s="48" t="s">
-        <v>348</v>
-      </c>
-      <c r="G50" s="19" t="s">
-        <v>349</v>
-      </c>
+    <row r="50" spans="2:14">
+      <c r="D50" s="19"/>
+      <c r="E50" s="47"/>
+      <c r="F50" s="48"/>
+      <c r="G50" s="19"/>
       <c r="J50" s="19">
         <v>1</v>
       </c>
       <c r="K50" s="47" t="s">
-        <v>356</v>
+        <v>318</v>
       </c>
       <c r="L50" s="19" t="s">
-        <v>357</v>
+        <v>319</v>
       </c>
       <c r="M50" s="48" t="s">
-        <v>358</v>
+        <v>320</v>
       </c>
       <c r="N50" s="19" t="s">
-        <v>359</v>
+        <v>321</v>
       </c>
     </row>
     <row r="51" spans="2:14" ht="28.8">
-      <c r="D51" s="19">
-        <v>2</v>
-      </c>
-      <c r="E51" s="47" t="s">
-        <v>350</v>
-      </c>
-      <c r="F51" s="48" t="s">
-        <v>351</v>
-      </c>
-      <c r="G51" s="19" t="s">
-        <v>352</v>
-      </c>
+      <c r="D51" s="19"/>
+      <c r="E51" s="47"/>
+      <c r="F51" s="48"/>
+      <c r="G51" s="19"/>
       <c r="J51" s="19">
         <v>2</v>
       </c>
       <c r="K51" s="47" t="s">
-        <v>360</v>
+        <v>322</v>
       </c>
       <c r="L51" s="19" t="s">
-        <v>361</v>
+        <v>323</v>
       </c>
       <c r="M51" s="48" t="s">
-        <v>362</v>
+        <v>324</v>
       </c>
       <c r="N51" s="19" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="52" spans="2:14" ht="28.8">
-      <c r="D52" s="19">
-        <v>3</v>
-      </c>
-      <c r="E52" s="47" t="s">
-        <v>353</v>
-      </c>
-      <c r="F52" s="48" t="s">
-        <v>354</v>
-      </c>
-      <c r="G52" s="19" t="s">
-        <v>355</v>
-      </c>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14">
+      <c r="D52" s="19"/>
+      <c r="E52" s="47"/>
+      <c r="F52" s="48"/>
+      <c r="G52" s="19"/>
       <c r="J52" s="19">
         <v>3</v>
       </c>
       <c r="K52" s="47" t="s">
-        <v>364</v>
+        <v>326</v>
       </c>
       <c r="L52" s="19" t="s">
-        <v>365</v>
+        <v>327</v>
       </c>
       <c r="M52" s="48" t="s">
-        <v>366</v>
+        <v>328</v>
       </c>
       <c r="N52" s="19" t="s">
-        <v>367</v>
+        <v>329</v>
       </c>
     </row>
     <row r="53" spans="2:14">
@@ -5284,176 +5310,216 @@
         <v>4</v>
       </c>
       <c r="K53" s="47" t="s">
-        <v>368</v>
+        <v>330</v>
       </c>
       <c r="L53" s="19" t="s">
-        <v>369</v>
+        <v>331</v>
       </c>
       <c r="M53" s="48" t="s">
-        <v>370</v>
+        <v>332</v>
       </c>
       <c r="N53" s="19" t="s">
-        <v>371</v>
+        <v>333</v>
       </c>
     </row>
     <row r="63" spans="2:14" ht="20.399999999999999">
       <c r="B63" s="13" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="65" spans="4:14">
-      <c r="D65" s="45" t="s">
+      <c r="D63" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I63" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="65" spans="4:14" ht="15.6">
+      <c r="D65" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="E65" s="45" t="s">
+      <c r="E65" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="F65" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="G65" s="45" t="s">
-        <v>223</v>
-      </c>
-      <c r="J65" s="45" t="s">
+      <c r="F65" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="G65" s="49" t="s">
+        <v>339</v>
+      </c>
+      <c r="J65" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K65" s="45" t="s">
-        <v>25</v>
-      </c>
-      <c r="L65" s="45" t="s">
-        <v>271</v>
-      </c>
-      <c r="M65" s="45" t="s">
+      <c r="K65" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="L65" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="M65" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="N65" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N65" s="45" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="66" spans="4:14" ht="28.8">
-      <c r="D66" s="19">
+    </row>
+    <row r="66" spans="4:14" ht="45.6">
+      <c r="D66" s="22">
         <v>1</v>
       </c>
-      <c r="E66" s="47" t="s">
-        <v>318</v>
-      </c>
-      <c r="F66" s="48" t="s">
-        <v>319</v>
-      </c>
-      <c r="G66" s="19" t="s">
-        <v>320</v>
-      </c>
-      <c r="J66" s="19">
+      <c r="E66" s="24" t="s">
+        <v>340</v>
+      </c>
+      <c r="F66" s="23" t="s">
+        <v>341</v>
+      </c>
+      <c r="G66" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="J66" s="22">
         <v>1</v>
       </c>
-      <c r="K66" s="47" t="s">
-        <v>324</v>
-      </c>
-      <c r="L66" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="M66" s="48" t="s">
-        <v>325</v>
-      </c>
-      <c r="N66" s="19" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="67" spans="4:14" ht="28.8">
-      <c r="D67" s="19">
+      <c r="K66" s="26" t="s">
+        <v>349</v>
+      </c>
+      <c r="L66" s="26" t="s">
+        <v>350</v>
+      </c>
+      <c r="M66" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="N66" s="35" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="67" spans="4:14" ht="91.2">
+      <c r="D67" s="22">
         <v>2</v>
       </c>
-      <c r="E67" s="47" t="s">
-        <v>321</v>
-      </c>
-      <c r="F67" s="48" t="s">
-        <v>322</v>
-      </c>
-      <c r="G67" s="19" t="s">
-        <v>323</v>
-      </c>
-      <c r="J67" s="19">
+      <c r="E67" s="24" t="s">
+        <v>343</v>
+      </c>
+      <c r="F67" s="23" t="s">
+        <v>344</v>
+      </c>
+      <c r="G67" s="53" t="s">
+        <v>345</v>
+      </c>
+      <c r="J67" s="22">
         <v>2</v>
       </c>
-      <c r="K67" s="47" t="s">
-        <v>327</v>
-      </c>
-      <c r="L67" s="19" t="s">
-        <v>328</v>
-      </c>
-      <c r="M67" s="48" t="s">
-        <v>329</v>
-      </c>
-      <c r="N67" s="19" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="68" spans="4:14" ht="28.8">
-      <c r="J68" s="19">
+      <c r="K67" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="L67" s="26" t="s">
+        <v>350</v>
+      </c>
+      <c r="M67" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="N67" s="35" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="68" spans="4:14" ht="31.2">
+      <c r="J68" s="22">
         <v>3</v>
       </c>
-      <c r="K68" s="47" t="s">
-        <v>331</v>
-      </c>
-      <c r="L68" s="19" t="s">
-        <v>332</v>
-      </c>
-      <c r="M68" s="48" t="s">
-        <v>333</v>
-      </c>
-      <c r="N68" s="19" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="69" spans="4:14">
-      <c r="J69" s="19">
+      <c r="K68" s="54" t="s">
+        <v>354</v>
+      </c>
+      <c r="L68" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="M68" s="27" t="s">
+        <v>356</v>
+      </c>
+      <c r="N68" s="35" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="69" spans="4:14" ht="31.2">
+      <c r="J69" s="22">
         <v>4</v>
       </c>
-      <c r="K69" s="47" t="s">
-        <v>335</v>
-      </c>
-      <c r="L69" s="19" t="s">
-        <v>336</v>
-      </c>
-      <c r="M69" s="48" t="s">
-        <v>337</v>
-      </c>
-      <c r="N69" s="19" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="70" spans="4:14" ht="28.8">
-      <c r="J70" s="19">
+      <c r="K69" s="26" t="s">
+        <v>357</v>
+      </c>
+      <c r="L69" s="26" t="s">
+        <v>358</v>
+      </c>
+      <c r="M69" s="27" t="s">
+        <v>359</v>
+      </c>
+      <c r="N69" s="35" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="70" spans="4:14" ht="31.2">
+      <c r="J70" s="22">
         <v>5</v>
       </c>
-      <c r="K70" s="47" t="s">
-        <v>339</v>
-      </c>
-      <c r="L70" s="19" t="s">
-        <v>340</v>
-      </c>
-      <c r="M70" s="48" t="s">
-        <v>341</v>
-      </c>
-      <c r="N70" s="19" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="71" spans="4:14" ht="28.8">
-      <c r="J71" s="19">
+      <c r="K70" s="26" t="s">
+        <v>360</v>
+      </c>
+      <c r="L70" s="26" t="s">
+        <v>361</v>
+      </c>
+      <c r="M70" s="27" t="s">
+        <v>362</v>
+      </c>
+      <c r="N70" s="35" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="71" spans="4:14" ht="31.2">
+      <c r="J71" s="22">
         <v>6</v>
       </c>
-      <c r="K71" s="47" t="s">
-        <v>343</v>
-      </c>
-      <c r="L71" s="19" t="s">
-        <v>344</v>
-      </c>
-      <c r="M71" s="48" t="s">
-        <v>345</v>
-      </c>
-      <c r="N71" s="19" t="s">
-        <v>346</v>
+      <c r="K71" s="26" t="s">
+        <v>363</v>
+      </c>
+      <c r="L71" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="M71" s="27" t="s">
+        <v>365</v>
+      </c>
+      <c r="N71" s="35" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="72" spans="4:14" ht="31.2">
+      <c r="J72" s="22">
+        <v>7</v>
+      </c>
+      <c r="K72" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="L72" s="26" t="s">
+        <v>367</v>
+      </c>
+      <c r="M72" s="27" t="s">
+        <v>368</v>
+      </c>
+      <c r="N72" s="35" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="73" spans="4:14" ht="31.2">
+      <c r="J73" s="22">
+        <v>8</v>
+      </c>
+      <c r="K73" s="26" t="s">
+        <v>369</v>
+      </c>
+      <c r="L73" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="M73" s="27" t="s">
+        <v>371</v>
+      </c>
+      <c r="N73" s="35" t="s">
+        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Screen shot & other things
</commit_message>
<xml_diff>
--- a/Report/Amazon Sales Report.xlsx
+++ b/Report/Amazon Sales Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prafull Wahatule\Desktop\BI Amazon Sale Report\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C9D5B0-3414-4A71-A85C-B33C1199C3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA935F0-53AA-4B19-B17B-63D84E3DD870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{1DE24626-BF60-4871-8242-B0FFC979D36A}"/>
   </bookViews>
   <sheets>
     <sheet name="KYV - Column" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="288">
   <si>
     <t>Know Your Value/Column</t>
   </si>
@@ -1212,6 +1212,169 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Shows which product categories generate the highest revenue. Helps identify top-performing and low-performing categories.</t>
+  </si>
+  <si>
+    <t>Compares contribution of Amazon (FBA) vs Merchant (FBM) fulfilment to total sales. Useful for understanding operational dependency.</t>
+  </si>
+  <si>
+    <t>Displays total sales distribution across states. Helps identify high-performing regions and potential markets for growth.</t>
+  </si>
+  <si>
+    <t>Compares sales generated from promotional vs non-promotional orders. Evaluates the impact of marketing offers on sales.</t>
+  </si>
+  <si>
+    <t>Tracks monthly revenue pattern to identify seasonality, growth, or decline trends in sales over time.</t>
+  </si>
+  <si>
+    <t>Shows the percentage contribution of Amazon-fulfilled (FBA) orders in total sales, useful for evaluating dependency on Amazon.</t>
+  </si>
+  <si>
+    <t>Shows the percentage contribution of Merchant-fulfilled (FBM) orders in total sales, highlighting seller-driven fulfilment performance.</t>
+  </si>
+  <si>
+    <t>Displays total revenue generated from Amazon-fulfilled (FBA) orders. Indicates Amazon’s direct sales impact.</t>
+  </si>
+  <si>
+    <t>Displays total revenue generated from Merchant-fulfilled (FBM) orders. Useful for tracking independent seller performance.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Shows the percentage of total sales that came </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>without any promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Helps understand how much revenue was generated organically.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Displays the percentage of total sales made </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>under promotional offers or discounts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Useful to analyze the effectiveness of promotions on sales growth.</t>
+    </r>
+  </si>
+  <si>
+    <t>Identifies the best revenue-generating SKUs. Helps focus on top-performing products to improve revenue strategy.</t>
+  </si>
+  <si>
+    <t>Shows which products are selling the most units. Useful for inventory and customer preference analysis.</t>
+  </si>
+  <si>
+    <t>Reveals which size variants contribute more sales. Helps optimize production, stock levels, and supply chain planning.</t>
+  </si>
+  <si>
+    <t>Tracks monthly demand trends across categories. Useful to identify seasonality and demand spikes.</t>
+  </si>
+  <si>
+    <t>Measures category-wise revenue contribution. Helps understand which product categories drive overall business performance.</t>
+  </si>
+  <si>
+    <t>Shows the distribution of total quantity fulfilled by Amazon (FBA) and Merchant (FBM). Helps compare fulfilment efficiency.</t>
+  </si>
+  <si>
+    <t>Compares the average delivery value between fulfilment types to identify which model brings higher order value.</t>
+  </si>
+  <si>
+    <t>Tracks delivery success rate over time. Helps monitor performance trends and identify seasonal delivery issues.</t>
+  </si>
+  <si>
+    <t>Highlights how much quantity each fulfilment type handles across cities. Useful for operational and logistics planning.</t>
+  </si>
+  <si>
+    <t>Shows percentage of total sales handled via Amazon FBA. Useful to measure Amazon’s operational dominance.</t>
+  </si>
+  <si>
+    <t>Displays the sales percentage handled via Merchant (FBM). Helps evaluate merchant-driven performance.</t>
+  </si>
+  <si>
+    <t>Visualizes total quantity sold across India using a map — helps identify high-performing regions geographically.</t>
+  </si>
+  <si>
+    <t>Highlights the top 5 states generating the highest total sales — useful for regional performance tracking.</t>
+  </si>
+  <si>
+    <t>Displays the top 5 cities contributing most to overall sales — helps identify key urban markets.</t>
+  </si>
+  <si>
+    <t>Shows the bottom 5 states by total sales — helps spot low-performing regions for targeted improvement.</t>
+  </si>
+  <si>
+    <t>Provides a detailed regional summary showing sales, quantity, and fulfilment split for each state and city.</t>
+  </si>
+  <si>
+    <t>Shows how total quantity is distributed between “Promotion Applied” and “No Promotion” — helps understand offer participation.</t>
+  </si>
+  <si>
+    <t>Compares monthly sales between promotion types — highlights how promotions impact monthly revenue trends.</t>
+  </si>
+  <si>
+    <t>Displays sales and quantity variation across product sizes — helps analyze which sizes perform better during promotions.</t>
+  </si>
+  <si>
+    <t>Highlights the top 5 promotion IDs that drove the highest quantity of orders — useful for evaluating most effective campaigns.</t>
+  </si>
+  <si>
+    <t>Compares total sales generated under each promotion type — shows contribution of promotional vs non-promotional orders.</t>
+  </si>
+  <si>
+    <t>Tracks order movement by status group — helps identify fulfillment and cancellation trends over time.</t>
+  </si>
+  <si>
+    <t>Shows how total ordered quantity changes month by month — useful for spotting seasonality or demand surges.</t>
+  </si>
+  <si>
+    <t>Displays overall monthly sales growth — helps in understanding business performance trends.</t>
+  </si>
+  <si>
+    <t>Highlights how different product categories perform each month — reveals seasonal demand patterns.</t>
+  </si>
+  <si>
+    <t>Compares monthly sales between Amazon (FBA) and Merchant (FBM) — helps analyze fulfillment efficiency over time.</t>
+  </si>
+  <si>
+    <t>Shows revenue contribution from B2B vs B2C orders — useful for tracking business-type growth trends.</t>
+  </si>
+  <si>
+    <t>Displays distribution of total sales by different shipping types each month — helps evaluate delivery mode preferences and performance.</t>
   </si>
 </sst>
 </file>
@@ -1547,7 +1710,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1630,22 +1793,22 @@
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1660,20 +1823,19 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1686,51 +1848,32 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -3517,7 +3660,7 @@
       <c r="B17" s="17">
         <v>12</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="C17" s="51" t="s">
         <v>136</v>
       </c>
       <c r="D17" s="17" t="s">
@@ -3570,16 +3713,16 @@
     <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" customWidth="1"/>
-    <col min="6" max="6" width="94.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="144.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="43.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="130.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="42.44140625" customWidth="1"/>
+    <col min="12" max="12" width="43.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="132" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.109375" customWidth="1"/>
-    <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="31.21875" customWidth="1"/>
     <col min="17" max="17" width="40.5546875" customWidth="1"/>
     <col min="18" max="18" width="25.88671875" customWidth="1"/>
@@ -3588,97 +3731,91 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15" thickBot="1"/>
     <row r="2" spans="1:19">
-      <c r="A2" s="69"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="71"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="63"/>
     </row>
     <row r="3" spans="1:19" ht="23.4">
-      <c r="A3" s="72"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
+      <c r="A3" s="64"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
       <c r="F3" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="57"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="73"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="65"/>
       <c r="S3" s="11"/>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="72"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="73"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="65"/>
       <c r="S4" s="11"/>
     </row>
     <row r="5" spans="1:19" ht="21">
-      <c r="A5" s="72"/>
+      <c r="A5" s="64"/>
       <c r="B5" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="44"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
       <c r="H5" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
-      <c r="P5" s="57"/>
-      <c r="Q5" s="57"/>
-      <c r="R5" s="73"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="65"/>
       <c r="S5" s="11"/>
     </row>
     <row r="6" spans="1:19" ht="15.6">
-      <c r="A6" s="72"/>
-      <c r="B6" s="44"/>
+      <c r="A6" s="64"/>
       <c r="C6" s="15" t="s">
         <v>7</v>
       </c>
@@ -3691,8 +3828,7 @@
       <c r="F6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="44"/>
-      <c r="H6" s="57"/>
+      <c r="H6" s="11"/>
       <c r="I6" s="39" t="s">
         <v>7</v>
       </c>
@@ -3702,18 +3838,15 @@
       <c r="K6" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="44"/>
-      <c r="M6" s="44"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="73"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
+      <c r="R6" s="65"/>
       <c r="S6" s="11"/>
     </row>
     <row r="7" spans="1:19" ht="31.2">
-      <c r="A7" s="72"/>
-      <c r="B7" s="44"/>
+      <c r="A7" s="64"/>
       <c r="C7" s="28">
         <v>1</v>
       </c>
@@ -3726,8 +3859,7 @@
       <c r="F7" s="41" t="s">
         <v>183</v>
       </c>
-      <c r="G7" s="44"/>
-      <c r="H7" s="57"/>
+      <c r="H7" s="11"/>
       <c r="I7" s="19">
         <v>1</v>
       </c>
@@ -3737,18 +3869,15 @@
       <c r="K7" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="73"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="65"/>
       <c r="S7" s="11"/>
     </row>
     <row r="8" spans="1:19" ht="31.2">
-      <c r="A8" s="72"/>
-      <c r="B8" s="44"/>
+      <c r="A8" s="64"/>
       <c r="C8" s="28">
         <v>2</v>
       </c>
@@ -3761,8 +3890,7 @@
       <c r="F8" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="G8" s="44"/>
-      <c r="H8" s="57"/>
+      <c r="H8" s="11"/>
       <c r="I8" s="19">
         <v>2</v>
       </c>
@@ -3772,18 +3900,15 @@
       <c r="K8" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="L8" s="44"/>
-      <c r="M8" s="44"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="73"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="65"/>
       <c r="S8" s="11"/>
     </row>
     <row r="9" spans="1:19" ht="31.2">
-      <c r="A9" s="72"/>
-      <c r="B9" s="44"/>
+      <c r="A9" s="64"/>
       <c r="C9" s="28">
         <v>3</v>
       </c>
@@ -3796,8 +3921,7 @@
       <c r="F9" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="G9" s="44"/>
-      <c r="H9" s="57"/>
+      <c r="H9" s="11"/>
       <c r="I9" s="19">
         <v>3</v>
       </c>
@@ -3807,18 +3931,15 @@
       <c r="K9" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="57"/>
-      <c r="P9" s="57"/>
-      <c r="Q9" s="57"/>
-      <c r="R9" s="73"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="65"/>
       <c r="S9" s="11"/>
     </row>
     <row r="10" spans="1:19" ht="46.8">
-      <c r="A10" s="72"/>
-      <c r="B10" s="44"/>
+      <c r="A10" s="64"/>
       <c r="C10" s="28">
         <v>4</v>
       </c>
@@ -3831,8 +3952,7 @@
       <c r="F10" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="G10" s="44"/>
-      <c r="H10" s="57"/>
+      <c r="H10" s="11"/>
       <c r="I10" s="19">
         <v>4</v>
       </c>
@@ -3842,24 +3962,18 @@
       <c r="K10" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="73"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="65"/>
       <c r="S10" s="11"/>
     </row>
     <row r="11" spans="1:19" ht="15.6">
-      <c r="A11" s="72"/>
-      <c r="B11" s="57"/>
-      <c r="C11" s="57"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="57"/>
+      <c r="A11" s="64"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="H11" s="11"/>
       <c r="I11" s="19">
         <v>5</v>
       </c>
@@ -3869,24 +3983,18 @@
       <c r="K11" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="L11" s="44"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="57"/>
-      <c r="O11" s="57"/>
-      <c r="P11" s="57"/>
-      <c r="Q11" s="57"/>
-      <c r="R11" s="73"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="65"/>
       <c r="S11" s="11"/>
     </row>
     <row r="12" spans="1:19" ht="15.6">
-      <c r="A12" s="72"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="57"/>
+      <c r="A12" s="64"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="H12" s="11"/>
       <c r="I12" s="19">
         <v>6</v>
       </c>
@@ -3896,24 +4004,18 @@
       <c r="K12" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="57"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="57"/>
-      <c r="Q12" s="57"/>
-      <c r="R12" s="73"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="65"/>
       <c r="S12" s="11"/>
     </row>
     <row r="13" spans="1:19" ht="15.6">
-      <c r="A13" s="72"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="57"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="57"/>
+      <c r="A13" s="64"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="H13" s="11"/>
       <c r="I13" s="19">
         <v>7</v>
       </c>
@@ -3923,147 +4025,93 @@
       <c r="K13" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="L13" s="44"/>
-      <c r="M13" s="44"/>
-      <c r="N13" s="57"/>
-      <c r="O13" s="57"/>
-      <c r="P13" s="57"/>
-      <c r="Q13" s="57"/>
-      <c r="R13" s="73"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="65"/>
       <c r="S13" s="11"/>
     </row>
     <row r="14" spans="1:19" ht="15.6">
-      <c r="A14" s="72"/>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="57"/>
+      <c r="A14" s="64"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="H14" s="11"/>
       <c r="I14" s="32"/>
       <c r="J14" s="33"/>
       <c r="K14" s="34"/>
-      <c r="L14" s="44"/>
-      <c r="M14" s="44"/>
-      <c r="N14" s="57"/>
-      <c r="O14" s="57"/>
-      <c r="P14" s="57"/>
-      <c r="Q14" s="57"/>
-      <c r="R14" s="73"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="65"/>
       <c r="S14" s="11"/>
     </row>
     <row r="15" spans="1:19" ht="15.6">
-      <c r="A15" s="72"/>
-      <c r="B15" s="57"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
+      <c r="A15" s="64"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
       <c r="K15" s="32"/>
       <c r="L15" s="33"/>
       <c r="M15" s="34"/>
-      <c r="N15" s="57"/>
-      <c r="O15" s="57"/>
-      <c r="P15" s="57"/>
-      <c r="Q15" s="57"/>
-      <c r="R15" s="73"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="65"/>
       <c r="S15" s="11"/>
     </row>
     <row r="16" spans="1:19" ht="15.6">
-      <c r="A16" s="74"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="58"/>
-      <c r="J16" s="58"/>
+      <c r="A16" s="66"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="52"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="52"/>
       <c r="K16" s="35"/>
       <c r="L16" s="36"/>
       <c r="M16" s="37"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="58"/>
-      <c r="P16" s="58"/>
-      <c r="Q16" s="58"/>
-      <c r="R16" s="83"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="52"/>
+      <c r="P16" s="52"/>
+      <c r="Q16" s="52"/>
+      <c r="R16" s="75"/>
       <c r="S16" s="11"/>
     </row>
     <row r="17" spans="1:19">
-      <c r="A17" s="72"/>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="44"/>
-      <c r="J17" s="44"/>
-      <c r="K17" s="44"/>
-      <c r="L17" s="44"/>
-      <c r="M17" s="44"/>
-      <c r="N17" s="44"/>
-      <c r="O17" s="44"/>
-      <c r="P17" s="44"/>
-      <c r="Q17" s="44"/>
-      <c r="R17" s="75"/>
+      <c r="A17" s="64"/>
+      <c r="R17" s="67"/>
     </row>
     <row r="18" spans="1:19" ht="20.399999999999999">
-      <c r="A18" s="72"/>
+      <c r="A18" s="64"/>
       <c r="B18" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="C18" s="59"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="44"/>
-      <c r="L18" s="44"/>
-      <c r="M18" s="44"/>
-      <c r="N18" s="57"/>
-      <c r="O18" s="57"/>
-      <c r="P18" s="44"/>
-      <c r="Q18" s="57"/>
-      <c r="R18" s="73"/>
+      <c r="C18" s="53"/>
+      <c r="J18" s="11"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="65"/>
       <c r="S18" s="11"/>
     </row>
     <row r="19" spans="1:19" ht="21">
-      <c r="A19" s="72"/>
-      <c r="B19" s="44"/>
+      <c r="A19" s="64"/>
       <c r="C19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44"/>
-      <c r="K19" s="44"/>
-      <c r="L19" s="44"/>
-      <c r="M19" s="44"/>
-      <c r="N19" s="44"/>
-      <c r="O19" s="44"/>
-      <c r="P19" s="44"/>
-      <c r="Q19" s="44"/>
-      <c r="R19" s="75"/>
+      <c r="R19" s="67"/>
     </row>
     <row r="20" spans="1:19" ht="15.6">
-      <c r="A20" s="72"/>
-      <c r="B20" s="57"/>
-      <c r="C20" s="44"/>
+      <c r="A20" s="64"/>
+      <c r="B20" s="11"/>
       <c r="D20" s="3" t="s">
         <v>7</v>
       </c>
@@ -4079,21 +4127,12 @@
       <c r="H20" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="44"/>
-      <c r="N20" s="44"/>
-      <c r="O20" s="57"/>
-      <c r="P20" s="57"/>
-      <c r="Q20" s="44"/>
-      <c r="R20" s="75"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="R20" s="67"/>
     </row>
     <row r="21" spans="1:19" ht="15.6">
-      <c r="A21" s="72"/>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
+      <c r="A21" s="64"/>
       <c r="D21" s="28">
         <v>1</v>
       </c>
@@ -4106,22 +4145,13 @@
       <c r="G21" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="H21" s="24"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="44"/>
-      <c r="L21" s="44"/>
-      <c r="M21" s="44"/>
-      <c r="N21" s="44"/>
-      <c r="O21" s="44"/>
-      <c r="P21" s="44"/>
-      <c r="Q21" s="44"/>
-      <c r="R21" s="75"/>
+      <c r="H21" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="R21" s="67"/>
     </row>
     <row r="22" spans="1:19" ht="15.6">
-      <c r="A22" s="72"/>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
+      <c r="A22" s="64"/>
       <c r="D22" s="28">
         <v>2</v>
       </c>
@@ -4134,22 +4164,13 @@
       <c r="G22" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="H22" s="24"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44"/>
-      <c r="K22" s="44"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="44"/>
-      <c r="N22" s="44"/>
-      <c r="O22" s="44"/>
-      <c r="P22" s="44"/>
-      <c r="Q22" s="44"/>
-      <c r="R22" s="75"/>
+      <c r="H22" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="R22" s="67"/>
     </row>
     <row r="23" spans="1:19" ht="15.6">
-      <c r="A23" s="72"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
+      <c r="A23" s="64"/>
       <c r="D23" s="28">
         <v>3</v>
       </c>
@@ -4162,22 +4183,13 @@
       <c r="G23" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="H23" s="24"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44"/>
-      <c r="K23" s="44"/>
-      <c r="L23" s="44"/>
-      <c r="M23" s="44"/>
-      <c r="N23" s="44"/>
-      <c r="O23" s="44"/>
-      <c r="P23" s="44"/>
-      <c r="Q23" s="44"/>
-      <c r="R23" s="75"/>
+      <c r="H23" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="R23" s="67"/>
     </row>
     <row r="24" spans="1:19" ht="15.6">
-      <c r="A24" s="72"/>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
+      <c r="A24" s="64"/>
       <c r="D24" s="28">
         <v>4</v>
       </c>
@@ -4190,22 +4202,13 @@
       <c r="G24" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="H24" s="24"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="44"/>
-      <c r="L24" s="44"/>
-      <c r="M24" s="44"/>
-      <c r="N24" s="44"/>
-      <c r="O24" s="44"/>
-      <c r="P24" s="44"/>
-      <c r="Q24" s="44"/>
-      <c r="R24" s="75"/>
+      <c r="H24" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="R24" s="67"/>
     </row>
     <row r="25" spans="1:19" ht="15.6">
-      <c r="A25" s="72"/>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
+      <c r="A25" s="64"/>
       <c r="D25" s="28">
         <v>5</v>
       </c>
@@ -4218,128 +4221,58 @@
       <c r="G25" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="H25" s="24"/>
-      <c r="I25" s="44"/>
-      <c r="J25" s="44"/>
-      <c r="K25" s="44"/>
-      <c r="L25" s="44"/>
-      <c r="M25" s="44"/>
-      <c r="N25" s="44"/>
-      <c r="O25" s="44"/>
-      <c r="P25" s="44"/>
-      <c r="Q25" s="44"/>
-      <c r="R25" s="75"/>
+      <c r="H25" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="R25" s="67"/>
     </row>
     <row r="26" spans="1:19">
-      <c r="A26" s="72"/>
-      <c r="B26" s="44"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
-      <c r="P26" s="44"/>
-      <c r="Q26" s="44"/>
-      <c r="R26" s="75"/>
+      <c r="A26" s="64"/>
+      <c r="R26" s="67"/>
     </row>
     <row r="27" spans="1:19">
-      <c r="A27" s="74"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="47"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="47"/>
-      <c r="P27" s="47"/>
-      <c r="Q27" s="47"/>
-      <c r="R27" s="79"/>
+      <c r="A27" s="66"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="46"/>
+      <c r="Q27" s="46"/>
+      <c r="R27" s="71"/>
     </row>
     <row r="28" spans="1:19">
-      <c r="A28" s="72"/>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="44"/>
-      <c r="I28" s="44"/>
-      <c r="J28" s="44"/>
-      <c r="K28" s="44"/>
-      <c r="L28" s="44"/>
-      <c r="M28" s="44"/>
-      <c r="N28" s="44"/>
-      <c r="O28" s="44"/>
-      <c r="P28" s="44"/>
-      <c r="Q28" s="44"/>
-      <c r="R28" s="75"/>
+      <c r="A28" s="64"/>
+      <c r="R28" s="67"/>
     </row>
     <row r="29" spans="1:19" ht="20.399999999999999">
-      <c r="A29" s="72"/>
+      <c r="A29" s="64"/>
       <c r="B29" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44"/>
-      <c r="K29" s="44"/>
-      <c r="L29" s="44"/>
-      <c r="M29" s="44"/>
-      <c r="N29" s="44"/>
-      <c r="O29" s="44"/>
-      <c r="P29" s="44"/>
-      <c r="Q29" s="44"/>
-      <c r="R29" s="75"/>
+      <c r="R29" s="67"/>
     </row>
     <row r="30" spans="1:19" ht="20.399999999999999">
-      <c r="A30" s="72"/>
-      <c r="B30" s="44"/>
+      <c r="A30" s="64"/>
       <c r="C30" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
       <c r="H30" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44"/>
-      <c r="K30" s="44"/>
-      <c r="L30" s="44"/>
-      <c r="M30" s="44"/>
-      <c r="N30" s="44"/>
-      <c r="O30" s="44"/>
-      <c r="P30" s="44"/>
-      <c r="Q30" s="44"/>
-      <c r="R30" s="75"/>
+      <c r="R30" s="67"/>
     </row>
     <row r="31" spans="1:19" ht="15.6">
-      <c r="A31" s="72"/>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
+      <c r="A31" s="64"/>
       <c r="D31" s="29" t="s">
         <v>7</v>
       </c>
@@ -4349,8 +4282,6 @@
       <c r="F31" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="G31" s="44"/>
-      <c r="H31" s="44"/>
       <c r="I31" s="3" t="s">
         <v>7</v>
       </c>
@@ -4366,16 +4297,10 @@
       <c r="M31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="N31" s="44"/>
-      <c r="O31" s="44"/>
-      <c r="P31" s="44"/>
-      <c r="Q31" s="44"/>
-      <c r="R31" s="75"/>
+      <c r="R31" s="67"/>
     </row>
     <row r="32" spans="1:19" ht="15.6">
-      <c r="A32" s="72"/>
-      <c r="B32" s="44"/>
-      <c r="C32" s="44"/>
+      <c r="A32" s="64"/>
       <c r="D32" s="19">
         <v>1</v>
       </c>
@@ -4385,29 +4310,25 @@
       <c r="F32" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
       <c r="I32" s="20">
         <v>1</v>
       </c>
       <c r="J32" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="K32" s="25"/>
+      <c r="K32" s="25" t="s">
+        <v>179</v>
+      </c>
       <c r="L32" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="M32" s="20"/>
-      <c r="N32" s="44"/>
-      <c r="O32" s="44"/>
-      <c r="P32" s="44"/>
-      <c r="Q32" s="44"/>
-      <c r="R32" s="75"/>
+      <c r="M32" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="R32" s="67"/>
     </row>
     <row r="33" spans="1:18" ht="15.6">
-      <c r="A33" s="72"/>
-      <c r="B33" s="44"/>
-      <c r="C33" s="44"/>
+      <c r="A33" s="64"/>
       <c r="D33" s="19">
         <v>2</v>
       </c>
@@ -4417,29 +4338,25 @@
       <c r="F33" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
       <c r="I33" s="20">
         <v>2</v>
       </c>
       <c r="J33" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="K33" s="25"/>
+      <c r="K33" s="25" t="s">
+        <v>179</v>
+      </c>
       <c r="L33" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="M33" s="20"/>
-      <c r="N33" s="44"/>
-      <c r="O33" s="44"/>
-      <c r="P33" s="44"/>
-      <c r="Q33" s="44"/>
-      <c r="R33" s="75"/>
+      <c r="M33" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="R33" s="67"/>
     </row>
     <row r="34" spans="1:18" ht="15.6">
-      <c r="A34" s="72"/>
-      <c r="B34" s="44"/>
-      <c r="C34" s="44"/>
+      <c r="A34" s="64"/>
       <c r="D34" s="19">
         <v>3</v>
       </c>
@@ -4449,29 +4366,25 @@
       <c r="F34" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="G34" s="44"/>
-      <c r="H34" s="44"/>
       <c r="I34" s="20">
         <v>3</v>
       </c>
       <c r="J34" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="K34" s="25"/>
+      <c r="K34" s="25" t="s">
+        <v>181</v>
+      </c>
       <c r="L34" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="M34" s="20"/>
-      <c r="N34" s="44"/>
-      <c r="O34" s="44"/>
-      <c r="P34" s="44"/>
-      <c r="Q34" s="44"/>
-      <c r="R34" s="75"/>
+      <c r="M34" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="R34" s="67"/>
     </row>
     <row r="35" spans="1:18" ht="15.6">
-      <c r="A35" s="72"/>
-      <c r="B35" s="44"/>
-      <c r="C35" s="44"/>
+      <c r="A35" s="64"/>
       <c r="D35" s="19">
         <v>4</v>
       </c>
@@ -4481,181 +4394,97 @@
       <c r="F35" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="G35" s="44"/>
-      <c r="H35" s="44"/>
       <c r="I35" s="20">
         <v>4</v>
       </c>
       <c r="J35" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="K35" s="25"/>
+      <c r="K35" s="25" t="s">
+        <v>168</v>
+      </c>
       <c r="L35" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="M35" s="20"/>
-      <c r="N35" s="44"/>
-      <c r="O35" s="44"/>
-      <c r="P35" s="44"/>
-      <c r="Q35" s="44"/>
-      <c r="R35" s="75"/>
+      <c r="M35" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="R35" s="67"/>
     </row>
     <row r="36" spans="1:18" ht="15.6">
-      <c r="A36" s="72"/>
-      <c r="B36" s="44"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
-      <c r="F36" s="44"/>
-      <c r="G36" s="44"/>
-      <c r="H36" s="44"/>
+      <c r="A36" s="64"/>
       <c r="I36" s="20">
         <v>5</v>
       </c>
       <c r="J36" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="K36" s="25"/>
+      <c r="K36" s="25" t="s">
+        <v>160</v>
+      </c>
       <c r="L36" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="M36" s="20"/>
-      <c r="N36" s="44"/>
-      <c r="O36" s="44"/>
-      <c r="P36" s="44"/>
-      <c r="Q36" s="44"/>
-      <c r="R36" s="75"/>
+      <c r="M36" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="R36" s="67"/>
     </row>
     <row r="37" spans="1:18" ht="15.6">
-      <c r="A37" s="72"/>
-      <c r="B37" s="44"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="44"/>
-      <c r="F37" s="44"/>
-      <c r="G37" s="44"/>
-      <c r="H37" s="44"/>
+      <c r="A37" s="64"/>
       <c r="I37" s="42"/>
       <c r="J37" s="43"/>
-      <c r="K37" s="44"/>
       <c r="L37" s="42"/>
       <c r="M37" s="42"/>
-      <c r="N37" s="44"/>
-      <c r="O37" s="44"/>
-      <c r="P37" s="44"/>
-      <c r="Q37" s="44"/>
-      <c r="R37" s="75"/>
+      <c r="R37" s="67"/>
     </row>
     <row r="38" spans="1:18" ht="15.6">
-      <c r="A38" s="74"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="45"/>
-      <c r="J38" s="46"/>
-      <c r="K38" s="47"/>
-      <c r="L38" s="45"/>
-      <c r="M38" s="45"/>
-      <c r="N38" s="47"/>
-      <c r="O38" s="47"/>
-      <c r="P38" s="47"/>
-      <c r="Q38" s="47"/>
-      <c r="R38" s="79"/>
+      <c r="A38" s="66"/>
+      <c r="B38" s="46"/>
+      <c r="C38" s="46"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="46"/>
+      <c r="I38" s="44"/>
+      <c r="J38" s="45"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="44"/>
+      <c r="M38" s="44"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="46"/>
+      <c r="Q38" s="46"/>
+      <c r="R38" s="71"/>
     </row>
     <row r="39" spans="1:18">
-      <c r="A39" s="72"/>
-      <c r="B39" s="44"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="44"/>
-      <c r="G39" s="44"/>
-      <c r="H39" s="44"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="44"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="44"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="44"/>
-      <c r="P39" s="44"/>
-      <c r="Q39" s="44"/>
-      <c r="R39" s="75"/>
+      <c r="A39" s="64"/>
+      <c r="R39" s="67"/>
     </row>
     <row r="40" spans="1:18">
-      <c r="A40" s="72"/>
-      <c r="B40" s="44"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="44"/>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="44"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="44"/>
-      <c r="L40" s="44"/>
-      <c r="M40" s="44"/>
-      <c r="N40" s="44"/>
-      <c r="O40" s="44"/>
-      <c r="P40" s="44"/>
-      <c r="Q40" s="44"/>
-      <c r="R40" s="75"/>
+      <c r="A40" s="64"/>
+      <c r="R40" s="67"/>
     </row>
     <row r="41" spans="1:18" ht="20.399999999999999">
-      <c r="A41" s="72"/>
+      <c r="A41" s="64"/>
       <c r="B41" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="44"/>
-      <c r="D41" s="44"/>
-      <c r="E41" s="44"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="44"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="44"/>
-      <c r="L41" s="44"/>
-      <c r="M41" s="44"/>
-      <c r="N41" s="44"/>
-      <c r="O41" s="44"/>
-      <c r="P41" s="44"/>
-      <c r="Q41" s="44"/>
-      <c r="R41" s="75"/>
+      <c r="R41" s="67"/>
     </row>
     <row r="42" spans="1:18" ht="20.399999999999999">
-      <c r="A42" s="72"/>
-      <c r="B42" s="44"/>
+      <c r="A42" s="64"/>
       <c r="C42" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
-      <c r="F42" s="44"/>
-      <c r="G42" s="44"/>
       <c r="H42" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I42" s="44"/>
-      <c r="J42" s="44"/>
-      <c r="K42" s="44"/>
-      <c r="L42" s="44"/>
-      <c r="M42" s="44"/>
-      <c r="N42" s="44"/>
-      <c r="O42" s="44"/>
-      <c r="P42" s="44"/>
-      <c r="Q42" s="44"/>
-      <c r="R42" s="75"/>
+      <c r="R42" s="67"/>
     </row>
     <row r="43" spans="1:18" ht="15.6">
-      <c r="A43" s="72"/>
-      <c r="B43" s="44"/>
-      <c r="C43" s="44"/>
+      <c r="A43" s="64"/>
       <c r="D43" s="29" t="s">
         <v>7</v>
       </c>
@@ -4665,23 +4494,27 @@
       <c r="F43" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="G43" s="44"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="44"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="44"/>
-      <c r="L43" s="44"/>
-      <c r="M43" s="44"/>
-      <c r="N43" s="60"/>
-      <c r="O43" s="44"/>
-      <c r="P43" s="61"/>
-      <c r="Q43" s="44"/>
-      <c r="R43" s="75"/>
+      <c r="I43" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="N43" s="54"/>
+      <c r="P43" s="55"/>
+      <c r="R43" s="67"/>
     </row>
     <row r="44" spans="1:18" ht="15.6">
-      <c r="A44" s="72"/>
-      <c r="B44" s="44"/>
-      <c r="C44" s="44"/>
+      <c r="A44" s="64"/>
       <c r="D44" s="20">
         <v>1</v>
       </c>
@@ -4691,31 +4524,27 @@
       <c r="F44" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="G44" s="44"/>
-      <c r="H44" s="44"/>
-      <c r="I44" s="48">
+      <c r="I44" s="47">
         <v>1</v>
       </c>
       <c r="J44" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="K44" s="50" t="s">
+      <c r="K44" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="L44" s="48" t="s">
+      <c r="L44" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="M44" s="48"/>
-      <c r="N44" s="62"/>
-      <c r="O44" s="44"/>
-      <c r="P44" s="63"/>
-      <c r="Q44" s="44"/>
-      <c r="R44" s="75"/>
+      <c r="M44" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="N44" s="16"/>
+      <c r="P44" s="56"/>
+      <c r="R44" s="67"/>
     </row>
     <row r="45" spans="1:18" ht="15.6">
-      <c r="A45" s="72"/>
-      <c r="B45" s="44"/>
-      <c r="C45" s="44"/>
+      <c r="A45" s="64"/>
       <c r="D45" s="20">
         <v>2</v>
       </c>
@@ -4725,31 +4554,27 @@
       <c r="F45" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="G45" s="44"/>
-      <c r="H45" s="44"/>
-      <c r="I45" s="48">
+      <c r="I45" s="47">
         <v>2</v>
       </c>
       <c r="J45" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="K45" s="50" t="s">
+      <c r="K45" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="L45" s="48" t="s">
+      <c r="L45" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="M45" s="48"/>
-      <c r="N45" s="62"/>
-      <c r="O45" s="44"/>
-      <c r="P45" s="63"/>
-      <c r="Q45" s="44"/>
-      <c r="R45" s="75"/>
+      <c r="M45" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="N45" s="16"/>
+      <c r="P45" s="56"/>
+      <c r="R45" s="67"/>
     </row>
     <row r="46" spans="1:18" ht="15.6">
-      <c r="A46" s="72"/>
-      <c r="B46" s="44"/>
-      <c r="C46" s="44"/>
+      <c r="A46" s="64"/>
       <c r="D46" s="20">
         <v>3</v>
       </c>
@@ -4759,277 +4584,191 @@
       <c r="F46" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="G46" s="44"/>
-      <c r="H46" s="44"/>
-      <c r="I46" s="48">
+      <c r="I46" s="47">
         <v>3</v>
       </c>
       <c r="J46" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="K46" s="50" t="s">
+      <c r="K46" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="25" t="s">
+      <c r="L46" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="M46" s="48"/>
-      <c r="N46" s="62"/>
-      <c r="O46" s="44"/>
-      <c r="P46" s="63"/>
-      <c r="Q46" s="44"/>
-      <c r="R46" s="75"/>
+      <c r="M46" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="N46" s="16"/>
+      <c r="P46" s="56"/>
+      <c r="R46" s="67"/>
     </row>
     <row r="47" spans="1:18" ht="15.6">
-      <c r="A47" s="72"/>
-      <c r="B47" s="44"/>
-      <c r="C47" s="44"/>
+      <c r="A47" s="64"/>
       <c r="D47" s="20">
         <v>4</v>
       </c>
-      <c r="E47" s="49" t="s">
+      <c r="E47" s="48" t="s">
         <v>195</v>
       </c>
-      <c r="F47" s="17"/>
-      <c r="G47" s="44"/>
-      <c r="H47" s="44"/>
-      <c r="I47" s="48">
+      <c r="F47" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="I47" s="47">
         <v>4</v>
       </c>
       <c r="J47" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="K47" s="50" t="s">
+      <c r="K47" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="L47" s="48" t="s">
+      <c r="L47" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="M47" s="48"/>
-      <c r="N47" s="62"/>
-      <c r="O47" s="44"/>
-      <c r="P47" s="44"/>
-      <c r="Q47" s="44"/>
-      <c r="R47" s="75"/>
+      <c r="M47" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="N47" s="16"/>
+      <c r="R47" s="67"/>
     </row>
     <row r="48" spans="1:18" ht="15.6">
-      <c r="A48" s="72"/>
-      <c r="B48" s="44"/>
-      <c r="C48" s="44"/>
+      <c r="A48" s="64"/>
       <c r="D48" s="20">
         <v>5</v>
       </c>
-      <c r="E48" s="49" t="s">
+      <c r="E48" s="48" t="s">
         <v>196</v>
       </c>
-      <c r="F48" s="17"/>
-      <c r="G48" s="44"/>
-      <c r="H48" s="44"/>
-      <c r="I48" s="48">
+      <c r="F48" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="I48" s="47">
         <v>5</v>
       </c>
       <c r="J48" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="K48" s="50" t="s">
+      <c r="K48" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="L48" s="48" t="s">
+      <c r="L48" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="M48" s="48"/>
-      <c r="N48" s="62"/>
-      <c r="O48" s="44"/>
-      <c r="P48" s="44"/>
-      <c r="Q48" s="44"/>
-      <c r="R48" s="75"/>
+      <c r="M48" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="N48" s="16"/>
+      <c r="R48" s="67"/>
     </row>
     <row r="49" spans="1:18" ht="15.6">
-      <c r="A49" s="72"/>
-      <c r="B49" s="44"/>
-      <c r="C49" s="44"/>
+      <c r="A49" s="64"/>
       <c r="D49" s="20">
         <v>6</v>
       </c>
-      <c r="E49" s="49" t="s">
+      <c r="E49" s="48" t="s">
         <v>197</v>
       </c>
-      <c r="F49" s="17"/>
-      <c r="G49" s="44"/>
-      <c r="H49" s="44"/>
-      <c r="I49" s="48">
+      <c r="F49" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="I49" s="47">
         <v>6</v>
       </c>
-      <c r="J49" s="48" t="s">
+      <c r="J49" s="47" t="s">
         <v>203</v>
       </c>
-      <c r="K49" s="50" t="s">
+      <c r="K49" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="L49" s="48" t="s">
+      <c r="L49" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="M49" s="48"/>
-      <c r="N49" s="62"/>
-      <c r="O49" s="44"/>
-      <c r="P49" s="44"/>
-      <c r="Q49" s="44"/>
-      <c r="R49" s="75"/>
+      <c r="M49" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="N49" s="16"/>
+      <c r="R49" s="67"/>
     </row>
     <row r="50" spans="1:18" ht="15.6">
-      <c r="A50" s="72"/>
-      <c r="B50" s="44"/>
-      <c r="C50" s="44"/>
+      <c r="A50" s="64"/>
       <c r="D50" s="20">
         <v>7</v>
       </c>
-      <c r="E50" s="49" t="s">
+      <c r="E50" s="48" t="s">
         <v>198</v>
       </c>
-      <c r="F50" s="17"/>
-      <c r="G50" s="44"/>
-      <c r="H50" s="44"/>
-      <c r="I50" s="44"/>
-      <c r="J50" s="62"/>
-      <c r="K50" s="64"/>
-      <c r="L50" s="62"/>
-      <c r="M50" s="62"/>
-      <c r="N50" s="62"/>
-      <c r="O50" s="44"/>
-      <c r="P50" s="44"/>
-      <c r="Q50" s="44"/>
-      <c r="R50" s="75"/>
+      <c r="F50" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="J50" s="16"/>
+      <c r="K50" s="57"/>
+      <c r="L50" s="16"/>
+      <c r="M50" s="16"/>
+      <c r="N50" s="16"/>
+      <c r="R50" s="67"/>
     </row>
     <row r="51" spans="1:18">
-      <c r="A51" s="72"/>
-      <c r="B51" s="44"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
-      <c r="F51" s="44"/>
-      <c r="G51" s="44"/>
-      <c r="H51" s="44"/>
-      <c r="I51" s="44"/>
-      <c r="J51" s="62"/>
-      <c r="K51" s="64"/>
-      <c r="L51" s="62"/>
-      <c r="M51" s="62"/>
-      <c r="N51" s="62"/>
-      <c r="O51" s="44"/>
-      <c r="P51" s="44"/>
-      <c r="Q51" s="44"/>
-      <c r="R51" s="75"/>
+      <c r="A51" s="64"/>
+      <c r="J51" s="16"/>
+      <c r="K51" s="57"/>
+      <c r="L51" s="16"/>
+      <c r="M51" s="16"/>
+      <c r="N51" s="16"/>
+      <c r="R51" s="67"/>
     </row>
     <row r="52" spans="1:18">
-      <c r="A52" s="74"/>
-      <c r="B52" s="47"/>
-      <c r="C52" s="47"/>
-      <c r="D52" s="47"/>
-      <c r="E52" s="47"/>
-      <c r="F52" s="47"/>
-      <c r="G52" s="47"/>
-      <c r="H52" s="47"/>
-      <c r="I52" s="47"/>
-      <c r="J52" s="65"/>
-      <c r="K52" s="66"/>
-      <c r="L52" s="65"/>
-      <c r="M52" s="65"/>
-      <c r="N52" s="65"/>
-      <c r="O52" s="47"/>
-      <c r="P52" s="47"/>
-      <c r="Q52" s="47"/>
-      <c r="R52" s="79"/>
+      <c r="A52" s="66"/>
+      <c r="B52" s="46"/>
+      <c r="C52" s="46"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="46"/>
+      <c r="I52" s="46"/>
+      <c r="J52" s="58"/>
+      <c r="K52" s="59"/>
+      <c r="L52" s="58"/>
+      <c r="M52" s="58"/>
+      <c r="N52" s="58"/>
+      <c r="O52" s="46"/>
+      <c r="P52" s="46"/>
+      <c r="Q52" s="46"/>
+      <c r="R52" s="71"/>
     </row>
     <row r="53" spans="1:18">
-      <c r="A53" s="72"/>
-      <c r="B53" s="44"/>
-      <c r="C53" s="44"/>
-      <c r="D53" s="44"/>
-      <c r="E53" s="44"/>
-      <c r="F53" s="44"/>
-      <c r="G53" s="44"/>
-      <c r="H53" s="44"/>
-      <c r="I53" s="44"/>
-      <c r="J53" s="62"/>
-      <c r="K53" s="64"/>
-      <c r="L53" s="62"/>
-      <c r="M53" s="62"/>
-      <c r="N53" s="62"/>
-      <c r="O53" s="44"/>
-      <c r="P53" s="44"/>
-      <c r="Q53" s="44"/>
-      <c r="R53" s="75"/>
+      <c r="A53" s="64"/>
+      <c r="J53" s="16"/>
+      <c r="K53" s="57"/>
+      <c r="L53" s="16"/>
+      <c r="M53" s="16"/>
+      <c r="N53" s="16"/>
+      <c r="R53" s="67"/>
     </row>
     <row r="54" spans="1:18">
-      <c r="A54" s="72"/>
-      <c r="B54" s="44"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="44"/>
-      <c r="E54" s="44"/>
-      <c r="F54" s="44"/>
-      <c r="G54" s="44"/>
-      <c r="H54" s="44"/>
-      <c r="I54" s="44"/>
-      <c r="J54" s="44"/>
-      <c r="K54" s="44"/>
-      <c r="L54" s="44"/>
-      <c r="M54" s="44"/>
-      <c r="N54" s="44"/>
-      <c r="O54" s="44"/>
-      <c r="P54" s="44"/>
-      <c r="Q54" s="44"/>
-      <c r="R54" s="75"/>
+      <c r="A54" s="64"/>
+      <c r="R54" s="67"/>
     </row>
     <row r="55" spans="1:18" ht="20.399999999999999">
-      <c r="A55" s="72"/>
+      <c r="A55" s="64"/>
       <c r="B55" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="44"/>
-      <c r="F55" s="44"/>
-      <c r="G55" s="44"/>
-      <c r="H55" s="44"/>
-      <c r="I55" s="44"/>
-      <c r="J55" s="44"/>
-      <c r="K55" s="44"/>
-      <c r="L55" s="44"/>
-      <c r="M55" s="44"/>
-      <c r="N55" s="44"/>
-      <c r="O55" s="44"/>
-      <c r="P55" s="44"/>
-      <c r="Q55" s="44"/>
-      <c r="R55" s="75"/>
+      <c r="R55" s="67"/>
     </row>
     <row r="56" spans="1:18" ht="20.399999999999999">
-      <c r="A56" s="72"/>
-      <c r="B56" s="44"/>
+      <c r="A56" s="64"/>
       <c r="C56" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D56" s="44"/>
-      <c r="E56" s="44"/>
-      <c r="F56" s="44"/>
-      <c r="G56" s="44"/>
       <c r="H56" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I56" s="44"/>
-      <c r="J56" s="44"/>
-      <c r="K56" s="44"/>
-      <c r="L56" s="44"/>
-      <c r="M56" s="44"/>
-      <c r="N56" s="44"/>
-      <c r="O56" s="44"/>
-      <c r="P56" s="44"/>
-      <c r="Q56" s="44"/>
-      <c r="R56" s="75"/>
+      <c r="R56" s="67"/>
     </row>
     <row r="57" spans="1:18" ht="15.6">
-      <c r="A57" s="72"/>
-      <c r="B57" s="44"/>
-      <c r="C57" s="44"/>
+      <c r="A57" s="64"/>
       <c r="D57" s="29" t="s">
         <v>7</v>
       </c>
@@ -5039,8 +4778,6 @@
       <c r="F57" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="G57" s="44"/>
-      <c r="H57" s="44"/>
       <c r="I57" s="3" t="s">
         <v>7</v>
       </c>
@@ -5056,16 +4793,11 @@
       <c r="M57" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="N57" s="60"/>
-      <c r="O57" s="44"/>
-      <c r="P57" s="44"/>
-      <c r="Q57" s="44"/>
-      <c r="R57" s="75"/>
+      <c r="N57" s="54"/>
+      <c r="R57" s="67"/>
     </row>
     <row r="58" spans="1:18" ht="15.6">
-      <c r="A58" s="72"/>
-      <c r="B58" s="44"/>
-      <c r="C58" s="44"/>
+      <c r="A58" s="64"/>
       <c r="D58" s="20">
         <v>1</v>
       </c>
@@ -5075,8 +4807,6 @@
       <c r="F58" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="G58" s="44"/>
-      <c r="H58" s="44"/>
       <c r="I58" s="20">
         <v>1</v>
       </c>
@@ -5089,17 +4819,14 @@
       <c r="L58" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="M58" s="51"/>
-      <c r="N58" s="62"/>
-      <c r="O58" s="44"/>
-      <c r="P58" s="44"/>
-      <c r="Q58" s="44"/>
-      <c r="R58" s="75"/>
+      <c r="M58" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="N58" s="16"/>
+      <c r="R58" s="67"/>
     </row>
     <row r="59" spans="1:18" ht="15.6">
-      <c r="A59" s="72"/>
-      <c r="B59" s="44"/>
-      <c r="C59" s="44"/>
+      <c r="A59" s="64"/>
       <c r="D59" s="20">
         <v>2</v>
       </c>
@@ -5109,8 +4836,6 @@
       <c r="F59" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="G59" s="44"/>
-      <c r="H59" s="44"/>
       <c r="I59" s="20">
         <v>2</v>
       </c>
@@ -5123,22 +4848,14 @@
       <c r="L59" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="M59" s="51"/>
-      <c r="N59" s="62"/>
-      <c r="O59" s="44"/>
-      <c r="P59" s="44"/>
-      <c r="Q59" s="44"/>
-      <c r="R59" s="75"/>
+      <c r="M59" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="N59" s="16"/>
+      <c r="R59" s="67"/>
     </row>
     <row r="60" spans="1:18" ht="15.6">
-      <c r="A60" s="72"/>
-      <c r="B60" s="44"/>
-      <c r="C60" s="44"/>
-      <c r="D60" s="44"/>
-      <c r="E60" s="44"/>
-      <c r="F60" s="44"/>
-      <c r="G60" s="44"/>
-      <c r="H60" s="44"/>
+      <c r="A60" s="64"/>
       <c r="I60" s="20">
         <v>3</v>
       </c>
@@ -5151,22 +4868,14 @@
       <c r="L60" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="M60" s="51"/>
-      <c r="N60" s="62"/>
-      <c r="O60" s="44"/>
-      <c r="P60" s="44"/>
-      <c r="Q60" s="44"/>
-      <c r="R60" s="75"/>
+      <c r="M60" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="N60" s="16"/>
+      <c r="R60" s="67"/>
     </row>
     <row r="61" spans="1:18" ht="15.6">
-      <c r="A61" s="72"/>
-      <c r="B61" s="44"/>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="44"/>
-      <c r="F61" s="44"/>
-      <c r="G61" s="44"/>
-      <c r="H61" s="44"/>
+      <c r="A61" s="64"/>
       <c r="I61" s="20">
         <v>4</v>
       </c>
@@ -5179,22 +4888,14 @@
       <c r="L61" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="M61" s="51"/>
-      <c r="N61" s="62"/>
-      <c r="O61" s="44"/>
-      <c r="P61" s="44"/>
-      <c r="Q61" s="44"/>
-      <c r="R61" s="75"/>
-    </row>
-    <row r="62" spans="1:18" ht="31.2">
-      <c r="A62" s="72"/>
-      <c r="B62" s="44"/>
-      <c r="C62" s="44"/>
-      <c r="D62" s="44"/>
-      <c r="E62" s="44"/>
-      <c r="F62" s="44"/>
-      <c r="G62" s="44"/>
-      <c r="H62" s="44"/>
+      <c r="M61" s="17" t="s">
+        <v>274</v>
+      </c>
+      <c r="N61" s="16"/>
+      <c r="R61" s="67"/>
+    </row>
+    <row r="62" spans="1:18" ht="15.6">
+      <c r="A62" s="64"/>
       <c r="I62" s="20">
         <v>5</v>
       </c>
@@ -5207,145 +4908,70 @@
       <c r="L62" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="M62" s="51"/>
-      <c r="N62" s="62"/>
-      <c r="O62" s="44"/>
-      <c r="P62" s="44"/>
-      <c r="Q62" s="44"/>
-      <c r="R62" s="75"/>
+      <c r="M62" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="N62" s="16"/>
+      <c r="R62" s="67"/>
     </row>
     <row r="63" spans="1:18">
-      <c r="A63" s="72"/>
-      <c r="B63" s="44"/>
-      <c r="C63" s="44"/>
-      <c r="D63" s="44"/>
-      <c r="E63" s="44"/>
-      <c r="F63" s="44"/>
-      <c r="G63" s="44"/>
-      <c r="H63" s="44"/>
-      <c r="I63" s="62"/>
-      <c r="J63" s="44"/>
-      <c r="K63" s="64"/>
-      <c r="L63" s="62"/>
-      <c r="M63" s="67"/>
-      <c r="N63" s="62"/>
-      <c r="O63" s="44"/>
-      <c r="P63" s="44"/>
-      <c r="Q63" s="44"/>
-      <c r="R63" s="75"/>
+      <c r="A63" s="64"/>
+      <c r="I63" s="16"/>
+      <c r="K63" s="57"/>
+      <c r="L63" s="16"/>
+      <c r="M63" s="60"/>
+      <c r="N63" s="16"/>
+      <c r="R63" s="67"/>
     </row>
     <row r="64" spans="1:18">
-      <c r="A64" s="74"/>
-      <c r="B64" s="47"/>
-      <c r="C64" s="47"/>
-      <c r="D64" s="47"/>
-      <c r="E64" s="47"/>
-      <c r="F64" s="47"/>
-      <c r="G64" s="47"/>
-      <c r="H64" s="47"/>
-      <c r="I64" s="47"/>
-      <c r="J64" s="47"/>
-      <c r="K64" s="47"/>
-      <c r="L64" s="47"/>
-      <c r="M64" s="47"/>
-      <c r="N64" s="47"/>
-      <c r="O64" s="44"/>
-      <c r="P64" s="44"/>
-      <c r="Q64" s="44"/>
-      <c r="R64" s="75"/>
+      <c r="A64" s="66"/>
+      <c r="B64" s="46"/>
+      <c r="C64" s="46"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="46"/>
+      <c r="K64" s="46"/>
+      <c r="L64" s="46"/>
+      <c r="M64" s="46"/>
+      <c r="N64" s="46"/>
+      <c r="R64" s="67"/>
     </row>
     <row r="65" spans="1:20">
-      <c r="A65" s="72"/>
-      <c r="B65" s="44"/>
-      <c r="C65" s="44"/>
-      <c r="D65" s="44"/>
-      <c r="E65" s="44"/>
-      <c r="F65" s="44"/>
-      <c r="G65" s="44"/>
-      <c r="H65" s="44"/>
-      <c r="I65" s="44"/>
-      <c r="J65" s="44"/>
-      <c r="K65" s="44"/>
-      <c r="L65" s="44"/>
-      <c r="M65" s="44"/>
-      <c r="N65" s="44"/>
-      <c r="O65" s="44"/>
-      <c r="P65" s="44"/>
-      <c r="Q65" s="44"/>
-      <c r="R65" s="75"/>
+      <c r="A65" s="64"/>
+      <c r="R65" s="67"/>
     </row>
     <row r="66" spans="1:20">
-      <c r="A66" s="72"/>
-      <c r="B66" s="44"/>
-      <c r="C66" s="44"/>
-      <c r="D66" s="44"/>
-      <c r="E66" s="44"/>
-      <c r="F66" s="44"/>
-      <c r="G66" s="44"/>
-      <c r="H66" s="44"/>
-      <c r="I66" s="44"/>
-      <c r="J66" s="44"/>
-      <c r="K66" s="44"/>
-      <c r="L66" s="44"/>
-      <c r="M66" s="44"/>
-      <c r="N66" s="44"/>
-      <c r="O66" s="44"/>
-      <c r="P66" s="44"/>
-      <c r="Q66" s="44"/>
-      <c r="R66" s="75"/>
+      <c r="A66" s="64"/>
+      <c r="R66" s="67"/>
     </row>
     <row r="67" spans="1:20" ht="20.399999999999999">
-      <c r="A67" s="72"/>
+      <c r="A67" s="64"/>
       <c r="B67" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-      <c r="E67" s="44"/>
-      <c r="F67" s="44"/>
-      <c r="G67" s="44"/>
-      <c r="H67" s="44"/>
-      <c r="I67" s="44"/>
-      <c r="J67" s="44"/>
-      <c r="K67" s="44"/>
-      <c r="L67" s="44"/>
-      <c r="M67" s="44"/>
-      <c r="N67" s="44"/>
-      <c r="O67" s="44"/>
-      <c r="P67" s="44"/>
-      <c r="Q67" s="44"/>
-      <c r="R67" s="75"/>
+      <c r="R67" s="67"/>
     </row>
     <row r="68" spans="1:20" ht="20.399999999999999">
-      <c r="A68" s="72"/>
-      <c r="B68" s="44"/>
+      <c r="A68" s="64"/>
       <c r="C68" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D68" s="44"/>
-      <c r="E68" s="44"/>
-      <c r="F68" s="44"/>
-      <c r="G68" s="44"/>
       <c r="H68" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I68" s="44"/>
-      <c r="J68" s="44"/>
-      <c r="K68" s="44"/>
-      <c r="L68" s="44"/>
-      <c r="M68" s="44"/>
-      <c r="N68" s="44"/>
       <c r="O68" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="P68" s="57"/>
-      <c r="Q68" s="57"/>
-      <c r="R68" s="73"/>
+      <c r="P68" s="11"/>
+      <c r="Q68" s="11"/>
+      <c r="R68" s="65"/>
     </row>
     <row r="69" spans="1:20" ht="15.6">
-      <c r="A69" s="72"/>
-      <c r="B69" s="44"/>
-      <c r="C69" s="44"/>
+      <c r="A69" s="64"/>
       <c r="D69" s="29" t="s">
         <v>7</v>
       </c>
@@ -5355,8 +4981,6 @@
       <c r="F69" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="G69" s="44"/>
-      <c r="H69" s="44"/>
       <c r="I69" s="3" t="s">
         <v>7</v>
       </c>
@@ -5372,31 +4996,28 @@
       <c r="M69" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="N69" s="44"/>
-      <c r="O69" s="57"/>
+      <c r="O69" s="11"/>
       <c r="P69" s="39" t="s">
         <v>7</v>
       </c>
       <c r="Q69" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="R69" s="76" t="s">
+      <c r="R69" s="68" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="70" spans="1:20" ht="15.6">
-      <c r="A70" s="72"/>
-      <c r="B70" s="44"/>
-      <c r="C70" s="44"/>
+      <c r="A70" s="64"/>
       <c r="D70" s="20">
         <v>1</v>
       </c>
       <c r="E70" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="F70" s="20"/>
-      <c r="G70" s="44"/>
-      <c r="H70" s="44"/>
+      <c r="F70" s="17" t="s">
+        <v>258</v>
+      </c>
       <c r="I70" s="20">
         <v>1</v>
       </c>
@@ -5406,35 +5027,33 @@
       <c r="K70" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="L70" s="51" t="s">
+      <c r="L70" s="50" t="s">
         <v>228</v>
       </c>
-      <c r="M70" s="17"/>
-      <c r="N70" s="44"/>
-      <c r="O70" s="44"/>
+      <c r="M70" s="17" t="s">
+        <v>276</v>
+      </c>
       <c r="P70" s="17">
         <v>1</v>
       </c>
       <c r="Q70" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="R70" s="77" t="s">
+      <c r="R70" s="69" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="30">
-      <c r="A71" s="72"/>
-      <c r="B71" s="44"/>
-      <c r="C71" s="44"/>
+    <row r="71" spans="1:20" ht="31.2">
+      <c r="A71" s="64"/>
       <c r="D71" s="20">
         <v>2</v>
       </c>
       <c r="E71" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="F71" s="20"/>
-      <c r="G71" s="44"/>
-      <c r="H71" s="44"/>
+      <c r="F71" s="17" t="s">
+        <v>259</v>
+      </c>
       <c r="I71" s="20">
         <v>2</v>
       </c>
@@ -5444,31 +5063,24 @@
       <c r="K71" s="17" t="s">
         <v>233</v>
       </c>
-      <c r="L71" s="51" t="s">
+      <c r="L71" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="M71" s="17"/>
-      <c r="N71" s="44"/>
-      <c r="O71" s="44"/>
+      <c r="M71" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="P71" s="17">
         <v>2</v>
       </c>
       <c r="Q71" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="R71" s="78" t="s">
+      <c r="R71" s="70" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="72" spans="1:20" ht="15.6">
-      <c r="A72" s="72"/>
-      <c r="B72" s="44"/>
-      <c r="C72" s="44"/>
-      <c r="D72" s="44"/>
-      <c r="E72" s="44"/>
-      <c r="F72" s="44"/>
-      <c r="G72" s="44"/>
-      <c r="H72" s="44"/>
+      <c r="A72" s="64"/>
       <c r="I72" s="20">
         <v>3</v>
       </c>
@@ -5478,205 +5090,107 @@
       <c r="K72" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="L72" s="51" t="s">
+      <c r="L72" s="50" t="s">
         <v>230</v>
       </c>
-      <c r="M72" s="17"/>
-      <c r="N72" s="44"/>
-      <c r="O72" s="44"/>
-      <c r="P72" s="44"/>
-      <c r="Q72" s="44"/>
-      <c r="R72" s="75"/>
+      <c r="M72" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="R72" s="67"/>
     </row>
     <row r="73" spans="1:20" ht="15.6">
-      <c r="A73" s="72"/>
-      <c r="B73" s="44"/>
-      <c r="C73" s="44"/>
-      <c r="D73" s="44"/>
-      <c r="E73" s="44"/>
-      <c r="F73" s="44"/>
-      <c r="G73" s="44"/>
-      <c r="H73" s="44"/>
-      <c r="I73" s="53">
+      <c r="A73" s="64"/>
+      <c r="I73" s="20">
         <v>4</v>
       </c>
-      <c r="J73" s="54" t="s">
+      <c r="J73" s="21" t="s">
         <v>226</v>
       </c>
       <c r="K73" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="L73" s="55" t="s">
+      <c r="L73" s="50" t="s">
         <v>231</v>
       </c>
-      <c r="M73" s="17"/>
-      <c r="N73" s="44"/>
-      <c r="O73" s="44"/>
-      <c r="P73" s="44"/>
-      <c r="Q73" s="44"/>
-      <c r="R73" s="75"/>
+      <c r="M73" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="R73" s="67"/>
     </row>
     <row r="74" spans="1:20" ht="15.6">
-      <c r="A74" s="72"/>
-      <c r="B74" s="44"/>
-      <c r="C74" s="44"/>
-      <c r="D74" s="44"/>
-      <c r="E74" s="44"/>
-      <c r="F74" s="44"/>
-      <c r="G74" s="44"/>
-      <c r="H74" s="44"/>
-      <c r="I74" s="53">
+      <c r="A74" s="64"/>
+      <c r="I74" s="20">
         <v>5</v>
       </c>
-      <c r="J74" s="54" t="s">
+      <c r="J74" s="21" t="s">
         <v>227</v>
       </c>
       <c r="K74" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="L74" s="55" t="s">
+      <c r="L74" s="50" t="s">
         <v>232</v>
       </c>
-      <c r="M74" s="17"/>
-      <c r="N74" s="44"/>
-      <c r="O74" s="44"/>
-      <c r="P74" s="44"/>
-      <c r="Q74" s="44"/>
-      <c r="R74" s="75"/>
+      <c r="M74" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="R74" s="67"/>
     </row>
     <row r="75" spans="1:20">
-      <c r="A75" s="72"/>
-      <c r="B75" s="44"/>
-      <c r="C75" s="44"/>
-      <c r="D75" s="52"/>
-      <c r="E75" s="44"/>
-      <c r="F75" s="44"/>
-      <c r="G75" s="44"/>
-      <c r="H75" s="44"/>
-      <c r="I75" s="44"/>
-      <c r="J75" s="44"/>
-      <c r="K75" s="44"/>
-      <c r="L75" s="44"/>
-      <c r="M75" s="44"/>
-      <c r="N75" s="44"/>
-      <c r="O75" s="44"/>
-      <c r="P75" s="44"/>
-      <c r="Q75" s="44"/>
-      <c r="R75" s="75"/>
+      <c r="A75" s="64"/>
+      <c r="D75" s="16"/>
+      <c r="R75" s="67"/>
     </row>
     <row r="76" spans="1:20">
-      <c r="A76" s="74"/>
-      <c r="B76" s="47"/>
-      <c r="C76" s="47"/>
-      <c r="D76" s="47"/>
-      <c r="E76" s="47"/>
-      <c r="F76" s="47"/>
-      <c r="G76" s="47"/>
-      <c r="H76" s="47"/>
-      <c r="I76" s="47"/>
-      <c r="J76" s="47"/>
-      <c r="K76" s="47"/>
-      <c r="L76" s="47"/>
-      <c r="M76" s="47"/>
-      <c r="N76" s="47"/>
-      <c r="O76" s="47"/>
-      <c r="P76" s="47"/>
-      <c r="Q76" s="47"/>
-      <c r="R76" s="79"/>
+      <c r="A76" s="66"/>
+      <c r="B76" s="46"/>
+      <c r="C76" s="46"/>
+      <c r="D76" s="46"/>
+      <c r="E76" s="46"/>
+      <c r="F76" s="46"/>
+      <c r="G76" s="46"/>
+      <c r="H76" s="46"/>
+      <c r="I76" s="46"/>
+      <c r="J76" s="46"/>
+      <c r="K76" s="46"/>
+      <c r="L76" s="46"/>
+      <c r="M76" s="46"/>
+      <c r="N76" s="46"/>
+      <c r="O76" s="46"/>
+      <c r="P76" s="46"/>
+      <c r="Q76" s="46"/>
+      <c r="R76" s="71"/>
     </row>
     <row r="77" spans="1:20">
-      <c r="A77" s="72"/>
-      <c r="B77" s="44"/>
-      <c r="C77" s="44"/>
-      <c r="D77" s="44"/>
-      <c r="E77" s="44"/>
-      <c r="F77" s="44"/>
-      <c r="G77" s="44"/>
-      <c r="H77" s="44"/>
-      <c r="I77" s="44"/>
-      <c r="J77" s="44"/>
-      <c r="K77" s="44"/>
-      <c r="L77" s="44"/>
-      <c r="M77" s="44"/>
-      <c r="N77" s="44"/>
-      <c r="O77" s="44"/>
-      <c r="P77" s="44"/>
-      <c r="Q77" s="44"/>
-      <c r="R77" s="75"/>
+      <c r="A77" s="64"/>
+      <c r="R77" s="67"/>
       <c r="T77" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="78" spans="1:20">
-      <c r="A78" s="72"/>
-      <c r="B78" s="44"/>
-      <c r="C78" s="44"/>
-      <c r="D78" s="44"/>
-      <c r="E78" s="44"/>
-      <c r="F78" s="44"/>
-      <c r="G78" s="44"/>
-      <c r="H78" s="44"/>
-      <c r="I78" s="44"/>
-      <c r="J78" s="44"/>
-      <c r="K78" s="44"/>
-      <c r="L78" s="44"/>
-      <c r="M78" s="44"/>
-      <c r="N78" s="44"/>
-      <c r="O78" s="44"/>
-      <c r="P78" s="44"/>
-      <c r="Q78" s="44"/>
-      <c r="R78" s="75"/>
+      <c r="A78" s="64"/>
+      <c r="R78" s="67"/>
     </row>
     <row r="79" spans="1:20" ht="20.399999999999999">
-      <c r="A79" s="72"/>
+      <c r="A79" s="64"/>
       <c r="B79" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="C79" s="44"/>
-      <c r="D79" s="44"/>
-      <c r="E79" s="44"/>
-      <c r="F79" s="44"/>
-      <c r="G79" s="44"/>
-      <c r="H79" s="44"/>
-      <c r="I79" s="44"/>
-      <c r="J79" s="44"/>
-      <c r="K79" s="44"/>
-      <c r="L79" s="44"/>
-      <c r="M79" s="44"/>
-      <c r="N79" s="44"/>
-      <c r="O79" s="44"/>
-      <c r="P79" s="44"/>
-      <c r="Q79" s="44"/>
-      <c r="R79" s="75"/>
+      <c r="R79" s="67"/>
     </row>
     <row r="80" spans="1:20" ht="20.399999999999999">
-      <c r="A80" s="72"/>
-      <c r="B80" s="44"/>
+      <c r="A80" s="64"/>
       <c r="C80" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D80" s="44"/>
-      <c r="E80" s="44"/>
-      <c r="F80" s="44"/>
-      <c r="G80" s="44"/>
       <c r="H80" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I80" s="44"/>
-      <c r="J80" s="44"/>
-      <c r="K80" s="44"/>
-      <c r="L80" s="44"/>
-      <c r="M80" s="44"/>
-      <c r="N80" s="44"/>
-      <c r="O80" s="44"/>
-      <c r="P80" s="44"/>
-      <c r="Q80" s="44"/>
-      <c r="R80" s="75"/>
+      <c r="R80" s="67"/>
     </row>
     <row r="81" spans="1:18" ht="15.6">
-      <c r="A81" s="72"/>
-      <c r="B81" s="44"/>
-      <c r="C81" s="44"/>
+      <c r="A81" s="64"/>
       <c r="D81" s="29" t="s">
         <v>7</v>
       </c>
@@ -5686,8 +5200,6 @@
       <c r="F81" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="G81" s="44"/>
-      <c r="H81" s="44"/>
       <c r="I81" s="3" t="s">
         <v>7</v>
       </c>
@@ -5703,16 +5215,10 @@
       <c r="M81" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="N81" s="44"/>
-      <c r="O81" s="44"/>
-      <c r="P81" s="44"/>
-      <c r="Q81" s="44"/>
-      <c r="R81" s="75"/>
+      <c r="R81" s="67"/>
     </row>
     <row r="82" spans="1:18" ht="15.6">
-      <c r="A82" s="72"/>
-      <c r="B82" s="44"/>
-      <c r="C82" s="44"/>
+      <c r="A82" s="64"/>
       <c r="D82" s="19">
         <v>1</v>
       </c>
@@ -5722,8 +5228,6 @@
       <c r="F82" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="G82" s="44"/>
-      <c r="H82" s="44"/>
       <c r="I82" s="19">
         <v>1</v>
       </c>
@@ -5736,17 +5240,13 @@
       <c r="L82" s="24" t="s">
         <v>242</v>
       </c>
-      <c r="M82" s="24"/>
-      <c r="N82" s="44"/>
-      <c r="O82" s="44"/>
-      <c r="P82" s="44"/>
-      <c r="Q82" s="44"/>
-      <c r="R82" s="75"/>
+      <c r="M82" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="R82" s="67"/>
     </row>
     <row r="83" spans="1:18" ht="15.6">
-      <c r="A83" s="72"/>
-      <c r="B83" s="44"/>
-      <c r="C83" s="44"/>
+      <c r="A83" s="64"/>
       <c r="D83" s="19">
         <v>2</v>
       </c>
@@ -5756,8 +5256,6 @@
       <c r="F83" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="G83" s="44"/>
-      <c r="H83" s="44"/>
       <c r="I83" s="19">
         <v>2</v>
       </c>
@@ -5770,26 +5268,17 @@
       <c r="L83" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="M83" s="24"/>
-      <c r="N83" s="44"/>
-      <c r="O83" s="44"/>
-      <c r="P83" s="44"/>
-      <c r="Q83" s="44"/>
-      <c r="R83" s="75"/>
+      <c r="M83" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="R83" s="67"/>
     </row>
     <row r="84" spans="1:18" ht="15.6">
-      <c r="A84" s="72"/>
-      <c r="B84" s="44"/>
-      <c r="C84" s="44"/>
-      <c r="D84" s="44"/>
-      <c r="E84" s="44"/>
-      <c r="F84" s="44"/>
-      <c r="G84" s="44"/>
-      <c r="H84" s="44"/>
+      <c r="A84" s="64"/>
       <c r="I84" s="19">
         <v>3</v>
       </c>
-      <c r="J84" s="49" t="s">
+      <c r="J84" s="48" t="s">
         <v>167</v>
       </c>
       <c r="K84" s="17" t="s">
@@ -5798,22 +5287,13 @@
       <c r="L84" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="M84" s="24"/>
-      <c r="N84" s="44"/>
-      <c r="O84" s="44"/>
-      <c r="P84" s="44"/>
-      <c r="Q84" s="44"/>
-      <c r="R84" s="75"/>
+      <c r="M84" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="R84" s="67"/>
     </row>
     <row r="85" spans="1:18" ht="15.6">
-      <c r="A85" s="72"/>
-      <c r="B85" s="44"/>
-      <c r="C85" s="44"/>
-      <c r="D85" s="44"/>
-      <c r="E85" s="44"/>
-      <c r="F85" s="44"/>
-      <c r="G85" s="44"/>
-      <c r="H85" s="44"/>
+      <c r="A85" s="64"/>
       <c r="I85" s="19">
         <v>4</v>
       </c>
@@ -5826,22 +5306,13 @@
       <c r="L85" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="M85" s="24"/>
-      <c r="N85" s="44"/>
-      <c r="O85" s="44"/>
-      <c r="P85" s="44"/>
-      <c r="Q85" s="44"/>
-      <c r="R85" s="75"/>
+      <c r="M85" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="R85" s="67"/>
     </row>
     <row r="86" spans="1:18" ht="15.6">
-      <c r="A86" s="72"/>
-      <c r="B86" s="44"/>
-      <c r="C86" s="44"/>
-      <c r="D86" s="44"/>
-      <c r="E86" s="44"/>
-      <c r="F86" s="44"/>
-      <c r="G86" s="44"/>
-      <c r="H86" s="44"/>
+      <c r="A86" s="64"/>
       <c r="I86" s="19">
         <v>5</v>
       </c>
@@ -5854,22 +5325,13 @@
       <c r="L86" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="M86" s="24"/>
-      <c r="N86" s="44"/>
-      <c r="O86" s="44"/>
-      <c r="P86" s="44"/>
-      <c r="Q86" s="44"/>
-      <c r="R86" s="75"/>
+      <c r="M86" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="R86" s="67"/>
     </row>
     <row r="87" spans="1:18" ht="15.6">
-      <c r="A87" s="72"/>
-      <c r="B87" s="44"/>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
-      <c r="E87" s="44"/>
-      <c r="F87" s="44"/>
-      <c r="G87" s="44"/>
-      <c r="H87" s="44"/>
+      <c r="A87" s="64"/>
       <c r="I87" s="19">
         <v>6</v>
       </c>
@@ -5882,22 +5344,13 @@
       <c r="L87" s="24" t="s">
         <v>246</v>
       </c>
-      <c r="M87" s="24"/>
-      <c r="N87" s="44"/>
-      <c r="O87" s="44"/>
-      <c r="P87" s="44"/>
-      <c r="Q87" s="44"/>
-      <c r="R87" s="75"/>
+      <c r="M87" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="R87" s="67"/>
     </row>
     <row r="88" spans="1:18" ht="15.6">
-      <c r="A88" s="72"/>
-      <c r="B88" s="44"/>
-      <c r="C88" s="44"/>
-      <c r="D88" s="44"/>
-      <c r="E88" s="44"/>
-      <c r="F88" s="44"/>
-      <c r="G88" s="44"/>
-      <c r="H88" s="44"/>
+      <c r="A88" s="64"/>
       <c r="I88" s="19">
         <v>7</v>
       </c>
@@ -5910,72 +5363,54 @@
       <c r="L88" s="24" t="s">
         <v>247</v>
       </c>
-      <c r="M88" s="24"/>
-      <c r="N88" s="44"/>
-      <c r="O88" s="44"/>
-      <c r="P88" s="44"/>
-      <c r="Q88" s="44"/>
-      <c r="R88" s="75"/>
+      <c r="M88" s="17" t="s">
+        <v>287</v>
+      </c>
+      <c r="R88" s="67"/>
     </row>
     <row r="89" spans="1:18">
-      <c r="A89" s="72"/>
-      <c r="B89" s="44"/>
-      <c r="C89" s="44"/>
-      <c r="D89" s="44"/>
-      <c r="E89" s="44"/>
-      <c r="F89" s="44"/>
-      <c r="G89" s="44"/>
-      <c r="H89" s="44"/>
-      <c r="I89" s="44"/>
-      <c r="J89" s="44"/>
-      <c r="K89" s="44"/>
-      <c r="L89" s="68"/>
-      <c r="M89" s="44"/>
-      <c r="N89" s="44"/>
-      <c r="O89" s="44"/>
-      <c r="P89" s="44"/>
-      <c r="Q89" s="44"/>
-      <c r="R89" s="75"/>
+      <c r="A89" s="64"/>
+      <c r="R89" s="67"/>
     </row>
     <row r="90" spans="1:18">
-      <c r="A90" s="74"/>
-      <c r="B90" s="47"/>
-      <c r="C90" s="47"/>
-      <c r="D90" s="47"/>
-      <c r="E90" s="47"/>
-      <c r="F90" s="47"/>
-      <c r="G90" s="47"/>
-      <c r="H90" s="47"/>
-      <c r="I90" s="47"/>
-      <c r="J90" s="47"/>
-      <c r="K90" s="47"/>
-      <c r="L90" s="47"/>
-      <c r="M90" s="47"/>
-      <c r="N90" s="47"/>
-      <c r="O90" s="47"/>
-      <c r="P90" s="47"/>
-      <c r="Q90" s="47"/>
-      <c r="R90" s="79"/>
+      <c r="A90" s="66"/>
+      <c r="B90" s="46"/>
+      <c r="C90" s="46"/>
+      <c r="D90" s="46"/>
+      <c r="E90" s="46"/>
+      <c r="F90" s="46"/>
+      <c r="G90" s="46"/>
+      <c r="H90" s="46"/>
+      <c r="I90" s="46"/>
+      <c r="J90" s="46"/>
+      <c r="K90" s="46"/>
+      <c r="L90" s="46"/>
+      <c r="M90" s="46"/>
+      <c r="N90" s="46"/>
+      <c r="O90" s="46"/>
+      <c r="P90" s="46"/>
+      <c r="Q90" s="46"/>
+      <c r="R90" s="71"/>
     </row>
     <row r="91" spans="1:18" ht="15" thickBot="1">
-      <c r="A91" s="80"/>
-      <c r="B91" s="81"/>
-      <c r="C91" s="81"/>
-      <c r="D91" s="81"/>
-      <c r="E91" s="81"/>
-      <c r="F91" s="81"/>
-      <c r="G91" s="81"/>
-      <c r="H91" s="81"/>
-      <c r="I91" s="81"/>
-      <c r="J91" s="81"/>
-      <c r="K91" s="81"/>
-      <c r="L91" s="81"/>
-      <c r="M91" s="81"/>
-      <c r="N91" s="81"/>
-      <c r="O91" s="81"/>
-      <c r="P91" s="81"/>
-      <c r="Q91" s="81"/>
-      <c r="R91" s="82"/>
+      <c r="A91" s="72"/>
+      <c r="B91" s="73"/>
+      <c r="C91" s="73"/>
+      <c r="D91" s="73"/>
+      <c r="E91" s="73"/>
+      <c r="F91" s="73"/>
+      <c r="G91" s="73"/>
+      <c r="H91" s="73"/>
+      <c r="I91" s="73"/>
+      <c r="J91" s="73"/>
+      <c r="K91" s="73"/>
+      <c r="L91" s="73"/>
+      <c r="M91" s="73"/>
+      <c r="N91" s="73"/>
+      <c r="O91" s="73"/>
+      <c r="P91" s="73"/>
+      <c r="Q91" s="73"/>
+      <c r="R91" s="74"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>